<commit_message>
📊 데이터 업데이트 - 2026-05-20 17:56
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>유사_최고실적</t>
+          <t>유사경기수</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
         <v>42.1</v>
       </c>
       <c r="AA2" t="n">
-        <v>67.2</v>
+        <v>466</v>
       </c>
     </row>
     <row r="3">
@@ -744,7 +744,7 @@
         <v>45.1</v>
       </c>
       <c r="AA3" t="n">
-        <v>69</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4">
@@ -841,7 +841,7 @@
         <v>37.3</v>
       </c>
       <c r="AA4" t="n">
-        <v>66.40000000000001</v>
+        <v>482</v>
       </c>
     </row>
     <row r="5">
@@ -938,7 +938,7 @@
         <v>52.1</v>
       </c>
       <c r="AA5" t="n">
-        <v>85.09999999999999</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6">
@@ -1035,7 +1035,7 @@
         <v>48.6</v>
       </c>
       <c r="AA6" t="n">
-        <v>91.40000000000001</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -1132,7 +1132,7 @@
         <v>44.3</v>
       </c>
       <c r="AA7" t="n">
-        <v>71.7</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8">
@@ -1229,7 +1229,7 @@
         <v>49.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>84.8</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9">
@@ -1326,7 +1326,7 @@
         <v>43.1</v>
       </c>
       <c r="AA9" t="n">
-        <v>69.59999999999999</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10">
@@ -1423,7 +1423,7 @@
         <v>49.1</v>
       </c>
       <c r="AA10" t="n">
-        <v>74.59999999999999</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11">
@@ -1520,7 +1520,7 @@
         <v>38.5</v>
       </c>
       <c r="AA11" t="n">
-        <v>66.40000000000001</v>
+        <v>532</v>
       </c>
     </row>
     <row r="12">
@@ -1617,7 +1617,7 @@
         <v>39.3</v>
       </c>
       <c r="AA12" t="n">
-        <v>66.09999999999999</v>
+        <v>537</v>
       </c>
     </row>
     <row r="13">
@@ -1714,7 +1714,7 @@
         <v>26</v>
       </c>
       <c r="AA13" t="n">
-        <v>71.5</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14">
@@ -1811,7 +1811,7 @@
         <v>35.8</v>
       </c>
       <c r="AA14" t="n">
-        <v>67.7</v>
+        <v>371</v>
       </c>
     </row>
     <row r="15">
@@ -1908,7 +1908,7 @@
         <v>42.6</v>
       </c>
       <c r="AA15" t="n">
-        <v>66.59999999999999</v>
+        <v>446</v>
       </c>
     </row>
     <row r="16">
@@ -2005,7 +2005,7 @@
         <v>48.9</v>
       </c>
       <c r="AA16" t="n">
-        <v>70.2</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17">
@@ -2102,7 +2102,7 @@
         <v>43.8</v>
       </c>
       <c r="AA17" t="n">
-        <v>69.7</v>
+        <v>370</v>
       </c>
     </row>
     <row r="18">
@@ -2199,7 +2199,7 @@
         <v>44.8</v>
       </c>
       <c r="AA18" t="n">
-        <v>72.5</v>
+        <v>324</v>
       </c>
     </row>
     <row r="19">
@@ -2296,7 +2296,7 @@
         <v>43.2</v>
       </c>
       <c r="AA19" t="n">
-        <v>66.40000000000001</v>
+        <v>426</v>
       </c>
     </row>
     <row r="20">
@@ -2393,7 +2393,7 @@
         <v>53</v>
       </c>
       <c r="AA20" t="n">
-        <v>75.8</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21">
@@ -2490,7 +2490,7 @@
         <v>50.8</v>
       </c>
       <c r="AA21" t="n">
-        <v>83.3</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22">
@@ -2587,7 +2587,7 @@
         <v>43.6</v>
       </c>
       <c r="AA22" t="n">
-        <v>74.2</v>
+        <v>264</v>
       </c>
     </row>
     <row r="23">
@@ -2684,7 +2684,7 @@
         <v>51.3</v>
       </c>
       <c r="AA23" t="n">
-        <v>74</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24">
@@ -2781,7 +2781,7 @@
         <v>45.4</v>
       </c>
       <c r="AA24" t="n">
-        <v>69.90000000000001</v>
+        <v>229</v>
       </c>
     </row>
     <row r="25">
@@ -2878,7 +2878,7 @@
         <v>54.8</v>
       </c>
       <c r="AA25" t="n">
-        <v>76.90000000000001</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26">
@@ -2975,7 +2975,7 @@
         <v>46.5</v>
       </c>
       <c r="AA26" t="n">
-        <v>71.40000000000001</v>
+        <v>217</v>
       </c>
     </row>
     <row r="27">
@@ -3072,7 +3072,7 @@
         <v>43.3</v>
       </c>
       <c r="AA27" t="n">
-        <v>68.2</v>
+        <v>402</v>
       </c>
     </row>
     <row r="28">
@@ -3169,7 +3169,7 @@
         <v>44.9</v>
       </c>
       <c r="AA28" t="n">
-        <v>75</v>
+        <v>256</v>
       </c>
     </row>
     <row r="29">
@@ -3266,7 +3266,7 @@
         <v>45.8</v>
       </c>
       <c r="AA29" t="n">
-        <v>67</v>
+        <v>321</v>
       </c>
     </row>
     <row r="30">
@@ -3363,7 +3363,7 @@
         <v>28.7</v>
       </c>
       <c r="AA30" t="n">
-        <v>66.8</v>
+        <v>223</v>
       </c>
     </row>
     <row r="31">
@@ -3460,7 +3460,7 @@
         <v>32.3</v>
       </c>
       <c r="AA31" t="n">
-        <v>62.3</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32">
@@ -3557,7 +3557,7 @@
         <v>34.3</v>
       </c>
       <c r="AA32" t="n">
-        <v>62.8</v>
+        <v>705</v>
       </c>
     </row>
     <row r="33">
@@ -3654,7 +3654,7 @@
         <v>31.8</v>
       </c>
       <c r="AA33" t="n">
-        <v>57.4</v>
+        <v>944</v>
       </c>
     </row>
     <row r="34">
@@ -3751,7 +3751,7 @@
         <v>34.6</v>
       </c>
       <c r="AA34" t="n">
-        <v>61.9</v>
+        <v>749</v>
       </c>
     </row>
     <row r="35">
@@ -3848,7 +3848,7 @@
         <v>31.1</v>
       </c>
       <c r="AA35" t="n">
-        <v>57.6</v>
+        <v>575</v>
       </c>
     </row>
     <row r="36">
@@ -3951,7 +3951,7 @@
         <v>32.9</v>
       </c>
       <c r="AA36" t="n">
-        <v>64.5</v>
+        <v>301</v>
       </c>
     </row>
     <row r="37">
@@ -4048,7 +4048,7 @@
         <v>35.3</v>
       </c>
       <c r="AA37" t="n">
-        <v>61.8</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38">
@@ -4145,7 +4145,7 @@
         <v>28.8</v>
       </c>
       <c r="AA38" t="n">
-        <v>56.1</v>
+        <v>715</v>
       </c>
     </row>
     <row r="39">
@@ -4242,7 +4242,7 @@
         <v>35.7</v>
       </c>
       <c r="AA39" t="n">
-        <v>63</v>
+        <v>745</v>
       </c>
     </row>
     <row r="40">
@@ -4339,7 +4339,7 @@
         <v>32.2</v>
       </c>
       <c r="AA40" t="n">
-        <v>57.2</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="41">
@@ -4436,7 +4436,7 @@
         <v>37</v>
       </c>
       <c r="AA41" t="n">
-        <v>63</v>
+        <v>729</v>
       </c>
     </row>
     <row r="42">
@@ -4533,7 +4533,7 @@
         <v>44.8</v>
       </c>
       <c r="AA42" t="n">
-        <v>58.6</v>
+        <v>29</v>
       </c>
     </row>
     <row r="43">
@@ -4630,7 +4630,7 @@
         <v>40.3</v>
       </c>
       <c r="AA43" t="n">
-        <v>55</v>
+        <v>320</v>
       </c>
     </row>
     <row r="44">
@@ -4727,7 +4727,7 @@
         <v>30.7</v>
       </c>
       <c r="AA44" t="n">
-        <v>55.9</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="45">
@@ -4824,7 +4824,7 @@
         <v>34.9</v>
       </c>
       <c r="AA45" t="n">
-        <v>58.6</v>
+        <v>816</v>
       </c>
     </row>
     <row r="46">
@@ -4927,7 +4927,7 @@
         <v>45.6</v>
       </c>
       <c r="AA46" t="n">
-        <v>61.1</v>
+        <v>316</v>
       </c>
     </row>
     <row r="47">
@@ -5030,7 +5030,7 @@
         <v>38.5</v>
       </c>
       <c r="AA47" t="n">
-        <v>62.1</v>
+        <v>169</v>
       </c>
     </row>
     <row r="48">
@@ -5127,7 +5127,7 @@
         <v>35.8</v>
       </c>
       <c r="AA48" t="n">
-        <v>60.9</v>
+        <v>729</v>
       </c>
     </row>
     <row r="49">
@@ -5224,7 +5224,7 @@
         <v>39.5</v>
       </c>
       <c r="AA49" t="n">
-        <v>56.2</v>
+        <v>365</v>
       </c>
     </row>
     <row r="50">
@@ -5321,7 +5321,7 @@
         <v>34.7</v>
       </c>
       <c r="AA50" t="n">
-        <v>61.7</v>
+        <v>757</v>
       </c>
     </row>
     <row r="51">
@@ -5418,7 +5418,7 @@
         <v>35.4</v>
       </c>
       <c r="AA51" t="n">
-        <v>61.4</v>
+        <v>823</v>
       </c>
     </row>
     <row r="52">
@@ -5515,7 +5515,7 @@
         <v>36.7</v>
       </c>
       <c r="AA52" t="n">
-        <v>61.6</v>
+        <v>703</v>
       </c>
     </row>
     <row r="53">
@@ -5612,7 +5612,7 @@
         <v>33.7</v>
       </c>
       <c r="AA53" t="n">
-        <v>61.6</v>
+        <v>713</v>
       </c>
     </row>
     <row r="54">
@@ -5709,7 +5709,7 @@
         <v>33.9</v>
       </c>
       <c r="AA54" t="n">
-        <v>60.3</v>
+        <v>879</v>
       </c>
     </row>
     <row r="55">
@@ -5812,7 +5812,7 @@
         <v>36</v>
       </c>
       <c r="AA55" t="n">
-        <v>57.4</v>
+        <v>835</v>
       </c>
     </row>
     <row r="56">
@@ -5915,7 +5915,7 @@
         <v>34.1</v>
       </c>
       <c r="AA56" t="n">
-        <v>57.1</v>
+        <v>592</v>
       </c>
     </row>
     <row r="57">
@@ -6012,7 +6012,7 @@
         <v>31.6</v>
       </c>
       <c r="AA57" t="n">
-        <v>57.7</v>
+        <v>589</v>
       </c>
     </row>
     <row r="58">
@@ -6109,7 +6109,7 @@
         <v>35</v>
       </c>
       <c r="AA58" t="n">
-        <v>61</v>
+        <v>792</v>
       </c>
     </row>
     <row r="59">
@@ -6206,7 +6206,7 @@
         <v>31.5</v>
       </c>
       <c r="AA59" t="n">
-        <v>59.8</v>
+        <v>480</v>
       </c>
     </row>
     <row r="60">
@@ -6303,7 +6303,7 @@
         <v>33.4</v>
       </c>
       <c r="AA60" t="n">
-        <v>56.7</v>
+        <v>649</v>
       </c>
     </row>
     <row r="61">
@@ -6406,7 +6406,7 @@
         <v>37.6</v>
       </c>
       <c r="AA61" t="n">
-        <v>58.5</v>
+        <v>407</v>
       </c>
     </row>
     <row r="62">
@@ -6509,7 +6509,7 @@
         <v>33.5</v>
       </c>
       <c r="AA62" t="n">
-        <v>63.6</v>
+        <v>209</v>
       </c>
     </row>
     <row r="63">
@@ -6606,7 +6606,7 @@
         <v>30.6</v>
       </c>
       <c r="AA63" t="n">
-        <v>55.8</v>
+        <v>627</v>
       </c>
     </row>
     <row r="64">
@@ -6703,7 +6703,7 @@
         <v>28.8</v>
       </c>
       <c r="AA64" t="n">
-        <v>56.1</v>
+        <v>715</v>
       </c>
     </row>
     <row r="65">
@@ -6806,7 +6806,7 @@
         <v>39.6</v>
       </c>
       <c r="AA65" t="n">
-        <v>59.7</v>
+        <v>596</v>
       </c>
     </row>
     <row r="66">
@@ -6909,7 +6909,7 @@
         <v>37.4</v>
       </c>
       <c r="AA66" t="n">
-        <v>61.5</v>
+        <v>353</v>
       </c>
     </row>
     <row r="67">
@@ -7012,7 +7012,7 @@
         <v>36.1</v>
       </c>
       <c r="AA67" t="n">
-        <v>60.9</v>
+        <v>571</v>
       </c>
     </row>
     <row r="68">
@@ -7109,7 +7109,7 @@
         <v>30.4</v>
       </c>
       <c r="AA68" t="n">
-        <v>59.8</v>
+        <v>381</v>
       </c>
     </row>
     <row r="69">
@@ -7212,7 +7212,7 @@
         <v>35.2</v>
       </c>
       <c r="AA69" t="n">
-        <v>58.1</v>
+        <v>744</v>
       </c>
     </row>
     <row r="70">
@@ -7315,7 +7315,7 @@
         <v>38.1</v>
       </c>
       <c r="AA70" t="n">
-        <v>57</v>
+        <v>653</v>
       </c>
     </row>
     <row r="71">
@@ -7418,7 +7418,7 @@
         <v>49.1</v>
       </c>
       <c r="AA71" t="n">
-        <v>63.5</v>
+        <v>293</v>
       </c>
     </row>
     <row r="72">
@@ -7521,7 +7521,7 @@
         <v>40.3</v>
       </c>
       <c r="AA72" t="n">
-        <v>61.9</v>
+        <v>360</v>
       </c>
     </row>
     <row r="73">
@@ -7624,7 +7624,7 @@
         <v>41.7</v>
       </c>
       <c r="AA73" t="n">
-        <v>59.6</v>
+        <v>302</v>
       </c>
     </row>
     <row r="74">
@@ -7721,7 +7721,7 @@
         <v>34.3</v>
       </c>
       <c r="AA74" t="n">
-        <v>60.4</v>
+        <v>566</v>
       </c>
     </row>
     <row r="75">
@@ -7818,7 +7818,7 @@
         <v>34.8</v>
       </c>
       <c r="AA75" t="n">
-        <v>63.1</v>
+        <v>597</v>
       </c>
     </row>
     <row r="76">
@@ -7921,7 +7921,7 @@
         <v>35.1</v>
       </c>
       <c r="AA76" t="n">
-        <v>56.6</v>
+        <v>756</v>
       </c>
     </row>
     <row r="77">
@@ -8018,7 +8018,7 @@
         <v>35.9</v>
       </c>
       <c r="AA77" t="n">
-        <v>61.1</v>
+        <v>785</v>
       </c>
     </row>
     <row r="78">
@@ -8115,7 +8115,7 @@
         <v>31.8</v>
       </c>
       <c r="AA78" t="n">
-        <v>56.8</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="79">
@@ -8212,7 +8212,7 @@
         <v>35.1</v>
       </c>
       <c r="AA79" t="n">
-        <v>59.7</v>
+        <v>812</v>
       </c>
     </row>
     <row r="80">
@@ -8309,7 +8309,7 @@
         <v>36.4</v>
       </c>
       <c r="AA80" t="n">
-        <v>60.8</v>
+        <v>701</v>
       </c>
     </row>
     <row r="81">
@@ -8406,7 +8406,7 @@
         <v>36.2</v>
       </c>
       <c r="AA81" t="n">
-        <v>58.7</v>
+        <v>520</v>
       </c>
     </row>
     <row r="82">
@@ -8503,7 +8503,7 @@
         <v>37.1</v>
       </c>
       <c r="AA82" t="n">
-        <v>62.9</v>
+        <v>693</v>
       </c>
     </row>
     <row r="83">
@@ -8606,7 +8606,7 @@
         <v>39.6</v>
       </c>
       <c r="AA83" t="n">
-        <v>57.6</v>
+        <v>571</v>
       </c>
     </row>
     <row r="84">
@@ -8703,7 +8703,7 @@
         <v>32.9</v>
       </c>
       <c r="AA84" t="n">
-        <v>55.2</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="85">
@@ -8800,7 +8800,7 @@
         <v>29.9</v>
       </c>
       <c r="AA85" t="n">
-        <v>55.4</v>
+        <v>612</v>
       </c>
     </row>
     <row r="86">
@@ -8897,7 +8897,7 @@
         <v>38.5</v>
       </c>
       <c r="AA86" t="n">
-        <v>62.3</v>
+        <v>478</v>
       </c>
     </row>
     <row r="87">
@@ -8994,7 +8994,7 @@
         <v>32.4</v>
       </c>
       <c r="AA87" t="n">
-        <v>55.5</v>
+        <v>679</v>
       </c>
     </row>
     <row r="88">
@@ -9091,7 +9091,7 @@
         <v>38.1</v>
       </c>
       <c r="AA88" t="n">
-        <v>59.2</v>
+        <v>478</v>
       </c>
     </row>
     <row r="89">
@@ -9194,7 +9194,7 @@
         <v>36</v>
       </c>
       <c r="AA89" t="n">
-        <v>59.4</v>
+        <v>561</v>
       </c>
     </row>
     <row r="90">
@@ -9291,7 +9291,7 @@
         <v>43.2</v>
       </c>
       <c r="AA90" t="n">
-        <v>64.59999999999999</v>
+        <v>370</v>
       </c>
     </row>
     <row r="91">
@@ -9388,7 +9388,7 @@
         <v>35.1</v>
       </c>
       <c r="AA91" t="n">
-        <v>59.7</v>
+        <v>812</v>
       </c>
     </row>
     <row r="92">
@@ -9485,7 +9485,7 @@
         <v>35</v>
       </c>
       <c r="AA92" t="n">
-        <v>57.6</v>
+        <v>838</v>
       </c>
     </row>
     <row r="93">
@@ -9582,7 +9582,7 @@
         <v>29</v>
       </c>
       <c r="AA93" t="n">
-        <v>56.8</v>
+        <v>651</v>
       </c>
     </row>
     <row r="94">
@@ -9679,7 +9679,7 @@
         <v>38.8</v>
       </c>
       <c r="AA94" t="n">
-        <v>61.2</v>
+        <v>446</v>
       </c>
     </row>
     <row r="95">
@@ -9776,7 +9776,7 @@
         <v>32.2</v>
       </c>
       <c r="AA95" t="n">
-        <v>57.2</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="96">
@@ -9873,7 +9873,7 @@
         <v>38.8</v>
       </c>
       <c r="AA96" t="n">
-        <v>64.09999999999999</v>
+        <v>641</v>
       </c>
     </row>
     <row r="97">
@@ -9970,7 +9970,7 @@
         <v>34.7</v>
       </c>
       <c r="AA97" t="n">
-        <v>59.8</v>
+        <v>779</v>
       </c>
     </row>
     <row r="98">
@@ -10067,7 +10067,7 @@
         <v>30.9</v>
       </c>
       <c r="AA98" t="n">
-        <v>58.8</v>
+        <v>537</v>
       </c>
     </row>
     <row r="99">
@@ -10164,7 +10164,7 @@
         <v>34.3</v>
       </c>
       <c r="AA99" t="n">
-        <v>60.7</v>
+        <v>760</v>
       </c>
     </row>
     <row r="100">
@@ -10261,7 +10261,7 @@
         <v>33.3</v>
       </c>
       <c r="AA100" t="n">
-        <v>60.6</v>
+        <v>795</v>
       </c>
     </row>
     <row r="101">
@@ -10358,7 +10358,7 @@
         <v>36.8</v>
       </c>
       <c r="AA101" t="n">
-        <v>62.8</v>
+        <v>725</v>
       </c>
     </row>
     <row r="102">
@@ -10455,7 +10455,7 @@
         <v>42.7</v>
       </c>
       <c r="AA102" t="n">
-        <v>60.8</v>
+        <v>344</v>
       </c>
     </row>
     <row r="103">
@@ -10552,7 +10552,7 @@
         <v>33.4</v>
       </c>
       <c r="AA103" t="n">
-        <v>62.1</v>
+        <v>335</v>
       </c>
     </row>
     <row r="104">
@@ -10649,7 +10649,7 @@
         <v>35.9</v>
       </c>
       <c r="AA104" t="n">
-        <v>62.5</v>
+        <v>797</v>
       </c>
     </row>
     <row r="105">
@@ -10746,7 +10746,7 @@
         <v>30.1</v>
       </c>
       <c r="AA105" t="n">
-        <v>45</v>
+        <v>993</v>
       </c>
     </row>
     <row r="106">
@@ -10843,7 +10843,7 @@
         <v>34.6</v>
       </c>
       <c r="AA106" t="n">
-        <v>47.8</v>
+        <v>598</v>
       </c>
     </row>
     <row r="107">
@@ -10940,7 +10940,7 @@
         <v>26.3</v>
       </c>
       <c r="AA107" t="n">
-        <v>49.2</v>
+        <v>834</v>
       </c>
     </row>
     <row r="108">
@@ -11043,7 +11043,7 @@
         <v>31</v>
       </c>
       <c r="AA108" t="n">
-        <v>49.7</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="109">
@@ -11146,7 +11146,7 @@
         <v>32</v>
       </c>
       <c r="AA109" t="n">
-        <v>50.6</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="110">
@@ -11243,7 +11243,7 @@
         <v>31.9</v>
       </c>
       <c r="AA110" t="n">
-        <v>53.3</v>
+        <v>749</v>
       </c>
     </row>
     <row r="111">
@@ -11346,7 +11346,7 @@
         <v>33.6</v>
       </c>
       <c r="AA111" t="n">
-        <v>54.1</v>
+        <v>891</v>
       </c>
     </row>
     <row r="112">
@@ -11449,7 +11449,7 @@
         <v>33</v>
       </c>
       <c r="AA112" t="n">
-        <v>48.1</v>
+        <v>790</v>
       </c>
     </row>
     <row r="113">
@@ -11546,7 +11546,7 @@
         <v>27.6</v>
       </c>
       <c r="AA113" t="n">
-        <v>45.5</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="114">
@@ -11643,7 +11643,7 @@
         <v>31.8</v>
       </c>
       <c r="AA114" t="n">
-        <v>48.6</v>
+        <v>796</v>
       </c>
     </row>
     <row r="115">
@@ -11740,7 +11740,7 @@
         <v>27.1</v>
       </c>
       <c r="AA115" t="n">
-        <v>48.4</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="116">
@@ -11843,7 +11843,7 @@
         <v>35.2</v>
       </c>
       <c r="AA116" t="n">
-        <v>51.6</v>
+        <v>608</v>
       </c>
     </row>
     <row r="117">
@@ -11940,7 +11940,7 @@
         <v>27.5</v>
       </c>
       <c r="AA117" t="n">
-        <v>48.2</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="118">
@@ -12037,7 +12037,7 @@
         <v>29.7</v>
       </c>
       <c r="AA118" t="n">
-        <v>49.5</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="119">
@@ -12134,7 +12134,7 @@
         <v>32.6</v>
       </c>
       <c r="AA119" t="n">
-        <v>54.7</v>
+        <v>678</v>
       </c>
     </row>
     <row r="120">
@@ -12237,7 +12237,7 @@
         <v>36.3</v>
       </c>
       <c r="AA120" t="n">
-        <v>51.9</v>
+        <v>576</v>
       </c>
     </row>
     <row r="121">
@@ -12340,7 +12340,7 @@
         <v>27</v>
       </c>
       <c r="AA121" t="n">
-        <v>45.3</v>
+        <v>684</v>
       </c>
     </row>
     <row r="122">
@@ -12437,7 +12437,7 @@
         <v>26.7</v>
       </c>
       <c r="AA122" t="n">
-        <v>47.7</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="123">
@@ -12540,7 +12540,7 @@
         <v>35.1</v>
       </c>
       <c r="AA123" t="n">
-        <v>47.3</v>
+        <v>885</v>
       </c>
     </row>
     <row r="124">
@@ -12643,7 +12643,7 @@
         <v>34.7</v>
       </c>
       <c r="AA124" t="n">
-        <v>46.5</v>
+        <v>144</v>
       </c>
     </row>
     <row r="125">
@@ -12740,7 +12740,7 @@
         <v>28.9</v>
       </c>
       <c r="AA125" t="n">
-        <v>54.1</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="126">
@@ -12837,7 +12837,7 @@
         <v>28.3</v>
       </c>
       <c r="AA126" t="n">
-        <v>50</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="127">
@@ -12934,7 +12934,7 @@
         <v>27.6</v>
       </c>
       <c r="AA127" t="n">
-        <v>47.4</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="128">
@@ -13031,7 +13031,7 @@
         <v>30.4</v>
       </c>
       <c r="AA128" t="n">
-        <v>46.4</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="129">
@@ -13134,7 +13134,7 @@
         <v>33.7</v>
       </c>
       <c r="AA129" t="n">
-        <v>51.4</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="130">
@@ -13237,7 +13237,7 @@
         <v>37.9</v>
       </c>
       <c r="AA130" t="n">
-        <v>46.7</v>
+        <v>478</v>
       </c>
     </row>
     <row r="131">
@@ -13334,7 +13334,7 @@
         <v>26.4</v>
       </c>
       <c r="AA131" t="n">
-        <v>49.5</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="132">
@@ -13437,7 +13437,7 @@
         <v>34</v>
       </c>
       <c r="AA132" t="n">
-        <v>49.8</v>
+        <v>952</v>
       </c>
     </row>
     <row r="133">
@@ -13540,7 +13540,7 @@
         <v>36.8</v>
       </c>
       <c r="AA133" t="n">
-        <v>53.6</v>
+        <v>429</v>
       </c>
     </row>
     <row r="134">
@@ -13637,7 +13637,7 @@
         <v>27.6</v>
       </c>
       <c r="AA134" t="n">
-        <v>45.5</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="135">
@@ -13734,7 +13734,7 @@
         <v>34.4</v>
       </c>
       <c r="AA135" t="n">
-        <v>48.5</v>
+        <v>588</v>
       </c>
     </row>
     <row r="136">
@@ -13831,7 +13831,7 @@
         <v>30.6</v>
       </c>
       <c r="AA136" t="n">
-        <v>48.2</v>
+        <v>978</v>
       </c>
     </row>
     <row r="137">
@@ -13928,7 +13928,7 @@
         <v>28.8</v>
       </c>
       <c r="AA137" t="n">
-        <v>50.3</v>
+        <v>888</v>
       </c>
     </row>
     <row r="138">
@@ -14025,7 +14025,7 @@
         <v>27.2</v>
       </c>
       <c r="AA138" t="n">
-        <v>47</v>
+        <v>983</v>
       </c>
     </row>
     <row r="139">
@@ -14128,7 +14128,7 @@
         <v>34.2</v>
       </c>
       <c r="AA139" t="n">
-        <v>49.3</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="140">
@@ -14231,7 +14231,7 @@
         <v>32</v>
       </c>
       <c r="AA140" t="n">
-        <v>47.9</v>
+        <v>653</v>
       </c>
     </row>
     <row r="141">
@@ -14334,7 +14334,7 @@
         <v>32.6</v>
       </c>
       <c r="AA141" t="n">
-        <v>46.3</v>
+        <v>884</v>
       </c>
     </row>
     <row r="142">
@@ -14437,7 +14437,7 @@
         <v>33.1</v>
       </c>
       <c r="AA142" t="n">
-        <v>45.6</v>
+        <v>848</v>
       </c>
     </row>
     <row r="143">
@@ -14540,7 +14540,7 @@
         <v>31.4</v>
       </c>
       <c r="AA143" t="n">
-        <v>45.2</v>
+        <v>912</v>
       </c>
     </row>
     <row r="144">
@@ -14637,7 +14637,7 @@
         <v>30.4</v>
       </c>
       <c r="AA144" t="n">
-        <v>46.4</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="145">
@@ -14734,7 +14734,7 @@
         <v>30.3</v>
       </c>
       <c r="AA145" t="n">
-        <v>45.3</v>
+        <v>928</v>
       </c>
     </row>
     <row r="146">
@@ -14837,7 +14837,7 @@
         <v>36.1</v>
       </c>
       <c r="AA146" t="n">
-        <v>54.3</v>
+        <v>521</v>
       </c>
     </row>
     <row r="147">
@@ -14934,7 +14934,7 @@
         <v>27</v>
       </c>
       <c r="AA147" t="n">
-        <v>51.7</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="148">
@@ -15037,7 +15037,7 @@
         <v>35.9</v>
       </c>
       <c r="AA148" t="n">
-        <v>53.9</v>
+        <v>518</v>
       </c>
     </row>
     <row r="149">
@@ -15134,7 +15134,7 @@
         <v>26.2</v>
       </c>
       <c r="AA149" t="n">
-        <v>50.5</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="150">
@@ -15231,7 +15231,7 @@
         <v>29</v>
       </c>
       <c r="AA150" t="n">
-        <v>54</v>
+        <v>957</v>
       </c>
     </row>
     <row r="151">
@@ -15328,7 +15328,7 @@
         <v>26.2</v>
       </c>
       <c r="AA151" t="n">
-        <v>47.9</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="152">
@@ -15425,7 +15425,7 @@
         <v>26.9</v>
       </c>
       <c r="AA152" t="n">
-        <v>45.9</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="153">
@@ -15522,7 +15522,7 @@
         <v>26.2</v>
       </c>
       <c r="AA153" t="n">
-        <v>51.7</v>
+        <v>868</v>
       </c>
     </row>
     <row r="154">
@@ -15619,7 +15619,7 @@
         <v>30.7</v>
       </c>
       <c r="AA154" t="n">
-        <v>51.6</v>
+        <v>797</v>
       </c>
     </row>
     <row r="155">
@@ -15716,7 +15716,7 @@
         <v>27.1</v>
       </c>
       <c r="AA155" t="n">
-        <v>48.4</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="156">
@@ -15813,7 +15813,7 @@
         <v>26</v>
       </c>
       <c r="AA156" t="n">
-        <v>45</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="157">
@@ -15910,7 +15910,7 @@
         <v>31.1</v>
       </c>
       <c r="AA157" t="n">
-        <v>49.5</v>
+        <v>849</v>
       </c>
     </row>
     <row r="158">
@@ -16007,7 +16007,7 @@
         <v>27.6</v>
       </c>
       <c r="AA158" t="n">
-        <v>46.4</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="159">
@@ -16104,7 +16104,7 @@
         <v>31.8</v>
       </c>
       <c r="AA159" t="n">
-        <v>53.3</v>
+        <v>782</v>
       </c>
     </row>
     <row r="160">
@@ -16201,7 +16201,7 @@
         <v>25.2</v>
       </c>
       <c r="AA160" t="n">
-        <v>50.9</v>
+        <v>923</v>
       </c>
     </row>
     <row r="161">
@@ -16304,7 +16304,7 @@
         <v>34.3</v>
       </c>
       <c r="AA161" t="n">
-        <v>48.8</v>
+        <v>674</v>
       </c>
     </row>
     <row r="162">
@@ -16401,7 +16401,7 @@
         <v>36.4</v>
       </c>
       <c r="AA162" t="n">
-        <v>49.8</v>
+        <v>500</v>
       </c>
     </row>
     <row r="163">
@@ -16504,7 +16504,7 @@
         <v>34.2</v>
       </c>
       <c r="AA163" t="n">
-        <v>45.8</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="164">
@@ -16607,7 +16607,7 @@
         <v>31</v>
       </c>
       <c r="AA164" t="n">
-        <v>47.8</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="165">
@@ -16704,7 +16704,7 @@
         <v>29.6</v>
       </c>
       <c r="AA165" t="n">
-        <v>46.1</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="166">
@@ -16801,7 +16801,7 @@
         <v>26.7</v>
       </c>
       <c r="AA166" t="n">
-        <v>45.3</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="167">
@@ -16898,7 +16898,7 @@
         <v>25.9</v>
       </c>
       <c r="AA167" t="n">
-        <v>50.7</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="168">
@@ -16995,7 +16995,7 @@
         <v>29</v>
       </c>
       <c r="AA168" t="n">
-        <v>53.8</v>
+        <v>606</v>
       </c>
     </row>
     <row r="169">
@@ -17092,7 +17092,7 @@
         <v>27.6</v>
       </c>
       <c r="AA169" t="n">
-        <v>49.6</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="170">
@@ -17195,7 +17195,7 @@
         <v>32.6</v>
       </c>
       <c r="AA170" t="n">
-        <v>54.1</v>
+        <v>916</v>
       </c>
     </row>
     <row r="171">
@@ -17292,7 +17292,7 @@
         <v>30.1</v>
       </c>
       <c r="AA171" t="n">
-        <v>50.4</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="172">
@@ -17389,7 +17389,7 @@
         <v>30.2</v>
       </c>
       <c r="AA172" t="n">
-        <v>48.6</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="173">
@@ -17486,7 +17486,7 @@
         <v>33.1</v>
       </c>
       <c r="AA173" t="n">
-        <v>51.8</v>
+        <v>785</v>
       </c>
     </row>
     <row r="174">
@@ -17583,7 +17583,7 @@
         <v>26.3</v>
       </c>
       <c r="AA174" t="n">
-        <v>48.4</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="175">
@@ -17680,7 +17680,7 @@
         <v>27.1</v>
       </c>
       <c r="AA175" t="n">
-        <v>51.4</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="176">
@@ -17777,7 +17777,7 @@
         <v>32.7</v>
       </c>
       <c r="AA176" t="n">
-        <v>51.4</v>
+        <v>698</v>
       </c>
     </row>
     <row r="177">
@@ -17874,7 +17874,7 @@
         <v>33.7</v>
       </c>
       <c r="AA177" t="n">
-        <v>53.7</v>
+        <v>867</v>
       </c>
     </row>
     <row r="178">
@@ -17971,7 +17971,7 @@
         <v>29.1</v>
       </c>
       <c r="AA178" t="n">
-        <v>51.2</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="179">
@@ -18068,7 +18068,7 @@
         <v>30.8</v>
       </c>
       <c r="AA179" t="n">
-        <v>49.6</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="180">
@@ -18165,7 +18165,7 @@
         <v>25.9</v>
       </c>
       <c r="AA180" t="n">
-        <v>50.7</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="181">
@@ -18262,7 +18262,7 @@
         <v>27.7</v>
       </c>
       <c r="AA181" t="n">
-        <v>51.6</v>
+        <v>675</v>
       </c>
     </row>
     <row r="182">
@@ -18359,7 +18359,7 @@
         <v>30.9</v>
       </c>
       <c r="AA182" t="n">
-        <v>53</v>
+        <v>825</v>
       </c>
     </row>
     <row r="183">
@@ -18456,7 +18456,7 @@
         <v>26.2</v>
       </c>
       <c r="AA183" t="n">
-        <v>50.4</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="184">
@@ -18553,7 +18553,7 @@
         <v>28.1</v>
       </c>
       <c r="AA184" t="n">
-        <v>48.6</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="185">
@@ -18650,7 +18650,7 @@
         <v>32.4</v>
       </c>
       <c r="AA185" t="n">
-        <v>54.8</v>
+        <v>695</v>
       </c>
     </row>
     <row r="186">
@@ -18747,7 +18747,7 @@
         <v>31.2</v>
       </c>
       <c r="AA186" t="n">
-        <v>50.9</v>
+        <v>792</v>
       </c>
     </row>
     <row r="187">
@@ -18844,7 +18844,7 @@
         <v>26.7</v>
       </c>
       <c r="AA187" t="n">
-        <v>52.2</v>
+        <v>439</v>
       </c>
     </row>
     <row r="188">
@@ -18941,7 +18941,7 @@
         <v>31.4</v>
       </c>
       <c r="AA188" t="n">
-        <v>53.9</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="189">
@@ -19038,7 +19038,7 @@
         <v>27.5</v>
       </c>
       <c r="AA189" t="n">
-        <v>47.1</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="190">
@@ -19135,7 +19135,7 @@
         <v>30.6</v>
       </c>
       <c r="AA190" t="n">
-        <v>51.1</v>
+        <v>929</v>
       </c>
     </row>
     <row r="191">
@@ -19232,7 +19232,7 @@
         <v>26.4</v>
       </c>
       <c r="AA191" t="n">
-        <v>42.6</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="192">
@@ -19329,7 +19329,7 @@
         <v>27.3</v>
       </c>
       <c r="AA192" t="n">
-        <v>41.1</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="193">
@@ -19426,7 +19426,7 @@
         <v>23</v>
       </c>
       <c r="AA193" t="n">
-        <v>47.3</v>
+        <v>725</v>
       </c>
     </row>
     <row r="194">
@@ -19523,7 +19523,7 @@
         <v>25.3</v>
       </c>
       <c r="AA194" t="n">
-        <v>43.2</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="195">
@@ -19620,7 +19620,7 @@
         <v>22.6</v>
       </c>
       <c r="AA195" t="n">
-        <v>38.2</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="196">
@@ -19723,7 +19723,7 @@
         <v>34.3</v>
       </c>
       <c r="AA196" t="n">
-        <v>41.4</v>
+        <v>840</v>
       </c>
     </row>
     <row r="197">
@@ -19820,7 +19820,7 @@
         <v>23.2</v>
       </c>
       <c r="AA197" t="n">
-        <v>42.4</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="198">
@@ -19917,7 +19917,7 @@
         <v>25.9</v>
       </c>
       <c r="AA198" t="n">
-        <v>44.4</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="199">
@@ -20014,7 +20014,7 @@
         <v>19.7</v>
       </c>
       <c r="AA199" t="n">
-        <v>39.1</v>
+        <v>238</v>
       </c>
     </row>
     <row r="200">
@@ -20117,7 +20117,7 @@
         <v>27.6</v>
       </c>
       <c r="AA200" t="n">
-        <v>46.7</v>
+        <v>891</v>
       </c>
     </row>
     <row r="201">
@@ -20214,7 +20214,7 @@
         <v>30</v>
       </c>
       <c r="AA201" t="n">
-        <v>42.2</v>
+        <v>180</v>
       </c>
     </row>
     <row r="202">
@@ -20311,7 +20311,7 @@
         <v>18.4</v>
       </c>
       <c r="AA202" t="n">
-        <v>39.3</v>
+        <v>425</v>
       </c>
     </row>
     <row r="203">
@@ -20414,7 +20414,7 @@
         <v>14.3</v>
       </c>
       <c r="AA203" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
     </row>
     <row r="204">
@@ -20517,7 +20517,7 @@
         <v>36</v>
       </c>
       <c r="AA204" t="n">
-        <v>41.5</v>
+        <v>530</v>
       </c>
     </row>
     <row r="205">
@@ -20614,7 +20614,7 @@
         <v>26.6</v>
       </c>
       <c r="AA205" t="n">
-        <v>41</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="206">
@@ -20717,7 +20717,7 @@
         <v>22.8</v>
       </c>
       <c r="AA206" t="n">
-        <v>40.3</v>
+        <v>632</v>
       </c>
     </row>
     <row r="207">
@@ -20814,7 +20814,7 @@
         <v>25.6</v>
       </c>
       <c r="AA207" t="n">
-        <v>43.9</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="208">
@@ -20911,7 +20911,7 @@
         <v>22.8</v>
       </c>
       <c r="AA208" t="n">
-        <v>41.3</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="209">
@@ -21008,7 +21008,7 @@
         <v>27</v>
       </c>
       <c r="AA209" t="n">
-        <v>41.5</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="210">
@@ -21105,7 +21105,7 @@
         <v>23.2</v>
       </c>
       <c r="AA210" t="n">
-        <v>42.4</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="211">
@@ -21202,7 +21202,7 @@
         <v>28</v>
       </c>
       <c r="AA211" t="n">
-        <v>43.1</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="212">
@@ -21305,7 +21305,7 @@
         <v>33.5</v>
       </c>
       <c r="AA212" t="n">
-        <v>43.4</v>
+        <v>999</v>
       </c>
     </row>
     <row r="213">
@@ -21402,7 +21402,7 @@
         <v>25.6</v>
       </c>
       <c r="AA213" t="n">
-        <v>44.4</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="214">
@@ -21505,7 +21505,7 @@
         <v>24.1</v>
       </c>
       <c r="AA214" t="n">
-        <v>40.3</v>
+        <v>759</v>
       </c>
     </row>
     <row r="215">
@@ -21608,7 +21608,7 @@
         <v>29</v>
       </c>
       <c r="AA215" t="n">
-        <v>46.6</v>
+        <v>994</v>
       </c>
     </row>
     <row r="216">
@@ -21705,7 +21705,7 @@
         <v>30.9</v>
       </c>
       <c r="AA216" t="n">
-        <v>41.6</v>
+        <v>459</v>
       </c>
     </row>
     <row r="217">
@@ -21808,7 +21808,7 @@
         <v>32.9</v>
       </c>
       <c r="AA217" t="n">
-        <v>43.5</v>
+        <v>827</v>
       </c>
     </row>
     <row r="218">
@@ -21905,7 +21905,7 @@
         <v>24.5</v>
       </c>
       <c r="AA218" t="n">
-        <v>38.2</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="219">
@@ -22002,7 +22002,7 @@
         <v>26.9</v>
       </c>
       <c r="AA219" t="n">
-        <v>44.6</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="220">
@@ -22099,7 +22099,7 @@
         <v>33.2</v>
       </c>
       <c r="AA220" t="n">
-        <v>50.7</v>
+        <v>211</v>
       </c>
     </row>
     <row r="221">
@@ -22196,7 +22196,7 @@
         <v>25.1</v>
       </c>
       <c r="AA221" t="n">
-        <v>43.3</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="222">
@@ -22293,7 +22293,7 @@
         <v>4.8</v>
       </c>
       <c r="AA222" t="n">
-        <v>47.6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="223">
@@ -22390,7 +22390,7 @@
         <v>23.5</v>
       </c>
       <c r="AA223" t="n">
-        <v>44.2</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="224">
@@ -22487,7 +22487,7 @@
         <v>27.3</v>
       </c>
       <c r="AA224" t="n">
-        <v>40.3</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="225">
@@ -22590,7 +22590,7 @@
         <v>31.3</v>
       </c>
       <c r="AA225" t="n">
-        <v>40.9</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="226">
@@ -22693,7 +22693,7 @@
         <v>27.4</v>
       </c>
       <c r="AA226" t="n">
-        <v>41</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="227">
@@ -22790,7 +22790,7 @@
         <v>24</v>
       </c>
       <c r="AA227" t="n">
-        <v>43.3</v>
+        <v>876</v>
       </c>
     </row>
     <row r="228">
@@ -22887,7 +22887,7 @@
         <v>22.8</v>
       </c>
       <c r="AA228" t="n">
-        <v>39.1</v>
+        <v>977</v>
       </c>
     </row>
     <row r="229">
@@ -22990,7 +22990,7 @@
         <v>24.6</v>
       </c>
       <c r="AA229" t="n">
-        <v>42</v>
+        <v>431</v>
       </c>
     </row>
     <row r="230">
@@ -23093,7 +23093,7 @@
         <v>25.1</v>
       </c>
       <c r="AA230" t="n">
-        <v>43.6</v>
+        <v>722</v>
       </c>
     </row>
     <row r="231">
@@ -23196,7 +23196,7 @@
         <v>28.5</v>
       </c>
       <c r="AA231" t="n">
-        <v>40</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="232">
@@ -23293,7 +23293,7 @@
         <v>24.6</v>
       </c>
       <c r="AA232" t="n">
-        <v>38.3</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="233">
@@ -23396,7 +23396,7 @@
         <v>35.9</v>
       </c>
       <c r="AA233" t="n">
-        <v>40.7</v>
+        <v>231</v>
       </c>
     </row>
     <row r="234">
@@ -23499,7 +23499,7 @@
         <v>27.9</v>
       </c>
       <c r="AA234" t="n">
-        <v>40.6</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="235">
@@ -23596,7 +23596,7 @@
         <v>25.2</v>
       </c>
       <c r="AA235" t="n">
-        <v>45.7</v>
+        <v>508</v>
       </c>
     </row>
     <row r="236">
@@ -23699,7 +23699,7 @@
         <v>31.1</v>
       </c>
       <c r="AA236" t="n">
-        <v>42.9</v>
+        <v>994</v>
       </c>
     </row>
     <row r="237">
@@ -23796,7 +23796,7 @@
         <v>20.8</v>
       </c>
       <c r="AA237" t="n">
-        <v>42.4</v>
+        <v>542</v>
       </c>
     </row>
     <row r="238">
@@ -23893,7 +23893,7 @@
         <v>23.7</v>
       </c>
       <c r="AA238" t="n">
-        <v>41.7</v>
+        <v>929</v>
       </c>
     </row>
     <row r="239">
@@ -23990,7 +23990,7 @@
         <v>26.3</v>
       </c>
       <c r="AA239" t="n">
-        <v>40.1</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="240">
@@ -24093,7 +24093,7 @@
         <v>33.8</v>
       </c>
       <c r="AA240" t="n">
-        <v>43</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="241">
@@ -24196,7 +24196,7 @@
         <v>32.5</v>
       </c>
       <c r="AA241" t="n">
-        <v>41.6</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="242">
@@ -24299,7 +24299,7 @@
         <v>34.3</v>
       </c>
       <c r="AA242" t="n">
-        <v>40.7</v>
+        <v>492</v>
       </c>
     </row>
     <row r="243">
@@ -24402,7 +24402,7 @@
         <v>30.8</v>
       </c>
       <c r="AA243" t="n">
-        <v>44.3</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="244">
@@ -24499,7 +24499,7 @@
         <v>27.7</v>
       </c>
       <c r="AA244" t="n">
-        <v>39.5</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="245">
@@ -24596,7 +24596,7 @@
         <v>30.5</v>
       </c>
       <c r="AA245" t="n">
-        <v>40.6</v>
+        <v>663</v>
       </c>
     </row>
     <row r="246">
@@ -24693,7 +24693,7 @@
         <v>23.8</v>
       </c>
       <c r="AA246" t="n">
-        <v>50.4</v>
+        <v>391</v>
       </c>
     </row>
     <row r="247">
@@ -24796,7 +24796,7 @@
         <v>35.4</v>
       </c>
       <c r="AA247" t="n">
-        <v>41.8</v>
+        <v>500</v>
       </c>
     </row>
     <row r="248">
@@ -24893,7 +24893,7 @@
         <v>18.4</v>
       </c>
       <c r="AA248" t="n">
-        <v>40</v>
+        <v>380</v>
       </c>
     </row>
     <row r="249">
@@ -24990,7 +24990,7 @@
         <v>24.7</v>
       </c>
       <c r="AA249" t="n">
-        <v>42.8</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="250">
@@ -25087,7 +25087,7 @@
         <v>20.1</v>
       </c>
       <c r="AA250" t="n">
-        <v>40.9</v>
+        <v>328</v>
       </c>
     </row>
     <row r="251">
@@ -25184,7 +25184,7 @@
         <v>21</v>
       </c>
       <c r="AA251" t="n">
-        <v>38.7</v>
+        <v>768</v>
       </c>
     </row>
     <row r="252">
@@ -25281,7 +25281,7 @@
         <v>28.3</v>
       </c>
       <c r="AA252" t="n">
-        <v>44.3</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="253">
@@ -25384,7 +25384,7 @@
         <v>28.6</v>
       </c>
       <c r="AA253" t="n">
-        <v>40.2</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="254">
@@ -25481,7 +25481,7 @@
         <v>21</v>
       </c>
       <c r="AA254" t="n">
-        <v>43.4</v>
+        <v>514</v>
       </c>
     </row>
     <row r="255">
@@ -25578,7 +25578,7 @@
         <v>24.1</v>
       </c>
       <c r="AA255" t="n">
-        <v>50.3</v>
+        <v>676</v>
       </c>
     </row>
     <row r="256">
@@ -25681,7 +25681,7 @@
         <v>27</v>
       </c>
       <c r="AA256" t="n">
-        <v>40.8</v>
+        <v>693</v>
       </c>
     </row>
     <row r="257">
@@ -25784,7 +25784,7 @@
         <v>26.3</v>
       </c>
       <c r="AA257" t="n">
-        <v>44.1</v>
+        <v>463</v>
       </c>
     </row>
     <row r="258">
@@ -25887,7 +25887,7 @@
         <v>26.1</v>
       </c>
       <c r="AA258" t="n">
-        <v>44.7</v>
+        <v>628</v>
       </c>
     </row>
     <row r="259">
@@ -25990,7 +25990,7 @@
         <v>31.5</v>
       </c>
       <c r="AA259" t="n">
-        <v>42</v>
+        <v>987</v>
       </c>
     </row>
     <row r="260">
@@ -26093,7 +26093,7 @@
         <v>29.1</v>
       </c>
       <c r="AA260" t="n">
-        <v>40.1</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="261">
@@ -26196,7 +26196,7 @@
         <v>20.4</v>
       </c>
       <c r="AA261" t="n">
-        <v>39.3</v>
+        <v>392</v>
       </c>
     </row>
     <row r="262">
@@ -26293,7 +26293,7 @@
         <v>25.9</v>
       </c>
       <c r="AA262" t="n">
-        <v>42.3</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="263">
@@ -26390,7 +26390,7 @@
         <v>25.9</v>
       </c>
       <c r="AA263" t="n">
-        <v>41.2</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="264">
@@ -26493,7 +26493,7 @@
         <v>28.5</v>
       </c>
       <c r="AA264" t="n">
-        <v>47.2</v>
+        <v>943</v>
       </c>
     </row>
     <row r="265">
@@ -26590,7 +26590,7 @@
         <v>30.1</v>
       </c>
       <c r="AA265" t="n">
-        <v>41.6</v>
+        <v>764</v>
       </c>
     </row>
     <row r="266">
@@ -26693,7 +26693,7 @@
         <v>28.9</v>
       </c>
       <c r="AA266" t="n">
-        <v>42.3</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="267">
@@ -26790,7 +26790,7 @@
         <v>21.1</v>
       </c>
       <c r="AA267" t="n">
-        <v>39.9</v>
+        <v>963</v>
       </c>
     </row>
     <row r="268">
@@ -26893,7 +26893,7 @@
         <v>29.1</v>
       </c>
       <c r="AA268" t="n">
-        <v>39.8</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="269">
@@ -26996,7 +26996,7 @@
         <v>24.5</v>
       </c>
       <c r="AA269" t="n">
-        <v>42</v>
+        <v>519</v>
       </c>
     </row>
     <row r="270">
@@ -27099,7 +27099,7 @@
         <v>26.1</v>
       </c>
       <c r="AA270" t="n">
-        <v>39.2</v>
+        <v>597</v>
       </c>
     </row>
     <row r="271">
@@ -27196,7 +27196,7 @@
         <v>20.5</v>
       </c>
       <c r="AA271" t="n">
-        <v>41.5</v>
+        <v>434</v>
       </c>
     </row>
     <row r="272">
@@ -27299,7 +27299,7 @@
         <v>29.3</v>
       </c>
       <c r="AA272" t="n">
-        <v>40.2</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="273">
@@ -27402,7 +27402,7 @@
         <v>31.5</v>
       </c>
       <c r="AA273" t="n">
-        <v>39.9</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="274">
@@ -27505,7 +27505,7 @@
         <v>30.6</v>
       </c>
       <c r="AA274" t="n">
-        <v>41.2</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="275">
@@ -27608,7 +27608,7 @@
         <v>25.8</v>
       </c>
       <c r="AA275" t="n">
-        <v>41.9</v>
+        <v>938</v>
       </c>
     </row>
     <row r="276">
@@ -27705,7 +27705,7 @@
         <v>30.2</v>
       </c>
       <c r="AA276" t="n">
-        <v>43.4</v>
+        <v>705</v>
       </c>
     </row>
     <row r="277">
@@ -27808,7 +27808,7 @@
         <v>23.4</v>
       </c>
       <c r="AA277" t="n">
-        <v>38.1</v>
+        <v>197</v>
       </c>
     </row>
     <row r="278">
@@ -27911,7 +27911,7 @@
         <v>30.7</v>
       </c>
       <c r="AA278" t="n">
-        <v>39.3</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="279">
@@ -28014,7 +28014,7 @@
         <v>29.1</v>
       </c>
       <c r="AA279" t="n">
-        <v>42.8</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="280">
@@ -28117,7 +28117,7 @@
         <v>30.4</v>
       </c>
       <c r="AA280" t="n">
-        <v>39.8</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="281">
@@ -28220,7 +28220,7 @@
         <v>27.2</v>
       </c>
       <c r="AA281" t="n">
-        <v>46.4</v>
+        <v>801</v>
       </c>
     </row>
     <row r="282">
@@ -28317,7 +28317,7 @@
         <v>25.6</v>
       </c>
       <c r="AA282" t="n">
-        <v>43.8</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="283">
@@ -28414,7 +28414,7 @@
         <v>23.1</v>
       </c>
       <c r="AA283" t="n">
-        <v>44.1</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="284">
@@ -28511,7 +28511,7 @@
         <v>24.7</v>
       </c>
       <c r="AA284" t="n">
-        <v>41.9</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="285">
@@ -28614,7 +28614,7 @@
         <v>26.1</v>
       </c>
       <c r="AA285" t="n">
-        <v>40.1</v>
+        <v>751</v>
       </c>
     </row>
     <row r="286">
@@ -28711,7 +28711,7 @@
         <v>25.9</v>
       </c>
       <c r="AA286" t="n">
-        <v>42.3</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="287">
@@ -28808,7 +28808,7 @@
         <v>19.9</v>
       </c>
       <c r="AA287" t="n">
-        <v>38.4</v>
+        <v>632</v>
       </c>
     </row>
     <row r="288">
@@ -28905,7 +28905,7 @@
         <v>18.3</v>
       </c>
       <c r="AA288" t="n">
-        <v>38.6</v>
+        <v>350</v>
       </c>
     </row>
     <row r="289">
@@ -29008,7 +29008,7 @@
         <v>28.2</v>
       </c>
       <c r="AA289" t="n">
-        <v>47.2</v>
+        <v>950</v>
       </c>
     </row>
     <row r="290">
@@ -29105,7 +29105,7 @@
         <v>25</v>
       </c>
       <c r="AA290" t="n">
-        <v>48.1</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="291">
@@ -29202,7 +29202,7 @@
         <v>27</v>
       </c>
       <c r="AA291" t="n">
-        <v>41.5</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="292">
@@ -29299,7 +29299,7 @@
         <v>29</v>
       </c>
       <c r="AA292" t="n">
-        <v>43.8</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="293">
@@ -29396,7 +29396,7 @@
         <v>24.7</v>
       </c>
       <c r="AA293" t="n">
-        <v>42.8</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="294">
@@ -29493,7 +29493,7 @@
         <v>25.3</v>
       </c>
       <c r="AA294" t="n">
-        <v>43.6</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="295">
@@ -29590,7 +29590,7 @@
         <v>23.7</v>
       </c>
       <c r="AA295" t="n">
-        <v>41.6</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="296">
@@ -29687,7 +29687,7 @@
         <v>32.2</v>
       </c>
       <c r="AA296" t="n">
-        <v>41.6</v>
+        <v>397</v>
       </c>
     </row>
     <row r="297">
@@ -29784,7 +29784,7 @@
         <v>30</v>
       </c>
       <c r="AA297" t="n">
-        <v>43.2</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="298">
@@ -29881,7 +29881,7 @@
         <v>23.2</v>
       </c>
       <c r="AA298" t="n">
-        <v>47.9</v>
+        <v>685</v>
       </c>
     </row>
     <row r="299">
@@ -29978,7 +29978,7 @@
         <v>24.3</v>
       </c>
       <c r="AA299" t="n">
-        <v>44.9</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="300">
@@ -30075,7 +30075,7 @@
         <v>23.1</v>
       </c>
       <c r="AA300" t="n">
-        <v>44.1</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="301">
@@ -30172,7 +30172,7 @@
         <v>31.8</v>
       </c>
       <c r="AA301" t="n">
-        <v>40.9</v>
+        <v>66</v>
       </c>
     </row>
     <row r="302">
@@ -30269,7 +30269,7 @@
         <v>28</v>
       </c>
       <c r="AA302" t="n">
-        <v>44.3</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="303">
@@ -30366,7 +30366,7 @@
         <v>25</v>
       </c>
       <c r="AA303" t="n">
-        <v>47.7</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="304">
@@ -30463,7 +30463,7 @@
         <v>23.6</v>
       </c>
       <c r="AA304" t="n">
-        <v>38.8</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="305">
@@ -30560,7 +30560,7 @@
         <v>25.9</v>
       </c>
       <c r="AA305" t="n">
-        <v>42.3</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="306">
@@ -30657,7 +30657,7 @@
         <v>25.8</v>
       </c>
       <c r="AA306" t="n">
-        <v>39.8</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="307">
@@ -30754,7 +30754,7 @@
         <v>27</v>
       </c>
       <c r="AA307" t="n">
-        <v>41.5</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="308">
@@ -30851,7 +30851,7 @@
         <v>21.4</v>
       </c>
       <c r="AA308" t="n">
-        <v>36.3</v>
+        <v>168</v>
       </c>
     </row>
     <row r="309">
@@ -30948,7 +30948,7 @@
         <v>31.6</v>
       </c>
       <c r="AA309" t="n">
-        <v>41.3</v>
+        <v>453</v>
       </c>
     </row>
     <row r="310">
@@ -31045,7 +31045,7 @@
         <v>22.6</v>
       </c>
       <c r="AA310" t="n">
-        <v>38.6</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="311">
@@ -31142,7 +31142,7 @@
         <v>21</v>
       </c>
       <c r="AA311" t="n">
-        <v>38.7</v>
+        <v>768</v>
       </c>
     </row>
     <row r="312">
@@ -31239,7 +31239,7 @@
         <v>23.6</v>
       </c>
       <c r="AA312" t="n">
-        <v>42</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="313">
@@ -31328,7 +31328,7 @@
         <v>34.3</v>
       </c>
       <c r="AA313" t="n">
-        <v>43.8</v>
+        <v>3236</v>
       </c>
     </row>
     <row r="314">
@@ -31417,7 +31417,7 @@
         <v>34.3</v>
       </c>
       <c r="AA314" t="n">
-        <v>43.8</v>
+        <v>3235</v>
       </c>
     </row>
     <row r="315">
@@ -31506,7 +31506,7 @@
         <v>34.3</v>
       </c>
       <c r="AA315" t="n">
-        <v>43.8</v>
+        <v>3235</v>
       </c>
     </row>
     <row r="316">
@@ -31595,7 +31595,7 @@
         <v>33.9</v>
       </c>
       <c r="AA316" t="n">
-        <v>43.8</v>
+        <v>3284</v>
       </c>
     </row>
     <row r="317">
@@ -31684,7 +31684,7 @@
         <v>34.1</v>
       </c>
       <c r="AA317" t="n">
-        <v>43.6</v>
+        <v>3265</v>
       </c>
     </row>
     <row r="318">
@@ -31773,7 +31773,7 @@
         <v>34.3</v>
       </c>
       <c r="AA318" t="n">
-        <v>43.8</v>
+        <v>3237</v>
       </c>
     </row>
     <row r="319">
@@ -31862,7 +31862,7 @@
         <v>34.3</v>
       </c>
       <c r="AA319" t="n">
-        <v>43.8</v>
+        <v>3240</v>
       </c>
     </row>
     <row r="320">
@@ -31951,7 +31951,7 @@
         <v>34.3</v>
       </c>
       <c r="AA320" t="n">
-        <v>43.8</v>
+        <v>3236</v>
       </c>
     </row>
     <row r="321">
@@ -32040,7 +32040,7 @@
         <v>34.2</v>
       </c>
       <c r="AA321" t="n">
-        <v>43.9</v>
+        <v>3256</v>
       </c>
     </row>
     <row r="322">
@@ -32129,7 +32129,7 @@
         <v>34.3</v>
       </c>
       <c r="AA322" t="n">
-        <v>43.8</v>
+        <v>3239</v>
       </c>
     </row>
     <row r="323">
@@ -32218,7 +32218,7 @@
         <v>33.7</v>
       </c>
       <c r="AA323" t="n">
-        <v>43.7</v>
+        <v>3290</v>
       </c>
     </row>
     <row r="324">
@@ -32307,7 +32307,7 @@
         <v>34.3</v>
       </c>
       <c r="AA324" t="n">
-        <v>43.8</v>
+        <v>3237</v>
       </c>
     </row>
     <row r="325">
@@ -32396,7 +32396,7 @@
         <v>34</v>
       </c>
       <c r="AA325" t="n">
-        <v>43.7</v>
+        <v>3268</v>
       </c>
     </row>
     <row r="326">
@@ -32485,7 +32485,7 @@
         <v>33.7</v>
       </c>
       <c r="AA326" t="n">
-        <v>43.7</v>
+        <v>3297</v>
       </c>
     </row>
     <row r="327">
@@ -32574,7 +32574,7 @@
         <v>34</v>
       </c>
       <c r="AA327" t="n">
-        <v>43.5</v>
+        <v>3277</v>
       </c>
     </row>
     <row r="328">
@@ -32663,7 +32663,7 @@
         <v>34</v>
       </c>
       <c r="AA328" t="n">
-        <v>43.8</v>
+        <v>3276</v>
       </c>
     </row>
     <row r="329">
@@ -32752,7 +32752,7 @@
         <v>34.3</v>
       </c>
       <c r="AA329" t="n">
-        <v>43.8</v>
+        <v>3237</v>
       </c>
     </row>
     <row r="330">
@@ -32841,7 +32841,7 @@
         <v>34.2</v>
       </c>
       <c r="AA330" t="n">
-        <v>43.9</v>
+        <v>3262</v>
       </c>
     </row>
     <row r="331">
@@ -32930,7 +32930,7 @@
         <v>33.9</v>
       </c>
       <c r="AA331" t="n">
-        <v>43.6</v>
+        <v>3280</v>
       </c>
     </row>
     <row r="332">
@@ -33019,7 +33019,7 @@
         <v>34.3</v>
       </c>
       <c r="AA332" t="n">
-        <v>43.5</v>
+        <v>3261</v>
       </c>
     </row>
     <row r="333">
@@ -33108,7 +33108,7 @@
         <v>34.3</v>
       </c>
       <c r="AA333" t="n">
-        <v>43.8</v>
+        <v>3241</v>
       </c>
     </row>
     <row r="334">
@@ -33197,7 +33197,7 @@
         <v>34.3</v>
       </c>
       <c r="AA334" t="n">
-        <v>43.8</v>
+        <v>3235</v>
       </c>
     </row>
     <row r="335">
@@ -33286,7 +33286,7 @@
         <v>34.3</v>
       </c>
       <c r="AA335" t="n">
-        <v>43.6</v>
+        <v>3256</v>
       </c>
     </row>
     <row r="336">
@@ -33375,7 +33375,7 @@
         <v>33.9</v>
       </c>
       <c r="AA336" t="n">
-        <v>43.9</v>
+        <v>3281</v>
       </c>
     </row>
     <row r="337">
@@ -33464,7 +33464,7 @@
         <v>34.2</v>
       </c>
       <c r="AA337" t="n">
-        <v>43.8</v>
+        <v>3253</v>
       </c>
     </row>
     <row r="338">
@@ -33553,7 +33553,7 @@
         <v>34.3</v>
       </c>
       <c r="AA338" t="n">
-        <v>43.6</v>
+        <v>3253</v>
       </c>
     </row>
     <row r="339">
@@ -33642,7 +33642,7 @@
         <v>34</v>
       </c>
       <c r="AA339" t="n">
-        <v>43.8</v>
+        <v>3268</v>
       </c>
     </row>
     <row r="340">
@@ -33731,7 +33731,7 @@
         <v>34.4</v>
       </c>
       <c r="AA340" t="n">
-        <v>43.7</v>
+        <v>3242</v>
       </c>
     </row>
     <row r="341">
@@ -33814,7 +33814,7 @@
         <v>30.9</v>
       </c>
       <c r="AA341" t="n">
-        <v>43.3</v>
+        <v>4070</v>
       </c>
     </row>
     <row r="342">
@@ -33903,7 +33903,7 @@
         <v>34.3</v>
       </c>
       <c r="AA342" t="n">
-        <v>43.8</v>
+        <v>3238</v>
       </c>
     </row>
     <row r="343">
@@ -33992,7 +33992,7 @@
         <v>34</v>
       </c>
       <c r="AA343" t="n">
-        <v>43.7</v>
+        <v>3273</v>
       </c>
     </row>
     <row r="344">
@@ -34081,7 +34081,7 @@
         <v>33.9</v>
       </c>
       <c r="AA344" t="n">
-        <v>43.8</v>
+        <v>3276</v>
       </c>
     </row>
     <row r="345">
@@ -34170,7 +34170,7 @@
         <v>34</v>
       </c>
       <c r="AA345" t="n">
-        <v>43.8</v>
+        <v>3273</v>
       </c>
     </row>
     <row r="346">
@@ -34259,7 +34259,7 @@
         <v>33.5</v>
       </c>
       <c r="AA346" t="n">
-        <v>43.7</v>
+        <v>3317</v>
       </c>
     </row>
     <row r="347">
@@ -34348,7 +34348,7 @@
         <v>34.2</v>
       </c>
       <c r="AA347" t="n">
-        <v>43.7</v>
+        <v>3260</v>
       </c>
     </row>
     <row r="348">
@@ -34437,7 +34437,7 @@
         <v>33.5</v>
       </c>
       <c r="AA348" t="n">
-        <v>43.7</v>
+        <v>3310</v>
       </c>
     </row>
     <row r="349">
@@ -34526,7 +34526,7 @@
         <v>33.9</v>
       </c>
       <c r="AA349" t="n">
-        <v>43.8</v>
+        <v>3281</v>
       </c>
     </row>
     <row r="350">
@@ -34615,7 +34615,7 @@
         <v>34</v>
       </c>
       <c r="AA350" t="n">
-        <v>43.6</v>
+        <v>3270</v>
       </c>
     </row>
     <row r="351">
@@ -34704,7 +34704,7 @@
         <v>34.3</v>
       </c>
       <c r="AA351" t="n">
-        <v>43.8</v>
+        <v>3236</v>
       </c>
     </row>
     <row r="352">
@@ -34793,7 +34793,7 @@
         <v>33.7</v>
       </c>
       <c r="AA352" t="n">
-        <v>43.9</v>
+        <v>3297</v>
       </c>
     </row>
     <row r="353">
@@ -34882,7 +34882,7 @@
         <v>33.5</v>
       </c>
       <c r="AA353" t="n">
-        <v>43.6</v>
+        <v>3317</v>
       </c>
     </row>
     <row r="354">
@@ -34971,7 +34971,7 @@
         <v>33.7</v>
       </c>
       <c r="AA354" t="n">
-        <v>43.5</v>
+        <v>3296</v>
       </c>
     </row>
     <row r="355">
@@ -35060,7 +35060,7 @@
         <v>34.3</v>
       </c>
       <c r="AA355" t="n">
-        <v>43.9</v>
+        <v>3240</v>
       </c>
     </row>
     <row r="356">
@@ -35149,7 +35149,7 @@
         <v>34.1</v>
       </c>
       <c r="AA356" t="n">
-        <v>43.5</v>
+        <v>3268</v>
       </c>
     </row>
     <row r="357">
@@ -35238,7 +35238,7 @@
         <v>33.5</v>
       </c>
       <c r="AA357" t="n">
-        <v>43.7</v>
+        <v>3310</v>
       </c>
     </row>
     <row r="358">
@@ -35327,7 +35327,7 @@
         <v>34.3</v>
       </c>
       <c r="AA358" t="n">
-        <v>43.8</v>
+        <v>3239</v>
       </c>
     </row>
     <row r="359">
@@ -35416,7 +35416,7 @@
         <v>34.3</v>
       </c>
       <c r="AA359" t="n">
-        <v>43.8</v>
+        <v>3237</v>
       </c>
     </row>
     <row r="360">
@@ -35505,7 +35505,7 @@
         <v>34.3</v>
       </c>
       <c r="AA360" t="n">
-        <v>43.5</v>
+        <v>3261</v>
       </c>
     </row>
     <row r="361">
@@ -35594,7 +35594,7 @@
         <v>34.3</v>
       </c>
       <c r="AA361" t="n">
-        <v>43.6</v>
+        <v>3244</v>
       </c>
     </row>
     <row r="362">
@@ -35683,7 +35683,7 @@
         <v>34.3</v>
       </c>
       <c r="AA362" t="n">
-        <v>43.8</v>
+        <v>3235</v>
       </c>
     </row>
     <row r="363">
@@ -35772,7 +35772,7 @@
         <v>34.3</v>
       </c>
       <c r="AA363" t="n">
-        <v>43.8</v>
+        <v>3238</v>
       </c>
     </row>
     <row r="364">
@@ -35861,7 +35861,7 @@
         <v>34.2</v>
       </c>
       <c r="AA364" t="n">
-        <v>43.7</v>
+        <v>3246</v>
       </c>
     </row>
     <row r="365">
@@ -35950,7 +35950,7 @@
         <v>34.1</v>
       </c>
       <c r="AA365" t="n">
-        <v>43.8</v>
+        <v>3255</v>
       </c>
     </row>
     <row r="366">
@@ -36039,7 +36039,7 @@
         <v>34.3</v>
       </c>
       <c r="AA366" t="n">
-        <v>43.6</v>
+        <v>3255</v>
       </c>
     </row>
     <row r="367">
@@ -36128,7 +36128,7 @@
         <v>33.7</v>
       </c>
       <c r="AA367" t="n">
-        <v>43.7</v>
+        <v>3294</v>
       </c>
     </row>
     <row r="368">
@@ -36217,7 +36217,7 @@
         <v>33.7</v>
       </c>
       <c r="AA368" t="n">
-        <v>43.8</v>
+        <v>3295</v>
       </c>
     </row>
     <row r="369">
@@ -36306,7 +36306,7 @@
         <v>34.3</v>
       </c>
       <c r="AA369" t="n">
-        <v>43.8</v>
+        <v>3235</v>
       </c>
     </row>
     <row r="370">
@@ -36395,7 +36395,7 @@
         <v>33.8</v>
       </c>
       <c r="AA370" t="n">
-        <v>43.7</v>
+        <v>3291</v>
       </c>
     </row>
     <row r="371">
@@ -36484,7 +36484,7 @@
         <v>34.3</v>
       </c>
       <c r="AA371" t="n">
-        <v>43.7</v>
+        <v>3241</v>
       </c>
     </row>
     <row r="372">
@@ -36573,7 +36573,7 @@
         <v>33.8</v>
       </c>
       <c r="AA372" t="n">
-        <v>43.7</v>
+        <v>3291</v>
       </c>
     </row>
     <row r="373">
@@ -36662,7 +36662,7 @@
         <v>33.8</v>
       </c>
       <c r="AA373" t="n">
-        <v>43.9</v>
+        <v>3286</v>
       </c>
     </row>
     <row r="374">
@@ -36751,7 +36751,7 @@
         <v>33.8</v>
       </c>
       <c r="AA374" t="n">
-        <v>43.7</v>
+        <v>3283</v>
       </c>
     </row>
     <row r="375">
@@ -36840,7 +36840,7 @@
         <v>33.7</v>
       </c>
       <c r="AA375" t="n">
-        <v>43.7</v>
+        <v>3293</v>
       </c>
     </row>
     <row r="376">
@@ -36929,7 +36929,7 @@
         <v>34.2</v>
       </c>
       <c r="AA376" t="n">
-        <v>43.9</v>
+        <v>3250</v>
       </c>
     </row>
     <row r="377">
@@ -37018,7 +37018,7 @@
         <v>34.2</v>
       </c>
       <c r="AA377" t="n">
-        <v>43.8</v>
+        <v>3244</v>
       </c>
     </row>
     <row r="378">
@@ -37107,7 +37107,7 @@
         <v>34.3</v>
       </c>
       <c r="AA378" t="n">
-        <v>43.8</v>
+        <v>3244</v>
       </c>
     </row>
     <row r="379">
@@ -37196,7 +37196,7 @@
         <v>33.6</v>
       </c>
       <c r="AA379" t="n">
-        <v>43.8</v>
+        <v>3307</v>
       </c>
     </row>
     <row r="380">
@@ -37285,7 +37285,7 @@
         <v>34.1</v>
       </c>
       <c r="AA380" t="n">
-        <v>43.5</v>
+        <v>3266</v>
       </c>
     </row>
     <row r="381">
@@ -37374,7 +37374,7 @@
         <v>34.4</v>
       </c>
       <c r="AA381" t="n">
-        <v>43.7</v>
+        <v>3242</v>
       </c>
     </row>
     <row r="382">
@@ -37463,7 +37463,7 @@
         <v>34.3</v>
       </c>
       <c r="AA382" t="n">
-        <v>43.7</v>
+        <v>3242</v>
       </c>
     </row>
     <row r="383">
@@ -37552,7 +37552,7 @@
         <v>34.2</v>
       </c>
       <c r="AA383" t="n">
-        <v>43.4</v>
+        <v>3270</v>
       </c>
     </row>
     <row r="384">
@@ -37641,7 +37641,7 @@
         <v>34.3</v>
       </c>
       <c r="AA384" t="n">
-        <v>43.8</v>
+        <v>3235</v>
       </c>
     </row>
     <row r="385">
@@ -37730,7 +37730,7 @@
         <v>34.1</v>
       </c>
       <c r="AA385" t="n">
-        <v>43.6</v>
+        <v>3264</v>
       </c>
     </row>
     <row r="386">
@@ -37819,7 +37819,7 @@
         <v>34.3</v>
       </c>
       <c r="AA386" t="n">
-        <v>43.8</v>
+        <v>3236</v>
       </c>
     </row>
     <row r="387">
@@ -37908,7 +37908,7 @@
         <v>34.3</v>
       </c>
       <c r="AA387" t="n">
-        <v>43.8</v>
+        <v>3239</v>
       </c>
     </row>
     <row r="388">
@@ -37997,7 +37997,7 @@
         <v>33.8</v>
       </c>
       <c r="AA388" t="n">
-        <v>43.9</v>
+        <v>3285</v>
       </c>
     </row>
     <row r="389">
@@ -38086,7 +38086,7 @@
         <v>33.7</v>
       </c>
       <c r="AA389" t="n">
-        <v>43.8</v>
+        <v>3298</v>
       </c>
     </row>
     <row r="390">
@@ -38175,7 +38175,7 @@
         <v>33.8</v>
       </c>
       <c r="AA390" t="n">
-        <v>43.8</v>
+        <v>3293</v>
       </c>
     </row>
     <row r="391">
@@ -38264,7 +38264,7 @@
         <v>34.3</v>
       </c>
       <c r="AA391" t="n">
-        <v>43.5</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="392">
@@ -38353,7 +38353,7 @@
         <v>34</v>
       </c>
       <c r="AA392" t="n">
-        <v>43.7</v>
+        <v>3268</v>
       </c>
     </row>
     <row r="393">
@@ -38442,7 +38442,7 @@
         <v>34.3</v>
       </c>
       <c r="AA393" t="n">
-        <v>43.8</v>
+        <v>3236</v>
       </c>
     </row>
     <row r="394">
@@ -38531,7 +38531,7 @@
         <v>34.1</v>
       </c>
       <c r="AA394" t="n">
-        <v>43.8</v>
+        <v>3256</v>
       </c>
     </row>
     <row r="395">
@@ -38620,7 +38620,7 @@
         <v>34.3</v>
       </c>
       <c r="AA395" t="n">
-        <v>43.8</v>
+        <v>3238</v>
       </c>
     </row>
     <row r="396">
@@ -38709,7 +38709,7 @@
         <v>34.3</v>
       </c>
       <c r="AA396" t="n">
-        <v>43.8</v>
+        <v>3235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 데이터 업데이트 - 2026-05-25 13:48
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,42 +556,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Notts County</t>
+          <t>IK Start</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Salford City</t>
+          <t>Valerenga</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="E2" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="F2" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>무승부</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="I2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>England League Two+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -605,22 +605,22 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="N2" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O2" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>2:2</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -629,97 +629,101 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>8</v>
+        <v>76.2</v>
       </c>
       <c r="T2" t="n">
-        <v>47.4</v>
+        <v>56.1</v>
       </c>
       <c r="U2" t="n">
-        <v>1.9</v>
+        <v>56.7</v>
       </c>
       <c r="V2" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="W2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="X2" t="n">
-        <v>41.7</v>
+        <v>40</v>
       </c>
       <c r="Y2" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="Z2" t="n">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="AA2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Suwon Bluewings</t>
+          <t>Notts County</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cheonan City</t>
+          <t>Salford City</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.5</v>
+        <v>2.6</v>
       </c>
       <c r="E3" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="F3" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
+        <v>2.6</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 2+</t>
+          <t>England League Two+</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="N3" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="O3" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -728,97 +732,101 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>57.7</v>
+        <v>8</v>
       </c>
       <c r="T3" t="n">
-        <v>47.7</v>
+        <v>47.4</v>
       </c>
       <c r="U3" t="n">
-        <v>35.3</v>
+        <v>1.9</v>
       </c>
       <c r="V3" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="W3" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="X3" t="n">
-        <v>20</v>
+        <v>41.7</v>
       </c>
       <c r="Y3" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="Z3" t="n">
-        <v>20</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AA3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>26/05/2026 0:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paju Citizen</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GimPo Citizen</t>
+          <t>Moss FK</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.7</v>
+        <v>1.7</v>
       </c>
       <c r="E4" t="n">
-        <v>3.1</v>
+        <v>4.1</v>
       </c>
       <c r="F4" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+        <v>4.1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 2+</t>
+          <t>Norway 1. Division+</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="N4" t="n">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="O4" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>3:2</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -827,70 +835,68 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>87.5</v>
       </c>
       <c r="T4" t="n">
-        <v>47.4</v>
+        <v>63.6</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>73.5</v>
       </c>
       <c r="V4" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="W4" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="X4" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="Y4" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="Z4" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="AA4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Los Angeles FC</t>
+          <t>Suwon Bluewings</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Seattle Sounders</t>
+          <t>Cheonan City</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="E5" t="n">
         <v>3.8</v>
       </c>
       <c r="F5" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+        <v>5.2</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -903,81 +909,93 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>42</v>
+      </c>
+      <c r="N5" t="n">
+        <v>35</v>
+      </c>
+      <c r="O5" t="n">
+        <v>23</v>
+      </c>
       <c r="P5" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="S5" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T5" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="U5" t="n">
+        <v>35.3</v>
+      </c>
       <c r="V5" t="n">
-        <v>45.5</v>
+        <v>40</v>
       </c>
       <c r="W5" t="n">
-        <v>27.3</v>
+        <v>40</v>
       </c>
       <c r="X5" t="n">
-        <v>27.3</v>
+        <v>20</v>
       </c>
       <c r="Y5" t="n">
-        <v>27.3</v>
+        <v>20</v>
       </c>
       <c r="Z5" t="n">
-        <v>4.5</v>
+        <v>20</v>
       </c>
       <c r="AA5" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>26/05/2026 3:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paderborn</t>
+          <t>Paju Citizen</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wolfsburg</t>
+          <t>GimPo Citizen</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
       <c r="E6" t="n">
-        <v>3.7</v>
+        <v>3.1</v>
       </c>
       <c r="F6" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Germany Bundesliga+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -991,17 +1009,17 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="N6" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="O6" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1015,68 +1033,68 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>32.3</v>
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>46.9</v>
+        <v>47.4</v>
       </c>
       <c r="U6" t="n">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>11.1</v>
+        <v>25</v>
       </c>
       <c r="W6" t="n">
-        <v>33.3</v>
+        <v>25</v>
       </c>
       <c r="X6" t="n">
-        <v>55.6</v>
+        <v>50</v>
       </c>
       <c r="Y6" t="n">
-        <v>44.4</v>
+        <v>50</v>
       </c>
       <c r="Z6" t="n">
-        <v>22.2</v>
+        <v>25</v>
       </c>
       <c r="AA6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>26/05/2026 4:00</t>
+          <t>26/05/2026 0:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>St Mirren</t>
+          <t>HamKam</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Partick Thistle</t>
+          <t>Lillestrom SK</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.7</v>
+        <v>2.9</v>
       </c>
       <c r="E7" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="F7" t="n">
-        <v>4.6</v>
+        <v>2.3</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Scotland Premiership+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1086,26 +1104,26 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="N7" t="n">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="O7" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1114,68 +1132,68 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>32.3</v>
       </c>
       <c r="T7" t="n">
-        <v>47.4</v>
+        <v>47</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="V7" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
         <v>33.3</v>
       </c>
-      <c r="X7" t="n">
-        <v>16.7</v>
-      </c>
       <c r="Y7" t="n">
-        <v>33.3</v>
+        <v>55.6</v>
       </c>
       <c r="Z7" t="n">
         <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>26/05/2026 7:00</t>
+          <t>26/05/2026 0:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>KFUM Oslo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Athletic Club MG</t>
+          <t>Rosenborg BK</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="E8" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1189,22 +1207,22 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="N8" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="O8" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1213,22 +1231,22 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>57.7</v>
       </c>
       <c r="T8" t="n">
-        <v>47.4</v>
+        <v>46.8</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>35.3</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="W8" t="n">
-        <v>66.7</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="Y8" t="n">
         <v>0</v>
@@ -1237,33 +1255,33 @@
         <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>26/05/2026 8:00</t>
+          <t>26/05/2026 0:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Aalesund FK</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.7</v>
+        <v>1.4</v>
       </c>
       <c r="E9" t="n">
-        <v>3.2</v>
+        <v>4.7</v>
       </c>
       <c r="F9" t="n">
-        <v>2.6</v>
+        <v>6.5</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
@@ -1274,7 +1292,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1284,26 +1302,26 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="N9" t="n">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="O9" t="n">
         <v>21</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1315,28 +1333,1493 @@
         <v>76.2</v>
       </c>
       <c r="T9" t="n">
-        <v>56.8</v>
+        <v>56.1</v>
       </c>
       <c r="U9" t="n">
         <v>56.7</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>100</v>
+      </c>
+      <c r="Z9" t="n">
         <v>50</v>
-      </c>
-      <c r="X9" t="n">
-        <v>50</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>0</v>
       </c>
       <c r="AA9" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>26/05/2026 0:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sarpsborg 08</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Molde</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Norway Eliteserien+</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>28</v>
+      </c>
+      <c r="N10" t="n">
+        <v>31</v>
+      </c>
+      <c r="O10" t="n">
+        <v>41</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T10" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="U10" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V10" t="n">
+        <v>50</v>
+      </c>
+      <c r="W10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X10" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>26/05/2026 0:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Raufoss IL</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>9</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>40</v>
+      </c>
+      <c r="N11" t="n">
+        <v>26</v>
+      </c>
+      <c r="O11" t="n">
+        <v>34</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T11" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="U11" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V11" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="W11" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="X11" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>26/05/2026 0:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ranheim Fotball</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>9</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>38</v>
+      </c>
+      <c r="N12" t="n">
+        <v>30</v>
+      </c>
+      <c r="O12" t="n">
+        <v>31</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T12" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="U12" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V12" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="W12" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="X12" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>26/05/2026 0:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>27</v>
+      </c>
+      <c r="N13" t="n">
+        <v>36</v>
+      </c>
+      <c r="O13" t="n">
+        <v>37</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="T13" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="U13" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" t="n">
+        <v>40</v>
+      </c>
+      <c r="X13" t="n">
+        <v>60</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>40</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>26/05/2026 0:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>IL Hodd</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Egersunds IK</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>38</v>
+      </c>
+      <c r="N14" t="n">
+        <v>34</v>
+      </c>
+      <c r="O14" t="n">
+        <v>28</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T14" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="U14" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V14" t="n">
+        <v>25</v>
+      </c>
+      <c r="W14" t="n">
+        <v>50</v>
+      </c>
+      <c r="X14" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>26/05/2026 0:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Stromsgodset IF</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Bryne FK</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>56</v>
+      </c>
+      <c r="N15" t="n">
+        <v>23</v>
+      </c>
+      <c r="O15" t="n">
+        <v>21</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T15" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="U15" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V15" t="n">
+        <v>75</v>
+      </c>
+      <c r="W15" t="n">
+        <v>25</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>26/05/2026 0:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>26</v>
+      </c>
+      <c r="N16" t="n">
+        <v>45</v>
+      </c>
+      <c r="O16" t="n">
+        <v>28</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T16" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="U16" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="n">
+        <v>50</v>
+      </c>
+      <c r="X16" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>26/05/2026 0:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Lyn Oslo</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Strommen IF</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>30</v>
+      </c>
+      <c r="N17" t="n">
+        <v>44</v>
+      </c>
+      <c r="O17" t="n">
+        <v>26</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T17" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="U17" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V17" t="n">
+        <v>40</v>
+      </c>
+      <c r="W17" t="n">
+        <v>40</v>
+      </c>
+      <c r="X17" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Los Angeles FC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Seattle Sounders</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>23</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>USA Major League Soccer+</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="W18" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="X18" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>26/05/2026 2:15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sandefjord</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fredrikstad</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>7</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Norway Eliteserien+</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>52</v>
+      </c>
+      <c r="N19" t="n">
+        <v>26</v>
+      </c>
+      <c r="O19" t="n">
+        <v>23</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>8</v>
+      </c>
+      <c r="T19" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="U19" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V19" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="W19" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="X19" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>26/05/2026 3:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Paderborn</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Wolfsburg</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>9</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Germany Bundesliga+</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>27</v>
+      </c>
+      <c r="N20" t="n">
+        <v>39</v>
+      </c>
+      <c r="O20" t="n">
+        <v>34</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T20" t="n">
+        <v>47</v>
+      </c>
+      <c r="U20" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V20" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="W20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X20" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>26/05/2026 4:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>St Mirren</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Partick Thistle</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Scotland Premiership+</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>25</v>
+      </c>
+      <c r="N21" t="n">
+        <v>39</v>
+      </c>
+      <c r="O21" t="n">
+        <v>37</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" t="n">
+        <v>50</v>
+      </c>
+      <c r="W21" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X21" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>26/05/2026 7:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Athletic Club MG</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>3</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>23</v>
+      </c>
+      <c r="N22" t="n">
+        <v>43</v>
+      </c>
+      <c r="O22" t="n">
+        <v>34</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="X22" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>26/05/2026 8:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Coritiba</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Brazil Serie A+</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>26</v>
+      </c>
+      <c r="N23" t="n">
+        <v>53</v>
+      </c>
+      <c r="O23" t="n">
+        <v>21</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T23" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="U23" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" t="n">
+        <v>50</v>
+      </c>
+      <c r="X23" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ODD Ballklubb</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>18</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="W24" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="X24" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 데이터 업데이트 - 2026-05-26 08:41
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -1050,7 +1050,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1089,22 +1089,22 @@
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>54.5</v>
+        <v>58.3</v>
       </c>
       <c r="W7" t="n">
-        <v>27.3</v>
+        <v>25</v>
       </c>
       <c r="X7" t="n">
-        <v>18.2</v>
+        <v>16.7</v>
       </c>
       <c r="Y7" t="n">
-        <v>45.5</v>
+        <v>50</v>
       </c>
       <c r="Z7" t="n">
-        <v>18.2</v>
+        <v>25</v>
       </c>
       <c r="AA7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
📊 데이터 업데이트 - 2026-05-26 17:12
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -628,7 +628,7 @@
         <v>32.3</v>
       </c>
       <c r="T2" t="n">
-        <v>47</v>
+        <v>46.3</v>
       </c>
       <c r="U2" t="n">
         <v>14.3</v>
@@ -727,7 +727,7 @@
         <v>32.3</v>
       </c>
       <c r="T3" t="n">
-        <v>47</v>
+        <v>46.3</v>
       </c>
       <c r="U3" t="n">
         <v>14.3</v>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1178,22 +1178,22 @@
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>50</v>
+        <v>51.6</v>
       </c>
       <c r="W8" t="n">
-        <v>20</v>
+        <v>19.4</v>
       </c>
       <c r="X8" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Y8" t="n">
-        <v>33.3</v>
+        <v>32.3</v>
       </c>
       <c r="Z8" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
📊 데이터 업데이트 - 2026-05-27 08:34
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,261 +556,259 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>27/05/2026 3:30</t>
+          <t>27/05/2026 7:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Greuther Fürth</t>
+          <t>LDU</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Essen</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="E2" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Always Ready</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Germany 2. Bundesliga+</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="N2" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="O2" t="n">
+        <v>19</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>8</v>
+      </c>
+      <c r="T2" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V2" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="W2" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="X2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="AA2" t="n">
         <v>52</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>0:2</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="T2" t="n">
-        <v>46.3</v>
-      </c>
-      <c r="U2" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="V2" t="n">
-        <v>100</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>100</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>27/05/2026 3:45</t>
+          <t>27/05/2026 7:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Saint-Etienne</t>
+          <t>Lanús</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Nice</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Mirassol SP</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I3" t="n">
+        <v>84</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>30</v>
+      </c>
+      <c r="N3" t="n">
+        <v>27</v>
+      </c>
+      <c r="O3" t="n">
+        <v>43</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
         <v>8</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>France Ligue 1+</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>35</v>
-      </c>
-      <c r="N3" t="n">
-        <v>37</v>
-      </c>
-      <c r="O3" t="n">
-        <v>28</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
-        <v>32.3</v>
-      </c>
       <c r="T3" t="n">
-        <v>46.3</v>
+        <v>46.5</v>
       </c>
       <c r="U3" t="n">
-        <v>14.3</v>
+        <v>1.9</v>
       </c>
       <c r="V3" t="n">
-        <v>25</v>
+        <v>40.5</v>
       </c>
       <c r="W3" t="n">
-        <v>50</v>
+        <v>13.1</v>
       </c>
       <c r="X3" t="n">
-        <v>25</v>
+        <v>46.4</v>
       </c>
       <c r="Y3" t="n">
-        <v>0</v>
+        <v>45.2</v>
       </c>
       <c r="Z3" t="n">
-        <v>0</v>
+        <v>13.1</v>
       </c>
       <c r="AA3" t="n">
-        <v>8</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>28/05/2026 9:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lanus</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mirassol</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.7</v>
-      </c>
+          <t>CA Platense</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>45</v>
+      </c>
       <c r="I4" t="n">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>45</v>
+      </c>
+      <c r="N4" t="n">
+        <v>26</v>
+      </c>
+      <c r="O4" t="n">
+        <v>29</v>
+      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -818,61 +816,69 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="S4" t="n">
+        <v>8</v>
+      </c>
+      <c r="T4" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U4" t="n">
+        <v>1.9</v>
+      </c>
       <c r="V4" t="n">
-        <v>58.8</v>
+        <v>48.2</v>
       </c>
       <c r="W4" t="n">
-        <v>17.6</v>
+        <v>14.1</v>
       </c>
       <c r="X4" t="n">
-        <v>23.5</v>
+        <v>37.6</v>
       </c>
       <c r="Y4" t="n">
-        <v>52.9</v>
+        <v>48.2</v>
       </c>
       <c r="Z4" t="n">
-        <v>17.6</v>
+        <v>21.2</v>
       </c>
       <c r="AA4" t="n">
-        <v>17</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>27/05/2026 9:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LDU de Quito</t>
+          <t>Universitario</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Always Ready</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.4</v>
+        <v>2.5</v>
       </c>
       <c r="E5" t="n">
-        <v>5.1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>6.6</v>
+        <v>2.9</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>38</v>
+      </c>
       <c r="I5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -881,7 +887,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -889,17 +895,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>30</v>
+      </c>
+      <c r="N5" t="n">
+        <v>32</v>
+      </c>
+      <c r="O5" t="n">
+        <v>38</v>
+      </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -907,70 +919,78 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="S5" t="n">
+        <v>8</v>
+      </c>
+      <c r="T5" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U5" t="n">
+        <v>1.9</v>
+      </c>
       <c r="V5" t="n">
-        <v>69.2</v>
+        <v>72.7</v>
       </c>
       <c r="W5" t="n">
-        <v>23.1</v>
+        <v>27.3</v>
       </c>
       <c r="X5" t="n">
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>46.2</v>
+        <v>27.3</v>
       </c>
       <c r="Z5" t="n">
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>28/05/2026 7:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gremio</t>
+          <t>Ind del Valle</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Atletico Torque</t>
+          <t>Rosario Central</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="E6" t="n">
-        <v>4.2</v>
+        <v>3.4</v>
       </c>
       <c r="F6" t="n">
-        <v>6.5</v>
+        <v>4</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>무승부</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>36</v>
+      </c>
       <c r="I6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana+</t>
+          <t>World CONMEBOL Libertadores+</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -978,17 +998,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>34</v>
+      </c>
+      <c r="N6" t="n">
+        <v>36</v>
+      </c>
+      <c r="O6" t="n">
+        <v>30</v>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -996,88 +1022,96 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
       <c r="V6" t="n">
-        <v>63.6</v>
+        <v>35.7</v>
       </c>
       <c r="W6" t="n">
-        <v>27.3</v>
+        <v>21.4</v>
       </c>
       <c r="X6" t="n">
-        <v>9.1</v>
+        <v>42.9</v>
       </c>
       <c r="Y6" t="n">
-        <v>27.3</v>
+        <v>21.4</v>
       </c>
       <c r="Z6" t="n">
-        <v>9.1</v>
+        <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>28/05/2026 9:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="E7" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="F7" t="n">
-        <v>5.2</v>
-      </c>
+          <t>Deportivo La Guaira</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>무승부</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>36</v>
+      </c>
       <c r="I7" t="n">
-        <v>12</v>
+        <v>107</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana+</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>34</v>
+      </c>
+      <c r="N7" t="n">
+        <v>36</v>
+      </c>
+      <c r="O7" t="n">
+        <v>30</v>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1085,88 +1119,96 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T7" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="U7" t="n">
+        <v>14.3</v>
+      </c>
       <c r="V7" t="n">
-        <v>58.3</v>
+        <v>47.7</v>
       </c>
       <c r="W7" t="n">
-        <v>25</v>
+        <v>15.9</v>
       </c>
       <c r="X7" t="n">
-        <v>16.7</v>
+        <v>36.4</v>
       </c>
       <c r="Y7" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="Z7" t="n">
-        <v>25</v>
+        <v>11.2</v>
       </c>
       <c r="AA7" t="n">
-        <v>12</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>28/05/2026 9:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Palestino</t>
+          <t>Peñarol</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Deportivo Riestra</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F8" t="n">
-        <v>3.1</v>
-      </c>
+          <t>Ind Santa Fe</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+          <t>무승부</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>38</v>
+      </c>
       <c r="I8" t="n">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana+</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>27</v>
+      </c>
+      <c r="N8" t="n">
+        <v>38</v>
+      </c>
+      <c r="O8" t="n">
+        <v>35</v>
+      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1174,113 +1216,1550 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T8" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="U8" t="n">
+        <v>14.3</v>
+      </c>
       <c r="V8" t="n">
-        <v>51.6</v>
+        <v>40.9</v>
       </c>
       <c r="W8" t="n">
-        <v>19.4</v>
+        <v>15.1</v>
       </c>
       <c r="X8" t="n">
-        <v>29</v>
+        <v>44.1</v>
       </c>
       <c r="Y8" t="n">
-        <v>32.3</v>
+        <v>46.2</v>
       </c>
       <c r="Z8" t="n">
-        <v>6.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AA8" t="n">
-        <v>31</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>28/05/2026 9:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>46</v>
+      </c>
+      <c r="I9" t="n">
+        <v>61</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>30</v>
+      </c>
+      <c r="N9" t="n">
+        <v>24</v>
+      </c>
+      <c r="O9" t="n">
+        <v>46</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>8</v>
+      </c>
+      <c r="T9" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U9" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V9" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="W9" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>27/05/2026 9:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Estudiantes La Plata</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ind Medellin</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores+</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>30</v>
+      </c>
+      <c r="N10" t="n">
+        <v>44</v>
+      </c>
+      <c r="O10" t="n">
+        <v>26</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" t="n">
+        <v>25</v>
+      </c>
+      <c r="W10" t="n">
+        <v>50</v>
+      </c>
+      <c r="X10" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>27/05/2026 9:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cusco FC</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores+</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>52</v>
+      </c>
+      <c r="N11" t="n">
+        <v>34</v>
+      </c>
+      <c r="O11" t="n">
+        <v>14</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>8</v>
+      </c>
+      <c r="T11" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>27/05/2026 9:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Nacional (URU)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Coquimbo Unido</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores+</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>35</v>
+      </c>
+      <c r="N12" t="n">
+        <v>40</v>
+      </c>
+      <c r="O12" t="n">
+        <v>25</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T12" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="U12" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V12" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="W12" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="X12" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>27/05/2026 9:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>San Lorenzo</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Deportivo Recoleta</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>35</v>
+      </c>
+      <c r="N13" t="n">
+        <v>49</v>
+      </c>
+      <c r="O13" t="n">
+        <v>16</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T13" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="U13" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V13" t="n">
+        <v>100</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>27/05/2026 9:30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Deportivo Cuenca</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>22</v>
+      </c>
+      <c r="N14" t="n">
+        <v>35</v>
+      </c>
+      <c r="O14" t="n">
+        <v>43</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>8</v>
+      </c>
+      <c r="T14" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U14" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" t="n">
+        <v>100</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>28/05/2026 7:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Libertad</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>UCV FC</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores+</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>50</v>
+      </c>
+      <c r="N15" t="n">
+        <v>22</v>
+      </c>
+      <c r="O15" t="n">
+        <v>28</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T15" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="U15" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="n">
+        <v>100</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>28/05/2026 7:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Caracas</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Botafogo</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>8</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>33</v>
+      </c>
+      <c r="N16" t="n">
+        <v>35</v>
+      </c>
+      <c r="O16" t="n">
+        <v>32</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T16" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="U16" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V16" t="n">
+        <v>25</v>
+      </c>
+      <c r="W16" t="n">
+        <v>50</v>
+      </c>
+      <c r="X16" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>25</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>28/05/2026 7:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Cienciano</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Juventud LP</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>29</v>
+      </c>
+      <c r="N17" t="n">
+        <v>49</v>
+      </c>
+      <c r="O17" t="n">
+        <v>22</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="n">
+        <v>50</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>28/05/2026 7:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Barracas Central</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>30</v>
+      </c>
+      <c r="N18" t="n">
+        <v>38</v>
+      </c>
+      <c r="O18" t="n">
+        <v>32</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>25</v>
+      </c>
+      <c r="W18" t="n">
+        <v>50</v>
+      </c>
+      <c r="X18" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>28/05/2026 7:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Olimpia Asunción</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Audax Italiano</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>61</v>
+      </c>
+      <c r="N19" t="n">
+        <v>23</v>
+      </c>
+      <c r="O19" t="n">
+        <v>16</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>8</v>
+      </c>
+      <c r="T19" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="U19" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V19" t="n">
+        <v>50</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Estudiantes L.P.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Independiente Medellin</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F20" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>9</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores+</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="W20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X20" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Sao Paulo</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Boston River</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Rosario Central</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>25</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores+</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="n">
+        <v>52</v>
+      </c>
+      <c r="W21" t="n">
+        <v>20</v>
+      </c>
+      <c r="X21" t="n">
+        <v>28</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>32</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Club Nacional</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Coquimbo Unido</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>12</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores+</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="W22" t="n">
+        <v>25</v>
+      </c>
+      <c r="X22" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Atletico-MG</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Puerto Cabello</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
         <v>1.2</v>
       </c>
-      <c r="E9" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="F9" t="n">
+      <c r="E23" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="F23" t="n">
         <v>12</v>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
         <v>9</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>World CONMEBOL Sudamericana+</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>❓</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="n">
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="n">
         <v>55.6</v>
       </c>
-      <c r="W9" t="n">
+      <c r="W23" t="n">
         <v>33.3</v>
       </c>
-      <c r="X9" t="n">
+      <c r="X23" t="n">
         <v>11.1</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Y23" t="n">
         <v>33.3</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="Z23" t="n">
         <v>11.1</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AA23" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Olimpia</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>A. Italiano</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>13</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="W24" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="X24" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 데이터 업데이트 - 2026-05-29 08:18
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA15"/>
+  <dimension ref="A1:AA22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,17 +556,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>29/05/2026 9:30</t>
+          <t>29/05/2026 7:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Boca Juniors</t>
+          <t>Cerro Porteño</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Universidad Católica</t>
+          <t>Sporting Cristal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -578,10 +578,10 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="I2" t="n">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -590,7 +590,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -599,17 +599,17 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="N2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -623,47 +623,47 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>8</v>
+        <v>32.3</v>
       </c>
       <c r="T2" t="n">
-        <v>46.8</v>
+        <v>44.6</v>
       </c>
       <c r="U2" t="n">
-        <v>1.9</v>
+        <v>14.3</v>
       </c>
       <c r="V2" t="n">
-        <v>64.3</v>
+        <v>66.2</v>
       </c>
       <c r="W2" t="n">
-        <v>10.7</v>
+        <v>16.9</v>
       </c>
       <c r="X2" t="n">
-        <v>25</v>
+        <v>16.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>57.1</v>
+        <v>52.3</v>
       </c>
       <c r="Z2" t="n">
-        <v>28.6</v>
+        <v>32.3</v>
       </c>
       <c r="AA2" t="n">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>28/05/2026 9:30</t>
+          <t>29/05/2026 9:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Peñarol</t>
+          <t>Boca Juniors</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ind Santa Fe</t>
+          <t>Universidad Católica</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -671,14 +671,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>무승부</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="I3" t="n">
-        <v>96</v>
+        <v>57</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -687,7 +687,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -696,22 +696,22 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="N3" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="O3" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -720,71 +720,77 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>32.3</v>
+        <v>8</v>
       </c>
       <c r="T3" t="n">
-        <v>45.7</v>
+        <v>48</v>
       </c>
       <c r="U3" t="n">
-        <v>14.3</v>
+        <v>1.9</v>
       </c>
       <c r="V3" t="n">
-        <v>41.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="W3" t="n">
-        <v>14.6</v>
+        <v>10.5</v>
       </c>
       <c r="X3" t="n">
-        <v>43.8</v>
+        <v>24.6</v>
       </c>
       <c r="Y3" t="n">
-        <v>46.9</v>
+        <v>57.9</v>
       </c>
       <c r="Z3" t="n">
-        <v>10.4</v>
+        <v>28.1</v>
       </c>
       <c r="AA3" t="n">
-        <v>96</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>29/05/2026 9:30</t>
+          <t>30/05/2026 2:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>KFUM Oslo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Barcelona SC</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>Tromso</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.4</v>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I4" t="n">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -793,22 +799,22 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="N4" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="O4" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -817,97 +823,95 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T4" t="n">
-        <v>46.8</v>
+        <v>48.5</v>
       </c>
       <c r="U4" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V4" t="n">
-        <v>37.9</v>
+        <v>41.2</v>
       </c>
       <c r="W4" t="n">
-        <v>19</v>
+        <v>11.8</v>
       </c>
       <c r="X4" t="n">
-        <v>43.1</v>
+        <v>47.1</v>
       </c>
       <c r="Y4" t="n">
-        <v>46.6</v>
+        <v>35.3</v>
       </c>
       <c r="Z4" t="n">
-        <v>13.8</v>
+        <v>0</v>
       </c>
       <c r="AA4" t="n">
-        <v>58</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>28/05/2026 9:30</t>
+          <t>29/05/2026 7:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Deportivo La Guaira</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="F5" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Junior Barranquilla</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
+        <v>59</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>CLA</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="N5" t="n">
+        <v>22</v>
+      </c>
+      <c r="O5" t="n">
         <v>36</v>
       </c>
-      <c r="O5" t="n">
-        <v>30</v>
-      </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -916,73 +920,77 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>32.3</v>
+        <v>8</v>
       </c>
       <c r="T5" t="n">
-        <v>45.7</v>
+        <v>48</v>
       </c>
       <c r="U5" t="n">
-        <v>14.3</v>
+        <v>1.9</v>
       </c>
       <c r="V5" t="n">
-        <v>20</v>
+        <v>37.3</v>
       </c>
       <c r="W5" t="n">
-        <v>60</v>
+        <v>18.6</v>
       </c>
       <c r="X5" t="n">
-        <v>20</v>
+        <v>44.1</v>
       </c>
       <c r="Y5" t="n">
-        <v>0</v>
+        <v>45.8</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="AA5" t="n">
-        <v>5</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>28/05/2026 9:30</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Shenyang City</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CA Platense</t>
+          <t>Shanghai SIPG</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="E6" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
+        <v>2.8</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>무승부</t>
+        </is>
+      </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>China Super League+</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -991,22 +999,22 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="N6" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="O6" t="n">
         <v>29</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1015,64 +1023,64 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>8</v>
+        <v>32.3</v>
       </c>
       <c r="T6" t="n">
-        <v>46.8</v>
+        <v>44.6</v>
       </c>
       <c r="U6" t="n">
-        <v>1.9</v>
+        <v>14.3</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="W6" t="n">
-        <v>33.3</v>
+        <v>41.7</v>
       </c>
       <c r="X6" t="n">
-        <v>66.7</v>
+        <v>25</v>
       </c>
       <c r="Y6" t="n">
-        <v>66.7</v>
+        <v>16.7</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>28/05/2026 9:30</t>
+          <t>29/05/2026 9:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bolívar</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Barcelona SC</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="E7" t="n">
-        <v>3.4</v>
+        <v>5.5</v>
       </c>
       <c r="F7" t="n">
-        <v>2.8</v>
+        <v>12.2</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1090,22 +1098,22 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="N7" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O7" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1117,7 +1125,7 @@
         <v>8</v>
       </c>
       <c r="T7" t="n">
-        <v>46.8</v>
+        <v>48</v>
       </c>
       <c r="U7" t="n">
         <v>1.9</v>
@@ -1126,52 +1134,52 @@
         <v>66.7</v>
       </c>
       <c r="W7" t="n">
-        <v>11.1</v>
+        <v>33.3</v>
       </c>
       <c r="X7" t="n">
-        <v>22.2</v>
+        <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>77.8</v>
+        <v>33.3</v>
       </c>
       <c r="Z7" t="n">
-        <v>11.1</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>28/05/2026 9:30</t>
+          <t>29/05/2026 9:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>River Plate</t>
+          <t>América de Cali</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Blooming</t>
+          <t>Macará</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="E8" t="n">
-        <v>10.2</v>
+        <v>3.5</v>
       </c>
       <c r="F8" t="n">
-        <v>24</v>
+        <v>5.2</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1189,13 +1197,13 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="N8" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="O8" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1216,61 +1224,61 @@
         <v>8</v>
       </c>
       <c r="T8" t="n">
-        <v>46.8</v>
+        <v>48</v>
       </c>
       <c r="U8" t="n">
         <v>1.9</v>
       </c>
       <c r="V8" t="n">
-        <v>100</v>
+        <v>37.5</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>37.5</v>
       </c>
       <c r="Y8" t="n">
-        <v>100</v>
+        <v>37.5</v>
       </c>
       <c r="Z8" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="AA8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>28/05/2026 9:30</t>
+          <t>29/05/2026 9:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RB Bragantino</t>
+          <t>CA Tigre</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Carabobo</t>
+          <t>Alianza Atlético</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="E9" t="n">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="F9" t="n">
-        <v>9.300000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1288,22 +1296,22 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="N9" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="O9" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1312,22 +1320,22 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>32.3</v>
+        <v>8</v>
       </c>
       <c r="T9" t="n">
-        <v>45.7</v>
+        <v>48</v>
       </c>
       <c r="U9" t="n">
-        <v>14.3</v>
+        <v>1.9</v>
       </c>
       <c r="V9" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="W9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="X9" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="Y9" t="n">
         <v>0</v>
@@ -1336,44 +1344,44 @@
         <v>0</v>
       </c>
       <c r="AA9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>29/05/2026 4:00</t>
+          <t>30/05/2026 2:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Casa Pia AC</t>
+          <t>Fredrikstad</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>União Torreense</t>
+          <t>IK Start</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2.3</v>
+        <v>1.7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="F10" t="n">
-        <v>3.3</v>
+        <v>4.2</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Portugal Primeira Liga+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1387,22 +1395,22 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="N10" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O10" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1411,68 +1419,68 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>32.3</v>
+        <v>76.2</v>
       </c>
       <c r="T10" t="n">
-        <v>45.7</v>
+        <v>51</v>
       </c>
       <c r="U10" t="n">
-        <v>14.3</v>
+        <v>56.7</v>
       </c>
       <c r="V10" t="n">
-        <v>33.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>66.7</v>
+        <v>28.6</v>
       </c>
       <c r="Y10" t="n">
-        <v>66.7</v>
+        <v>57.1</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>42.9</v>
       </c>
       <c r="AA10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>29/05/2026 7:00</t>
+          <t>30/05/2026 2:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cerro Porteño</t>
+          <t>Valerenga</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sporting Cristal</t>
+          <t>Kristiansund BK</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>1.6</v>
       </c>
       <c r="E11" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="F11" t="n">
-        <v>5.6</v>
+        <v>5</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1486,17 +1494,17 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="N11" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="O11" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1510,68 +1518,68 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>32.3</v>
+        <v>57.7</v>
       </c>
       <c r="T11" t="n">
-        <v>45.7</v>
+        <v>48.5</v>
       </c>
       <c r="U11" t="n">
-        <v>14.3</v>
+        <v>35.3</v>
       </c>
       <c r="V11" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="W11" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X11" t="n">
         <v>50</v>
       </c>
-      <c r="W11" t="n">
-        <v>50</v>
-      </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="Z11" t="n">
         <v>0</v>
       </c>
-      <c r="Y11" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>50</v>
-      </c>
       <c r="AA11" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>29/05/2026 7:00</t>
+          <t>30/05/2026 2:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Junior Barranquilla</t>
+          <t>Sarpsborg 08</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="E12" t="n">
-        <v>5.6</v>
+        <v>4.3</v>
       </c>
       <c r="F12" t="n">
-        <v>10</v>
+        <v>4.5</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1585,17 +1593,17 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="N12" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="O12" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1609,70 +1617,68 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T12" t="n">
-        <v>46.8</v>
+        <v>48.5</v>
       </c>
       <c r="U12" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V12" t="n">
-        <v>66.7</v>
+        <v>33.3</v>
       </c>
       <c r="W12" t="n">
         <v>33.3</v>
       </c>
       <c r="X12" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="Y12" t="n">
         <v>33.3</v>
       </c>
       <c r="Z12" t="n">
-        <v>0</v>
+        <v>16.7</v>
       </c>
       <c r="AA12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>30/05/2026 2:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bolívar</t>
+          <t>Rosenborg BK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Independ. Rivadavia</t>
+          <t>Bodo/Glimt</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="E13" t="n">
-        <v>3.4</v>
+        <v>4.5</v>
       </c>
       <c r="F13" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+        <v>1.6</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
       <c r="I13" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1682,20 +1688,26 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>26</v>
+      </c>
+      <c r="N13" t="n">
+        <v>18</v>
+      </c>
+      <c r="O13" t="n">
+        <v>57</v>
+      </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1:3</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1703,52 +1715,58 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
+      <c r="S13" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T13" t="n">
+        <v>51</v>
+      </c>
+      <c r="U13" t="n">
+        <v>56.7</v>
+      </c>
       <c r="V13" t="n">
-        <v>38.5</v>
+        <v>100</v>
       </c>
       <c r="W13" t="n">
-        <v>25.6</v>
+        <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>35.9</v>
+        <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>38.5</v>
+        <v>100</v>
       </c>
       <c r="Z13" t="n">
-        <v>10.3</v>
+        <v>0</v>
       </c>
       <c r="AA13" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>30/05/2026 2:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cerro Porteno</t>
+          <t>Aalesund FK</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sporting Cristal</t>
+          <t>HamKam</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="F14" t="n">
-        <v>5.6</v>
+        <v>3.2</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
@@ -1759,7 +1777,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1772,17 +1790,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>28</v>
+      </c>
+      <c r="N14" t="n">
+        <v>30</v>
+      </c>
+      <c r="O14" t="n">
+        <v>42</v>
+      </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1790,23 +1814,29 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
+      <c r="S14" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T14" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="U14" t="n">
+        <v>35.3</v>
+      </c>
       <c r="V14" t="n">
         <v>55.6</v>
       </c>
       <c r="W14" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="X14" t="n">
         <v>33.3</v>
       </c>
-      <c r="X14" t="n">
-        <v>11.1</v>
-      </c>
       <c r="Y14" t="n">
-        <v>33.3</v>
+        <v>22.2</v>
       </c>
       <c r="Z14" t="n">
-        <v>11.1</v>
+        <v>0</v>
       </c>
       <c r="AA14" t="n">
         <v>9</v>
@@ -1815,90 +1845,743 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>30/05/2026 3:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Penarol</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Catanzaro</t>
         </is>
       </c>
       <c r="D15" t="n">
         <v>1.8</v>
       </c>
       <c r="E15" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>8</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Italy Serie B+</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>50</v>
+      </c>
+      <c r="N15" t="n">
+        <v>33</v>
+      </c>
+      <c r="O15" t="n">
+        <v>17</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T15" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="U15" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V15" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="W15" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="X15" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>30/05/2026 3:45</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Nice</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Saint-Etienne</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>France Ligue 1+</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>29</v>
+      </c>
+      <c r="N16" t="n">
+        <v>47</v>
+      </c>
+      <c r="O16" t="n">
+        <v>24</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T16" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="U16" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V16" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="W16" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X16" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>30/05/2026 7:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Cerro Largo</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CA Cerro</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Uruguay Primera División - Apertura+</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>59</v>
+      </c>
+      <c r="N17" t="n">
+        <v>23</v>
+      </c>
+      <c r="O17" t="n">
+        <v>18</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T17" t="n">
+        <v>51</v>
+      </c>
+      <c r="U17" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cobresal</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nublense</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E18" t="n">
         <v>3.5</v>
       </c>
-      <c r="F15" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="F18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>30</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Chile Primera División+</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="W18" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="X18" t="n">
+        <v>40</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>30</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Shenyang Urban</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SHANGHAI SIPG</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>25</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>China Super League+</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="n">
+        <v>44</v>
+      </c>
+      <c r="W19" t="n">
+        <v>24</v>
+      </c>
+      <c r="X19" t="n">
+        <v>32</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>40</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Boca Juniors</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>U. Catolica</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>12</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores+</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="W20" t="n">
+        <v>25</v>
+      </c>
+      <c r="X20" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tigre</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Alianza Atletico</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F21" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>10</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="n">
+        <v>50</v>
+      </c>
+      <c r="W21" t="n">
+        <v>30</v>
+      </c>
+      <c r="X21" t="n">
         <v>20</v>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>World CONMEBOL Libertadores+</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
+      <c r="Y21" t="n">
+        <v>30</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>America de Cali</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Macara</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>14</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Sudamericana+</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>❓</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="n">
-        <v>60</v>
-      </c>
-      <c r="W15" t="n">
-        <v>20</v>
-      </c>
-      <c r="X15" t="n">
-        <v>20</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>40</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>15</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>20</v>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="n">
+        <v>50</v>
+      </c>
+      <c r="W22" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="X22" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 데이터 업데이트 - 2026-05-30 09:43
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA22"/>
+  <dimension ref="A1:AA48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,60 +556,66 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>29/05/2026 7:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cerro Porteño</t>
+          <t>Busan I'Park</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sporting Cristal</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>Paju Citizen</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.6</v>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="I2" t="n">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="N2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O2" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -623,90 +629,96 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>32.3</v>
+        <v>8</v>
       </c>
       <c r="T2" t="n">
-        <v>44.6</v>
+        <v>48</v>
       </c>
       <c r="U2" t="n">
-        <v>14.3</v>
+        <v>1.9</v>
       </c>
       <c r="V2" t="n">
-        <v>66.2</v>
+        <v>52.9</v>
       </c>
       <c r="W2" t="n">
-        <v>16.9</v>
+        <v>17.6</v>
       </c>
       <c r="X2" t="n">
-        <v>16.9</v>
+        <v>29.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>52.3</v>
+        <v>41.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>32.3</v>
+        <v>11.8</v>
       </c>
       <c r="AA2" t="n">
-        <v>65</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>29/05/2026 9:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Boca Juniors</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Universidad Católica</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>Lyn Oslo</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.2</v>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I3" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>Norway 1. Division+</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="N3" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="O3" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -720,72 +732,72 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T3" t="n">
-        <v>48</v>
+        <v>48.5</v>
       </c>
       <c r="U3" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V3" t="n">
-        <v>64.90000000000001</v>
+        <v>50</v>
       </c>
       <c r="W3" t="n">
-        <v>10.5</v>
+        <v>21.4</v>
       </c>
       <c r="X3" t="n">
-        <v>24.6</v>
+        <v>28.6</v>
       </c>
       <c r="Y3" t="n">
-        <v>57.9</v>
+        <v>35.7</v>
       </c>
       <c r="Z3" t="n">
-        <v>28.1</v>
+        <v>14.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>30/05/2026 2:00</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KFUM Oslo</t>
+          <t>Real Sociedad B</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tromso</t>
+          <t>Cultural Leonesa</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="E4" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="F4" t="n">
-        <v>2.4</v>
+        <v>3.1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I4" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -795,26 +807,26 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="N4" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="O4" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -823,90 +835,96 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>57.7</v>
+        <v>32.3</v>
       </c>
       <c r="T4" t="n">
-        <v>48.5</v>
+        <v>44.7</v>
       </c>
       <c r="U4" t="n">
-        <v>35.3</v>
+        <v>14.3</v>
       </c>
       <c r="V4" t="n">
-        <v>41.2</v>
+        <v>45.5</v>
       </c>
       <c r="W4" t="n">
-        <v>11.8</v>
+        <v>18.2</v>
       </c>
       <c r="X4" t="n">
-        <v>47.1</v>
+        <v>36.4</v>
       </c>
       <c r="Y4" t="n">
-        <v>35.3</v>
+        <v>18.2</v>
       </c>
       <c r="Z4" t="n">
         <v>0</v>
       </c>
       <c r="AA4" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>29/05/2026 7:00</t>
+          <t>31/05/2026 4:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Junior Barranquilla</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+          <t>Sporting Gijón</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.9</v>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I5" t="n">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>CLA</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="N5" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="O5" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -920,72 +938,72 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T5" t="n">
-        <v>48</v>
+        <v>48.5</v>
       </c>
       <c r="U5" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V5" t="n">
-        <v>37.3</v>
+        <v>50</v>
       </c>
       <c r="W5" t="n">
-        <v>18.6</v>
+        <v>20</v>
       </c>
       <c r="X5" t="n">
-        <v>44.1</v>
+        <v>30</v>
       </c>
       <c r="Y5" t="n">
-        <v>45.8</v>
+        <v>40</v>
       </c>
       <c r="Z5" t="n">
-        <v>13.6</v>
+        <v>10</v>
       </c>
       <c r="AA5" t="n">
-        <v>59</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Shenyang City</t>
+          <t>Vegalta Sendai</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Shanghai SIPG</t>
+          <t>Ventforet Kofu</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="E6" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="F6" t="n">
-        <v>2.8</v>
+        <v>4.5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>무승부</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>China Super League+</t>
+          <t>Japan J2/J3 League+</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -999,22 +1017,22 @@
         </is>
       </c>
       <c r="M6" t="n">
+        <v>35</v>
+      </c>
+      <c r="N6" t="n">
         <v>33</v>
       </c>
-      <c r="N6" t="n">
-        <v>38</v>
-      </c>
       <c r="O6" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1026,70 +1044,74 @@
         <v>32.3</v>
       </c>
       <c r="T6" t="n">
-        <v>44.6</v>
+        <v>44.7</v>
       </c>
       <c r="U6" t="n">
         <v>14.3</v>
       </c>
       <c r="V6" t="n">
-        <v>33.3</v>
+        <v>38.5</v>
       </c>
       <c r="W6" t="n">
-        <v>41.7</v>
+        <v>30.8</v>
       </c>
       <c r="X6" t="n">
-        <v>25</v>
+        <v>30.8</v>
       </c>
       <c r="Y6" t="n">
-        <v>16.7</v>
+        <v>15.4</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>29/05/2026 9:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Kataller Toyama</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Barcelona SC</t>
+          <t>Tegevajaro Miyazaki</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
       <c r="E7" t="n">
-        <v>5.5</v>
+        <v>3.2</v>
       </c>
       <c r="F7" t="n">
-        <v>12.2</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
+        <v>2.9</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>Japan J2/J3 League+</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1098,22 +1120,22 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="N7" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="O7" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1122,73 +1144,77 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T7" t="n">
-        <v>48</v>
+        <v>48.5</v>
       </c>
       <c r="U7" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V7" t="n">
-        <v>66.7</v>
+        <v>40</v>
       </c>
       <c r="W7" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="X7" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="Y7" t="n">
-        <v>33.3</v>
+        <v>46.7</v>
       </c>
       <c r="Z7" t="n">
-        <v>0</v>
+        <v>13.3</v>
       </c>
       <c r="AA7" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>29/05/2026 9:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>América de Cali</t>
+          <t>Qingdao West Coast</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Macará</t>
+          <t>Shanghai Shenhua</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="E8" t="n">
         <v>3.5</v>
       </c>
       <c r="F8" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
+        <v>2.9</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>무승부</t>
+        </is>
+      </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="I8" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana+</t>
+          <t>China Super League+</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1197,22 +1223,22 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="N8" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O8" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1221,73 +1247,77 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
         <v>48</v>
       </c>
       <c r="U8" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>37.5</v>
+        <v>28.6</v>
       </c>
       <c r="W8" t="n">
-        <v>25</v>
+        <v>35.7</v>
       </c>
       <c r="X8" t="n">
-        <v>37.5</v>
+        <v>35.7</v>
       </c>
       <c r="Y8" t="n">
-        <v>37.5</v>
+        <v>21.4</v>
       </c>
       <c r="Z8" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>29/05/2026 9:30</t>
+          <t>31/05/2026 5:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CA Tigre</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Alianza Atlético</t>
+          <t>Botafogo</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="E9" t="n">
-        <v>5.8</v>
+        <v>3.5</v>
       </c>
       <c r="F9" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+        <v>3.9</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>무승부</t>
+        </is>
+      </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana+</t>
+          <t>Brazil Serie A+</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1296,22 +1326,22 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="N9" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="O9" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1320,68 +1350,68 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>8</v>
+        <v>32.3</v>
       </c>
       <c r="T9" t="n">
-        <v>48</v>
+        <v>44.7</v>
       </c>
       <c r="U9" t="n">
-        <v>1.9</v>
+        <v>14.3</v>
       </c>
       <c r="V9" t="n">
-        <v>25</v>
+        <v>45.5</v>
       </c>
       <c r="W9" t="n">
-        <v>50</v>
+        <v>18.2</v>
       </c>
       <c r="X9" t="n">
-        <v>25</v>
+        <v>36.4</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>18.2</v>
       </c>
       <c r="Z9" t="n">
         <v>0</v>
       </c>
       <c r="AA9" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>30/05/2026 2:00</t>
+          <t>30/05/2026 9:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fredrikstad</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>IK Start</t>
+          <t>América Mineiro</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="E10" t="n">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
       <c r="F10" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1395,17 +1425,17 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="N10" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="O10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1419,68 +1449,68 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>76.2</v>
+        <v>8</v>
       </c>
       <c r="T10" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="U10" t="n">
-        <v>56.7</v>
+        <v>1.9</v>
       </c>
       <c r="V10" t="n">
-        <v>71.40000000000001</v>
+        <v>50</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="X10" t="n">
-        <v>28.6</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="n">
-        <v>57.1</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>42.9</v>
+        <v>0</v>
       </c>
       <c r="AA10" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>30/05/2026 2:00</t>
+          <t>30/05/2026 9:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Valerenga</t>
+          <t>Univ de Concepcion</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kristiansund BK</t>
+          <t>Unión La Calera</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="E11" t="n">
-        <v>4.4</v>
+        <v>3.4</v>
       </c>
       <c r="F11" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>Chile Primera División+</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1494,13 +1524,13 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="N11" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="O11" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1527,59 +1557,59 @@
         <v>35.3</v>
       </c>
       <c r="V11" t="n">
-        <v>16.7</v>
+        <v>40</v>
       </c>
       <c r="W11" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="X11" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="Y11" t="n">
-        <v>16.7</v>
+        <v>40</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AA11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>30/05/2026 2:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Yongin City</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sarpsborg 08</t>
+          <t>Daegu FC</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1.6</v>
+        <v>3.9</v>
       </c>
       <c r="E12" t="n">
-        <v>4.3</v>
+        <v>3.6</v>
       </c>
       <c r="F12" t="n">
-        <v>4.5</v>
+        <v>1.7</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1589,26 +1619,26 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="N12" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="O12" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1617,68 +1647,68 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>57.7</v>
+        <v>8</v>
       </c>
       <c r="T12" t="n">
-        <v>48.5</v>
+        <v>48</v>
       </c>
       <c r="U12" t="n">
-        <v>35.3</v>
+        <v>1.9</v>
       </c>
       <c r="V12" t="n">
-        <v>33.3</v>
+        <v>14.3</v>
       </c>
       <c r="W12" t="n">
-        <v>33.3</v>
+        <v>42.9</v>
       </c>
       <c r="X12" t="n">
-        <v>33.3</v>
+        <v>42.9</v>
       </c>
       <c r="Y12" t="n">
-        <v>33.3</v>
+        <v>14.3</v>
       </c>
       <c r="Z12" t="n">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="AA12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>30/05/2026 2:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Rosenborg BK</t>
+          <t>Asan Mugunghwa</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bodo/Glimt</t>
+          <t>Suwon Bluewings</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
       <c r="E13" t="n">
-        <v>4.5</v>
+        <v>3.3</v>
       </c>
       <c r="F13" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1692,17 +1722,17 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="N13" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="O13" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1716,57 +1746,57 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>76.2</v>
+        <v>57.7</v>
       </c>
       <c r="T13" t="n">
-        <v>51</v>
+        <v>48.5</v>
       </c>
       <c r="U13" t="n">
-        <v>56.7</v>
+        <v>35.3</v>
       </c>
       <c r="V13" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="Y13" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="Z13" t="n">
         <v>0</v>
       </c>
       <c r="AA13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>30/05/2026 2:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Aalesund FK</t>
+          <t>Suwon FC</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HamKam</t>
+          <t>Seongnam FC</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E14" t="n">
-        <v>3.7</v>
+        <v>3.3</v>
       </c>
       <c r="F14" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
@@ -1777,7 +1807,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1791,22 +1821,22 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="N14" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="O14" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>2:2</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1815,25 +1845,25 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>57.7</v>
+        <v>76.2</v>
       </c>
       <c r="T14" t="n">
-        <v>48.5</v>
+        <v>50</v>
       </c>
       <c r="U14" t="n">
-        <v>35.3</v>
+        <v>56.7</v>
       </c>
       <c r="V14" t="n">
-        <v>55.6</v>
+        <v>22.2</v>
       </c>
       <c r="W14" t="n">
-        <v>11.1</v>
+        <v>33.3</v>
       </c>
       <c r="X14" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="Y14" t="n">
         <v>33.3</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>22.2</v>
       </c>
       <c r="Z14" t="n">
         <v>0</v>
@@ -1845,38 +1875,38 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>30/05/2026 3:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Gimhae City</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Catanzaro</t>
+          <t>GimPo Citizen</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.8</v>
+        <v>4.7</v>
       </c>
       <c r="E15" t="n">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="F15" t="n">
-        <v>4.2</v>
+        <v>1.6</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Italy Serie B+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1886,26 +1916,26 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="N15" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="O15" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1914,68 +1944,68 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>32.3</v>
+        <v>57.7</v>
       </c>
       <c r="T15" t="n">
-        <v>44.6</v>
+        <v>48.5</v>
       </c>
       <c r="U15" t="n">
-        <v>14.3</v>
+        <v>35.3</v>
       </c>
       <c r="V15" t="n">
-        <v>62.5</v>
+        <v>11.1</v>
       </c>
       <c r="W15" t="n">
-        <v>12.5</v>
+        <v>11.1</v>
       </c>
       <c r="X15" t="n">
-        <v>25</v>
+        <v>77.8</v>
       </c>
       <c r="Y15" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="Z15" t="n">
-        <v>25</v>
+        <v>33.3</v>
       </c>
       <c r="AA15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>30/05/2026 3:45</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Chengdu Qianbao</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Saint-Etienne</t>
+          <t>Shandong Luneng</t>
         </is>
       </c>
       <c r="D16" t="n">
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
       <c r="F16" t="n">
-        <v>4.4</v>
+        <v>3.1</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>France Ligue 1+</t>
+          <t>China Super League+</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1989,22 +2019,22 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="N16" t="n">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="O16" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2013,68 +2043,68 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>32.3</v>
+        <v>57.7</v>
       </c>
       <c r="T16" t="n">
-        <v>44.6</v>
+        <v>48.5</v>
       </c>
       <c r="U16" t="n">
-        <v>14.3</v>
+        <v>35.3</v>
       </c>
       <c r="V16" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="W16" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="X16" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="Y16" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="Z16" t="n">
         <v>0</v>
       </c>
       <c r="AA16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>30/05/2026 7:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cerro Largo</t>
+          <t>Chongqing Tongliang</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CA Cerro</t>
+          <t>Beijing Guoan</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2.1</v>
+        <v>3.9</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F17" t="n">
-        <v>3.3</v>
+        <v>1.9</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Uruguay Primera División - Apertura+</t>
+          <t>China Super League+</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2084,21 +2114,21 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="N17" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="O17" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2112,70 +2142,68 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>76.2</v>
+        <v>8</v>
       </c>
       <c r="T17" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="U17" t="n">
-        <v>56.7</v>
+        <v>1.9</v>
       </c>
       <c r="V17" t="n">
-        <v>66.7</v>
+        <v>20</v>
       </c>
       <c r="W17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="X17" t="n">
-        <v>33.3</v>
+        <v>40</v>
       </c>
       <c r="Y17" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="Z17" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="AA17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cobresal</t>
+          <t>Sichuan FC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nublense</t>
+          <t>Qingdao Jonoon</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2.9</v>
+        <v>1.9</v>
       </c>
       <c r="E18" t="n">
         <v>3.5</v>
       </c>
       <c r="F18" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+        <v>3.7</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
       <c r="I18" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Chile Primera División+</t>
+          <t>China Super League+</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2185,20 +2213,26 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>48</v>
+      </c>
+      <c r="N18" t="n">
+        <v>21</v>
+      </c>
+      <c r="O18" t="n">
+        <v>31</v>
+      </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2206,88 +2240,98 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
+      <c r="S18" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T18" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="U18" t="n">
+        <v>35.3</v>
+      </c>
       <c r="V18" t="n">
-        <v>43.3</v>
+        <v>37.5</v>
       </c>
       <c r="W18" t="n">
-        <v>16.7</v>
+        <v>25</v>
       </c>
       <c r="X18" t="n">
-        <v>40</v>
+        <v>37.5</v>
       </c>
       <c r="Y18" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="Z18" t="n">
-        <v>6.7</v>
+        <v>0</v>
       </c>
       <c r="AA18" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Shenyang Urban</t>
+          <t>Racing Club (URU)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SHANGHAI SIPG</t>
+          <t>Defensor Sporting</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="E19" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="F19" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+        <v>3.9</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
       <c r="I19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Uruguay Primera División - Apertura+</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>51</v>
+      </c>
+      <c r="N19" t="n">
         <v>25</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>China Super League+</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="O19" t="n">
+        <v>24</v>
+      </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3:0</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2295,65 +2339,69 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
+      <c r="S19" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T19" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="U19" t="n">
+        <v>35.3</v>
+      </c>
       <c r="V19" t="n">
-        <v>44</v>
+        <v>83.3</v>
       </c>
       <c r="W19" t="n">
-        <v>24</v>
+        <v>16.7</v>
       </c>
       <c r="X19" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="Y19" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="Z19" t="n">
-        <v>12</v>
+        <v>16.7</v>
       </c>
       <c r="AA19" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Boca Juniors</t>
+          <t>Molde</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>U. Catolica</t>
+          <t>Sandefjord</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="F20" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
+        <v>4.8</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
       <c r="I20" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>World CONMEBOL Libertadores+</t>
+          <t>Norway Eliteserien+</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2366,17 +2414,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>44</v>
+      </c>
+      <c r="N20" t="n">
+        <v>27</v>
+      </c>
+      <c r="O20" t="n">
+        <v>29</v>
+      </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2384,204 +2438,2584 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
+      <c r="S20" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T20" t="n">
+        <v>50</v>
+      </c>
+      <c r="U20" t="n">
+        <v>56.7</v>
+      </c>
       <c r="V20" t="n">
-        <v>58.3</v>
+        <v>40</v>
       </c>
       <c r="W20" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="X20" t="n">
-        <v>16.7</v>
+        <v>40</v>
       </c>
       <c r="Y20" t="n">
-        <v>33.3</v>
+        <v>40</v>
       </c>
       <c r="Z20" t="n">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tigre</t>
+          <t>Moss FK</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Alianza Atletico</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1.2</v>
+        <v>2.8</v>
       </c>
       <c r="E21" t="n">
-        <v>5.8</v>
+        <v>3.9</v>
       </c>
       <c r="F21" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>8</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>23</v>
+      </c>
+      <c r="N21" t="n">
+        <v>34</v>
+      </c>
+      <c r="O21" t="n">
+        <v>43</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T21" t="n">
+        <v>50</v>
+      </c>
+      <c r="U21" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V21" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="W21" t="n">
         <v>12.5</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="n">
-        <v>10</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>World CONMEBOL Sudamericana+</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="n">
+      <c r="X21" t="n">
         <v>50</v>
       </c>
-      <c r="W21" t="n">
-        <v>30</v>
-      </c>
-      <c r="X21" t="n">
-        <v>20</v>
-      </c>
       <c r="Y21" t="n">
-        <v>30</v>
+        <v>37.5</v>
       </c>
       <c r="Z21" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA21" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>23:15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>AD Ceuta</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Albacete Balompie</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>8</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Spain Segunda División+</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>21</v>
+      </c>
+      <c r="N22" t="n">
+        <v>47</v>
+      </c>
+      <c r="O22" t="n">
+        <v>31</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T22" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="U22" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V22" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="W22" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="X22" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>31/05/2026 3:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Danubio FC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CA Progreso</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Uruguay Primera División - Apertura+</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>54</v>
+      </c>
+      <c r="N23" t="n">
+        <v>26</v>
+      </c>
+      <c r="O23" t="n">
+        <v>20</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>8</v>
+      </c>
+      <c r="T23" t="n">
+        <v>48</v>
+      </c>
+      <c r="U23" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V23" t="n">
+        <v>100</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>31/05/2026 4:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Coritiba</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Brazil Serie A+</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>41</v>
+      </c>
+      <c r="N24" t="n">
+        <v>30</v>
+      </c>
+      <c r="O24" t="n">
+        <v>29</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T24" t="n">
+        <v>50</v>
+      </c>
+      <c r="U24" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V24" t="n">
+        <v>60</v>
+      </c>
+      <c r="W24" t="n">
+        <v>40</v>
+      </c>
+      <c r="X24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>31/05/2026 4:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>La Serena</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Colo Colo</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Chile Primera División+</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>19</v>
+      </c>
+      <c r="N25" t="n">
+        <v>20</v>
+      </c>
+      <c r="O25" t="n">
+        <v>61</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T25" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="U25" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>31/05/2026 6:30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Univ de Chile</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Deportes Concepción</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Chile Primera División+</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>45</v>
+      </c>
+      <c r="N26" t="n">
+        <v>33</v>
+      </c>
+      <c r="O26" t="n">
+        <v>21</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T26" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="U26" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V26" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="W26" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>31/05/2026 8:30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>6</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>24</v>
+      </c>
+      <c r="N27" t="n">
+        <v>37</v>
+      </c>
+      <c r="O27" t="n">
+        <v>38</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T27" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="U27" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V27" t="n">
+        <v>50</v>
+      </c>
+      <c r="W27" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X27" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Atletico Paranaense</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Mirassol</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>24</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Brazil Serie A+</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="W28" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="X28" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Gremio</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Corinthians</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E29" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="n">
+        <v>28</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Brazil Serie A+</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="W29" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="X29" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Vitoria</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>27</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Brazil Serie A+</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="n">
+        <v>63</v>
+      </c>
+      <c r="W30" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="X30" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>37</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F31" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="n">
+        <v>20</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="n">
+        <v>65</v>
+      </c>
+      <c r="W31" t="n">
+        <v>15</v>
+      </c>
+      <c r="X31" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="n">
+        <v>15</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="n">
+        <v>60</v>
+      </c>
+      <c r="W32" t="n">
+        <v>20</v>
+      </c>
+      <c r="X32" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="n">
+        <v>16</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="W33" t="n">
+        <v>25</v>
+      </c>
+      <c r="X33" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Universidad de Chile</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Concepción</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="n">
+        <v>13</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Chile Primera División+</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="W34" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="X34" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>00:30</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>America de Cali</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Macara</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Universidad de Concepcion</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Union La Calera</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="n">
+        <v>38</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Chile Primera División+</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="W35" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="X35" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Henan Jianye</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Hangzhou Greentown</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
         <v>1.7</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E36" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F36" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="n">
+        <v>27</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>China Super League+</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="W36" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="X36" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>37</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Chengdu Better City</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Shandong Luneng</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F37" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="n">
+        <v>22</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>China Super League+</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="W37" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="X37" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Qingdao Youth Island</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Shanghai Shenhua</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E38" t="n">
         <v>3.5</v>
       </c>
-      <c r="F22" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="F38" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="n">
+        <v>34</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>China Super League+</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="W38" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="X38" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sichuan Jiuniu</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Qingdao Jonoon</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E39" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F39" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="n">
+        <v>32</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>China Super League+</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="n">
+        <v>50</v>
+      </c>
+      <c r="W39" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="X39" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>25</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Vissel Kobe</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Kashima</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E40" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="n">
+        <v>34</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Japan J1 League+</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="W40" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="X40" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ODD Ballklubb</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E41" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="n">
+        <v>24</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="W41" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="X41" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>CF Os Belenenses</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Farense</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E42" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="n">
+        <v>41</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Portugal Segunda Liga+</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="W42" t="n">
+        <v>22</v>
+      </c>
+      <c r="X42" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>39</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Suwon City FC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Seongnam FC</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="n">
+        <v>36</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>South Korea South-Korea K League 2+</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="W43" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="X43" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Granada CF</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Sporting Gijon</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="n">
+        <v>34</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Spain Segunda División+</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="W44" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="X44" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="AA44" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Cultural Leonesa</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F45" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="n">
+        <v>41</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Spain Segunda División+</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="W45" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="X45" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SS Reyes</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>UD Logroñés</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F46" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="n">
+        <v>23</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Spain Segunda División RFEF - Play-offs+</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="W46" t="n">
+        <v>13</v>
+      </c>
+      <c r="X46" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Meyrin</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Chênois</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E47" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="n">
         <v>14</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>World CONMEBOL Sudamericana+</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Switzerland 1. Liga Classic - Group 1+</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t>❓</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="W47" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="X47" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Racing Montevideo</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Defensor Sporting</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F48" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="n">
+        <v>28</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Uruguay Primera División - Apertura+</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
         <is>
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="n">
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="n">
         <v>50</v>
       </c>
-      <c r="W22" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="X22" t="n">
-        <v>28.6</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>14</v>
+      <c r="W48" t="n">
+        <v>25</v>
+      </c>
+      <c r="X48" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>25</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 데이터 업데이트 - 2026-05-31 09:58
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA48"/>
+  <dimension ref="A1:AA43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,42 +556,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Busan I'Park</t>
+          <t>Tianjin Teda</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Paju Citizen</t>
+          <t>Dalian Zhixing</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.6</v>
+        <v>2.9</v>
       </c>
       <c r="E2" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="F2" t="n">
-        <v>4.6</v>
+        <v>2.4</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="I2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 2+</t>
+          <t>China Super League+</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -601,26 +601,26 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="N2" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="O2" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -629,68 +629,68 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T2" t="n">
-        <v>48</v>
+        <v>49.5</v>
       </c>
       <c r="U2" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V2" t="n">
-        <v>52.9</v>
+        <v>40</v>
       </c>
       <c r="W2" t="n">
-        <v>17.6</v>
+        <v>6.7</v>
       </c>
       <c r="X2" t="n">
-        <v>29.4</v>
+        <v>53.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>41.2</v>
+        <v>46.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>11.8</v>
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>01/06/2026 0:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Egersunds IK</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Lyn Oslo</t>
+          <t>Stromsgodset IF</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.7</v>
+        <v>2.8</v>
       </c>
       <c r="E3" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="F3" t="n">
-        <v>4.2</v>
+        <v>2.1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="I3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -704,26 +704,26 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="N3" t="n">
         <v>33</v>
       </c>
       <c r="O3" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -732,72 +732,72 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>57.7</v>
+        <v>8</v>
       </c>
       <c r="T3" t="n">
-        <v>48.5</v>
+        <v>51.8</v>
       </c>
       <c r="U3" t="n">
-        <v>35.3</v>
+        <v>1.9</v>
       </c>
       <c r="V3" t="n">
-        <v>50</v>
+        <v>30.8</v>
       </c>
       <c r="W3" t="n">
-        <v>21.4</v>
+        <v>23.1</v>
       </c>
       <c r="X3" t="n">
-        <v>28.6</v>
+        <v>46.2</v>
       </c>
       <c r="Y3" t="n">
-        <v>35.7</v>
+        <v>38.5</v>
       </c>
       <c r="Z3" t="n">
-        <v>14.3</v>
+        <v>15.4</v>
       </c>
       <c r="AA3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>01/06/2026 8:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Real Sociedad B</t>
+          <t>Remo PA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cultural Leonesa</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E4" t="n">
         <v>3.2</v>
       </c>
       <c r="F4" t="n">
-        <v>3.1</v>
+        <v>2.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I4" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Spain Segunda División+</t>
+          <t>Brazil Serie A+</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -807,26 +807,26 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="N4" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="O4" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -835,57 +835,57 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>32.3</v>
+        <v>8</v>
       </c>
       <c r="T4" t="n">
-        <v>44.7</v>
+        <v>51.8</v>
       </c>
       <c r="U4" t="n">
-        <v>14.3</v>
+        <v>1.9</v>
       </c>
       <c r="V4" t="n">
-        <v>45.5</v>
+        <v>29.4</v>
       </c>
       <c r="W4" t="n">
-        <v>18.2</v>
+        <v>23.5</v>
       </c>
       <c r="X4" t="n">
-        <v>36.4</v>
+        <v>47.1</v>
       </c>
       <c r="Y4" t="n">
-        <v>18.2</v>
+        <v>41.2</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="AA4" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>31/05/2026 4:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Hwaseong FC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sporting Gijón</t>
+          <t>Gyeongnam</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="E5" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -893,19 +893,19 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I5" t="n">
         <v>10</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Spain Segunda División+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -914,17 +914,17 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N5" t="n">
+        <v>33</v>
+      </c>
+      <c r="O5" t="n">
         <v>29</v>
       </c>
-      <c r="O5" t="n">
-        <v>31</v>
-      </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -938,28 +938,28 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>57.7</v>
+        <v>32.3</v>
       </c>
       <c r="T5" t="n">
-        <v>48.5</v>
+        <v>44.4</v>
       </c>
       <c r="U5" t="n">
-        <v>35.3</v>
+        <v>14.3</v>
       </c>
       <c r="V5" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="W5" t="n">
+        <v>40</v>
+      </c>
+      <c r="X5" t="n">
         <v>20</v>
       </c>
-      <c r="X5" t="n">
-        <v>30</v>
-      </c>
       <c r="Y5" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="Z5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA5" t="n">
         <v>10</v>
@@ -968,42 +968,42 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Vegalta Sendai</t>
+          <t>RB Bragantino</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ventforet Kofu</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E6" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="F6" t="n">
-        <v>4.5</v>
+        <v>3.3</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>무승부</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Japan J2/J3 League+</t>
+          <t>Brazil Serie A+</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1017,22 +1017,22 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N6" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="O6" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1044,69 +1044,69 @@
         <v>32.3</v>
       </c>
       <c r="T6" t="n">
-        <v>44.7</v>
+        <v>44.4</v>
       </c>
       <c r="U6" t="n">
         <v>14.3</v>
       </c>
       <c r="V6" t="n">
-        <v>38.5</v>
+        <v>43.8</v>
       </c>
       <c r="W6" t="n">
-        <v>30.8</v>
+        <v>25</v>
       </c>
       <c r="X6" t="n">
-        <v>30.8</v>
+        <v>31.2</v>
       </c>
       <c r="Y6" t="n">
-        <v>15.4</v>
+        <v>25</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>01/06/2026 1:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kataller Toyama</t>
+          <t>Deportivo La Coruña</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tegevajaro Miyazaki</t>
+          <t>Las Palmas</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2.4</v>
+        <v>3.4</v>
       </c>
       <c r="E7" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="F7" t="n">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>무승부</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="I7" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Japan J2/J3 League+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1116,26 +1116,26 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="N7" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O7" t="n">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>2:2</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1144,72 +1144,72 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>57.7</v>
+        <v>76.2</v>
       </c>
       <c r="T7" t="n">
-        <v>48.5</v>
+        <v>51.9</v>
       </c>
       <c r="U7" t="n">
-        <v>35.3</v>
+        <v>56.7</v>
       </c>
       <c r="V7" t="n">
+        <v>20</v>
+      </c>
+      <c r="W7" t="n">
         <v>40</v>
-      </c>
-      <c r="W7" t="n">
-        <v>20</v>
       </c>
       <c r="X7" t="n">
         <v>40</v>
       </c>
       <c r="Y7" t="n">
-        <v>46.7</v>
+        <v>30</v>
       </c>
       <c r="Z7" t="n">
-        <v>13.3</v>
+        <v>30</v>
       </c>
       <c r="AA7" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>01/06/2026 1:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Qingdao West Coast</t>
+          <t>Gent</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Shanghai Shenhua</t>
+          <t>Racing Genk</t>
         </is>
       </c>
       <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F8" t="n">
         <v>2.2</v>
       </c>
-      <c r="E8" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2.9</v>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>무승부</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>China Super League+</t>
+          <t>Belgium Jupiler Pro League+</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1219,26 +1219,26 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>30</v>
       </c>
       <c r="N8" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="O8" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1247,72 +1247,72 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="T8" t="n">
-        <v>48</v>
+        <v>51.8</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="V8" t="n">
-        <v>28.6</v>
+        <v>40</v>
       </c>
       <c r="W8" t="n">
-        <v>35.7</v>
+        <v>20</v>
       </c>
       <c r="X8" t="n">
-        <v>35.7</v>
+        <v>40</v>
       </c>
       <c r="Y8" t="n">
-        <v>21.4</v>
+        <v>33.3</v>
       </c>
       <c r="Z8" t="n">
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="AA8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>31/05/2026 5:30</t>
+          <t>01/06/2026 1:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Limache</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Botafogo</t>
+          <t>Coquimbo Unido</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="E9" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="F9" t="n">
-        <v>3.9</v>
+        <v>2.5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>무승부</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="I9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>Chile Primera División+</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1322,101 +1322,105 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="N9" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="O9" t="n">
+        <v>33</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>3:2</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="T9" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="U9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="V9" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="W9" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X9" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y9" t="n">
         <v>25</v>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S9" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="T9" t="n">
-        <v>44.7</v>
-      </c>
-      <c r="U9" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="V9" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="W9" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="X9" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>18.2</v>
-      </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AA9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>30/05/2026 9:00</t>
+          <t>01/06/2026 3:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Juventud LP</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>América Mineiro</t>
+          <t>Montevideo Wanderers</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="E10" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="F10" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
+        <v>3.2</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>Uruguay Primera División - Apertura+</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1425,22 +1429,22 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="N10" t="n">
+        <v>28</v>
+      </c>
+      <c r="O10" t="n">
         <v>37</v>
       </c>
-      <c r="O10" t="n">
-        <v>15</v>
-      </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1449,64 +1453,68 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>8</v>
+        <v>32.3</v>
       </c>
       <c r="T10" t="n">
-        <v>48</v>
+        <v>44.4</v>
       </c>
       <c r="U10" t="n">
-        <v>1.9</v>
+        <v>14.3</v>
       </c>
       <c r="V10" t="n">
-        <v>50</v>
+        <v>56.2</v>
       </c>
       <c r="W10" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="X10" t="n">
-        <v>0</v>
+        <v>18.8</v>
       </c>
       <c r="Y10" t="n">
-        <v>0</v>
+        <v>37.5</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="AA10" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>30/05/2026 9:30</t>
+          <t>01/06/2026 6:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Univ de Concepcion</t>
+          <t>O Higgins</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Unión La Calera</t>
+          <t>Everton de Vina</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="E11" t="n">
         <v>3.4</v>
       </c>
       <c r="F11" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
+        <v>3.9</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>무승부</t>
+        </is>
+      </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I11" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1515,7 +1523,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1524,22 +1532,22 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="N11" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="O11" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1548,92 +1556,96 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>57.7</v>
+        <v>32.3</v>
       </c>
       <c r="T11" t="n">
-        <v>48.5</v>
+        <v>44.4</v>
       </c>
       <c r="U11" t="n">
-        <v>35.3</v>
+        <v>14.3</v>
       </c>
       <c r="V11" t="n">
-        <v>40</v>
+        <v>36.8</v>
       </c>
       <c r="W11" t="n">
-        <v>20</v>
+        <v>21.1</v>
       </c>
       <c r="X11" t="n">
-        <v>40</v>
+        <v>42.1</v>
       </c>
       <c r="Y11" t="n">
-        <v>40</v>
+        <v>26.3</v>
       </c>
       <c r="Z11" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>01/06/2026 8:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yongin City</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Daegu FC</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3.9</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F12" t="n">
         <v>3.6</v>
       </c>
-      <c r="F12" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I12" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 2+</t>
+          <t>Brazil Serie A+</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="N12" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O12" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1647,31 +1659,31 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T12" t="n">
-        <v>48</v>
+        <v>49.5</v>
       </c>
       <c r="U12" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V12" t="n">
-        <v>14.3</v>
+        <v>42.9</v>
       </c>
       <c r="W12" t="n">
-        <v>42.9</v>
+        <v>28.6</v>
       </c>
       <c r="X12" t="n">
-        <v>42.9</v>
+        <v>28.6</v>
       </c>
       <c r="Y12" t="n">
-        <v>14.3</v>
+        <v>19</v>
       </c>
       <c r="Z12" t="n">
         <v>0</v>
       </c>
       <c r="AA12" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
@@ -1682,29 +1694,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Asan Mugunghwa</t>
+          <t>Jeonnam Dragons</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Suwon Bluewings</t>
+          <t>Seoul E-Land</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="E13" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="F13" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1722,13 +1734,13 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N13" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O13" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -1749,28 +1761,28 @@
         <v>57.7</v>
       </c>
       <c r="T13" t="n">
-        <v>48.5</v>
+        <v>49.5</v>
       </c>
       <c r="U13" t="n">
         <v>35.3</v>
       </c>
       <c r="V13" t="n">
-        <v>40</v>
+        <v>66.7</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>60</v>
+        <v>33.3</v>
       </c>
       <c r="Y13" t="n">
-        <v>60</v>
+        <v>33.3</v>
       </c>
       <c r="Z13" t="n">
         <v>0</v>
       </c>
       <c r="AA13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1781,29 +1793,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Suwon FC</t>
+          <t>Ansan Greeners</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Seongnam FC</t>
+          <t>Cheonan City</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2.1</v>
+        <v>3.5</v>
       </c>
       <c r="E14" t="n">
         <v>3.3</v>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>1.9</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1817,59 +1829,59 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="N14" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="O14" t="n">
+        <v>32</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T14" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="U14" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="X14" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="Y14" t="n">
         <v>25</v>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S14" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="T14" t="n">
-        <v>50</v>
-      </c>
-      <c r="U14" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="V14" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="W14" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="X14" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>33.3</v>
-      </c>
       <c r="Z14" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="AA14" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1880,33 +1892,33 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Gimhae City</t>
+          <t>Poblense</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GimPo Citizen</t>
+          <t>CD Águilas</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4.7</v>
+        <v>2.5</v>
       </c>
       <c r="E15" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="F15" t="n">
-        <v>1.6</v>
+        <v>3</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 2+</t>
+          <t>Spain Segunda División RFEF - Play-offs+</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1916,21 +1928,21 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N15" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="O15" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1944,68 +1956,68 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>57.7</v>
+        <v>8</v>
       </c>
       <c r="T15" t="n">
-        <v>48.5</v>
+        <v>51.8</v>
       </c>
       <c r="U15" t="n">
-        <v>35.3</v>
+        <v>1.9</v>
       </c>
       <c r="V15" t="n">
-        <v>11.1</v>
+        <v>0</v>
       </c>
       <c r="W15" t="n">
-        <v>11.1</v>
+        <v>66.7</v>
       </c>
       <c r="X15" t="n">
-        <v>77.8</v>
+        <v>33.3</v>
       </c>
       <c r="Y15" t="n">
-        <v>66.7</v>
+        <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Chengdu Qianbao</t>
+          <t>Real Oviedo B</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Shandong Luneng</t>
+          <t>CD Coria</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E16" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="F16" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>China Super League+</t>
+          <t>Spain Segunda División RFEF - Play-offs+</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2019,22 +2031,22 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="N16" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="O16" t="n">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2043,57 +2055,47 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>57.7</v>
+        <v>32.3</v>
       </c>
       <c r="T16" t="n">
-        <v>48.5</v>
+        <v>44.4</v>
       </c>
       <c r="U16" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="V16" t="n">
-        <v>50</v>
-      </c>
-      <c r="W16" t="n">
-        <v>50</v>
-      </c>
-      <c r="X16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>25</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>0</v>
-      </c>
+        <v>14.3</v>
+      </c>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chongqing Tongliang</t>
+          <t>Wuhan Three Towns</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Beijing Guoan</t>
+          <t>Yunnan Yukun</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.9</v>
+        <v>2.8</v>
       </c>
       <c r="E17" t="n">
         <v>3.5</v>
       </c>
       <c r="F17" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
@@ -2118,22 +2120,22 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="N17" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="O17" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2142,25 +2144,25 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T17" t="n">
-        <v>48</v>
+        <v>49.5</v>
       </c>
       <c r="U17" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V17" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="n">
         <v>40</v>
-      </c>
-      <c r="X17" t="n">
-        <v>40</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>0</v>
       </c>
       <c r="Z17" t="n">
         <v>0</v>
@@ -2172,38 +2174,38 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sichuan FC</t>
+          <t>Albion FC (URU)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Qingdao Jonoon</t>
+          <t>CA Torque</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="E18" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>China Super League+</t>
+          <t>Uruguay Primera División - Apertura+</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2213,17 +2215,17 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="N18" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="O18" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
@@ -2244,65 +2246,65 @@
         <v>57.7</v>
       </c>
       <c r="T18" t="n">
-        <v>48.5</v>
+        <v>49.5</v>
       </c>
       <c r="U18" t="n">
         <v>35.3</v>
       </c>
       <c r="V18" t="n">
-        <v>37.5</v>
+        <v>42.9</v>
       </c>
       <c r="W18" t="n">
-        <v>25</v>
+        <v>28.6</v>
       </c>
       <c r="X18" t="n">
-        <v>37.5</v>
+        <v>28.6</v>
       </c>
       <c r="Y18" t="n">
-        <v>0</v>
+        <v>42.9</v>
       </c>
       <c r="Z18" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="AA18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Racing Club (URU)</t>
+          <t>São Bernardo SP</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Defensor Sporting</t>
+          <t>Novorizontino SP</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.9</v>
+        <v>2.8</v>
       </c>
       <c r="E19" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="F19" t="n">
-        <v>3.9</v>
+        <v>2.8</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Uruguay Primera División - Apertura+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2312,26 +2314,26 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="N19" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="O19" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2340,31 +2342,31 @@
         </is>
       </c>
       <c r="S19" t="n">
-        <v>57.7</v>
+        <v>32.3</v>
       </c>
       <c r="T19" t="n">
-        <v>48.5</v>
+        <v>44.4</v>
       </c>
       <c r="U19" t="n">
-        <v>35.3</v>
+        <v>14.3</v>
       </c>
       <c r="V19" t="n">
-        <v>83.3</v>
+        <v>20</v>
       </c>
       <c r="W19" t="n">
-        <v>16.7</v>
+        <v>40</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="Y19" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="Z19" t="n">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="AA19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -2375,33 +2377,33 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Molde</t>
+          <t>Londrina</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sandefjord</t>
+          <t>Vila Nova FC</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="E20" t="n">
-        <v>4.3</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>4.8</v>
+        <v>3</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2415,22 +2417,22 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="N20" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="O20" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2439,57 +2441,57 @@
         </is>
       </c>
       <c r="S20" t="n">
-        <v>76.2</v>
+        <v>32.3</v>
       </c>
       <c r="T20" t="n">
-        <v>50</v>
+        <v>44.4</v>
       </c>
       <c r="U20" t="n">
-        <v>56.7</v>
+        <v>14.3</v>
       </c>
       <c r="V20" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="W20" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="X20" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="Y20" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="Z20" t="n">
         <v>0</v>
       </c>
       <c r="AA20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>01/06/2026 0:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Moss FK</t>
+          <t>Strommen IF</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="E21" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="F21" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
@@ -2514,13 +2516,13 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="N21" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="O21" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
@@ -2541,7 +2543,7 @@
         <v>76.2</v>
       </c>
       <c r="T21" t="n">
-        <v>50</v>
+        <v>51.9</v>
       </c>
       <c r="U21" t="n">
         <v>56.7</v>
@@ -2550,16 +2552,16 @@
         <v>37.5</v>
       </c>
       <c r="W21" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="X21" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>25</v>
+      </c>
+      <c r="Z21" t="n">
         <v>12.5</v>
-      </c>
-      <c r="X21" t="n">
-        <v>50</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>0</v>
       </c>
       <c r="AA21" t="n">
         <v>8</v>
@@ -2568,38 +2570,38 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>01/06/2026 0:00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>AD Ceuta</t>
+          <t>Bryne FK</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Albacete Balompie</t>
+          <t>IL Hodd</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="E22" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="F22" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Spain Segunda División+</t>
+          <t>Norway 1. Division+</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2613,22 +2615,22 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="N22" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="O22" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2637,68 +2639,68 @@
         </is>
       </c>
       <c r="S22" t="n">
-        <v>32.3</v>
+        <v>57.7</v>
       </c>
       <c r="T22" t="n">
-        <v>44.7</v>
+        <v>49.5</v>
       </c>
       <c r="U22" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V22" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0</v>
+      </c>
+      <c r="X22" t="n">
         <v>14.3</v>
       </c>
-      <c r="V22" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="W22" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="X22" t="n">
-        <v>25</v>
-      </c>
       <c r="Y22" t="n">
-        <v>37.5</v>
+        <v>57.1</v>
       </c>
       <c r="Z22" t="n">
         <v>0</v>
       </c>
       <c r="AA22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>31/05/2026 3:00</t>
+          <t>01/06/2026 0:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Danubio FC</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CA Progreso</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="E23" t="n">
-        <v>3.2</v>
+        <v>5.7</v>
       </c>
       <c r="F23" t="n">
-        <v>3.7</v>
+        <v>7.5</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Uruguay Primera División - Apertura+</t>
+          <t>Norway 1. Division+</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2712,17 +2714,17 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="N23" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="O23" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>3:0</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2736,13 +2738,13 @@
         </is>
       </c>
       <c r="S23" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T23" t="n">
-        <v>48</v>
+        <v>49.5</v>
       </c>
       <c r="U23" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V23" t="n">
         <v>100</v>
@@ -2754,50 +2756,50 @@
         <v>0</v>
       </c>
       <c r="Y23" t="n">
-        <v>33.3</v>
+        <v>100</v>
       </c>
       <c r="Z23" t="n">
-        <v>33.3</v>
+        <v>100</v>
       </c>
       <c r="AA23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>31/05/2026 4:00</t>
+          <t>01/06/2026 0:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Raufoss IL</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.4</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>4.9</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>7.2</v>
+        <v>1.7</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>Norway 1. Division+</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2807,26 +2809,26 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M24" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="N24" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="O24" t="n">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>2:3</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2835,68 +2837,68 @@
         </is>
       </c>
       <c r="S24" t="n">
-        <v>76.2</v>
+        <v>87.5</v>
       </c>
       <c r="T24" t="n">
-        <v>50</v>
+        <v>61.5</v>
       </c>
       <c r="U24" t="n">
-        <v>56.7</v>
+        <v>73.5</v>
       </c>
       <c r="V24" t="n">
-        <v>60</v>
+        <v>57.1</v>
       </c>
       <c r="W24" t="n">
-        <v>40</v>
+        <v>14.3</v>
       </c>
       <c r="X24" t="n">
-        <v>0</v>
+        <v>28.6</v>
       </c>
       <c r="Y24" t="n">
-        <v>20</v>
+        <v>57.1</v>
       </c>
       <c r="Z24" t="n">
         <v>0</v>
       </c>
       <c r="AA24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>31/05/2026 4:00</t>
+          <t>01/06/2026 0:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>La Serena</t>
+          <t>Ranheim Fotball</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Colo Colo</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="D25" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E25" t="n">
         <v>4</v>
       </c>
-      <c r="E25" t="n">
-        <v>3.4</v>
-      </c>
       <c r="F25" t="n">
-        <v>1.9</v>
+        <v>3.7</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Chile Primera División+</t>
+          <t>Norway 1. Division+</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2906,26 +2908,26 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="N25" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="O25" t="n">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2934,58 +2936,68 @@
         </is>
       </c>
       <c r="S25" t="n">
-        <v>57.7</v>
+        <v>76.2</v>
       </c>
       <c r="T25" t="n">
-        <v>48.5</v>
+        <v>51.9</v>
       </c>
       <c r="U25" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
+        <v>56.7</v>
+      </c>
+      <c r="V25" t="n">
+        <v>25</v>
+      </c>
+      <c r="W25" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="X25" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>12.5</v>
+      </c>
       <c r="AA25" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>31/05/2026 6:30</t>
+          <t>01/06/2026 1:30</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Univ de Chile</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Deportes Concepción</t>
+          <t>Cadiz</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="F26" t="n">
-        <v>6.2</v>
+        <v>8.6</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Chile Primera División+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2999,17 +3011,17 @@
         </is>
       </c>
       <c r="M26" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="N26" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="O26" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -3023,19 +3035,19 @@
         </is>
       </c>
       <c r="S26" t="n">
-        <v>32.3</v>
+        <v>57.7</v>
       </c>
       <c r="T26" t="n">
-        <v>44.7</v>
+        <v>49.5</v>
       </c>
       <c r="U26" t="n">
-        <v>14.3</v>
+        <v>35.3</v>
       </c>
       <c r="V26" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="W26" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="X26" t="n">
         <v>0</v>
@@ -3047,44 +3059,44 @@
         <v>0</v>
       </c>
       <c r="AA26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>31/05/2026 8:30</t>
+          <t>01/06/2026 2:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>Atlético Baleares</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>Real Jaén</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="E27" t="n">
         <v>2.9</v>
       </c>
       <c r="F27" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>Spain Segunda División RFEF - Play-offs+</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -3098,17 +3110,17 @@
         </is>
       </c>
       <c r="M27" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N27" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="O27" t="n">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -3122,22 +3134,22 @@
         </is>
       </c>
       <c r="S27" t="n">
-        <v>57.7</v>
+        <v>32.3</v>
       </c>
       <c r="T27" t="n">
-        <v>48.5</v>
+        <v>44.4</v>
       </c>
       <c r="U27" t="n">
-        <v>35.3</v>
+        <v>14.3</v>
       </c>
       <c r="V27" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="W27" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="X27" t="n">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="Y27" t="n">
         <v>0</v>
@@ -3146,46 +3158,44 @@
         <v>0</v>
       </c>
       <c r="AA27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>01/06/2026 2:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Atletico Paranaense</t>
+          <t>UB Conquense</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>CD Ourense</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
       <c r="E28" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="F28" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+        <v>3.1</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
       <c r="I28" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>Spain Segunda División RFEF - Play-offs+</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -3198,17 +3208,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>10</v>
+      </c>
+      <c r="N28" t="n">
+        <v>50</v>
+      </c>
+      <c r="O28" t="n">
+        <v>40</v>
+      </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -3216,61 +3232,55 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="W28" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="X28" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="Y28" t="n">
-        <v>41.7</v>
-      </c>
-      <c r="Z28" t="n">
-        <v>16.7</v>
-      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>01/06/2026 4:00</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gremio</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Chapecoense SC</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>5.8</v>
       </c>
       <c r="F29" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+        <v>11.8</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
       <c r="I29" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -3287,17 +3297,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>72</v>
+      </c>
+      <c r="N29" t="n">
+        <v>19</v>
+      </c>
+      <c r="O29" t="n">
+        <v>9</v>
+      </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -3305,65 +3321,59 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="W29" t="n">
+      <c r="S29" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T29" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="U29" t="n">
         <v>14.3</v>
       </c>
-      <c r="X29" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="Y29" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>10.7</v>
-      </c>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>01/06/2026 8:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Vitoria</t>
+          <t>CRB AL</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="E30" t="n">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
       <c r="F30" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
       <c r="I30" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -3376,17 +3386,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>23</v>
+      </c>
+      <c r="N30" t="n">
+        <v>36</v>
+      </c>
+      <c r="O30" t="n">
+        <v>41</v>
+      </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3394,52 +3410,58 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
+      <c r="S30" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T30" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="U30" t="n">
+        <v>14.3</v>
+      </c>
       <c r="V30" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="W30" t="n">
-        <v>14.8</v>
+        <v>33.3</v>
       </c>
       <c r="X30" t="n">
-        <v>22.2</v>
+        <v>16.7</v>
       </c>
       <c r="Y30" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="Z30" t="n">
-        <v>14.8</v>
+        <v>0</v>
       </c>
       <c r="AA30" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Remo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Sao Paulo</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="E31" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="F31" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -3448,11 +3470,11 @@
       </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>Brazil Serie A+</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3462,7 +3484,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
@@ -3487,22 +3509,22 @@
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="W31" t="n">
-        <v>15</v>
+        <v>15.6</v>
       </c>
       <c r="X31" t="n">
-        <v>20</v>
+        <v>34.4</v>
       </c>
       <c r="Y31" t="n">
-        <v>20</v>
+        <v>37.5</v>
       </c>
       <c r="Z31" t="n">
-        <v>5</v>
+        <v>12.5</v>
       </c>
       <c r="AA31" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32">
@@ -3513,22 +3535,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Vasco DA Gama</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>Atletico-MG</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
       <c r="F32" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -3537,11 +3559,11 @@
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>Brazil Serie A+</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3576,48 +3598,48 @@
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="W32" t="n">
-        <v>20</v>
+        <v>19.4</v>
       </c>
       <c r="X32" t="n">
-        <v>20</v>
+        <v>30.6</v>
       </c>
       <c r="Y32" t="n">
-        <v>26.7</v>
+        <v>30.6</v>
       </c>
       <c r="Z32" t="n">
-        <v>6.7</v>
+        <v>5.6</v>
       </c>
       <c r="AA32" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Operario-PR</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>1.9</v>
       </c>
       <c r="E33" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="F33" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -3626,7 +3648,7 @@
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -3665,48 +3687,48 @@
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="n">
-        <v>56.2</v>
+        <v>46.2</v>
       </c>
       <c r="W33" t="n">
-        <v>25</v>
+        <v>23.1</v>
       </c>
       <c r="X33" t="n">
-        <v>18.8</v>
+        <v>30.8</v>
       </c>
       <c r="Y33" t="n">
-        <v>31.2</v>
+        <v>30.8</v>
       </c>
       <c r="Z33" t="n">
-        <v>12.5</v>
+        <v>3.8</v>
       </c>
       <c r="AA33" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>Huachipato</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Concepción</t>
+          <t>U. Catolica</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="F34" t="n">
-        <v>6.2</v>
+        <v>2.2</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -3715,7 +3737,7 @@
       </c>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -3729,7 +3751,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M34" t="inlineStr"/>
@@ -3754,48 +3776,48 @@
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="n">
-        <v>61.5</v>
+        <v>51.7</v>
       </c>
       <c r="W34" t="n">
-        <v>23.1</v>
+        <v>13.8</v>
       </c>
       <c r="X34" t="n">
-        <v>15.4</v>
+        <v>34.5</v>
       </c>
       <c r="Y34" t="n">
-        <v>30.8</v>
+        <v>31</v>
       </c>
       <c r="Z34" t="n">
-        <v>15.4</v>
+        <v>3.4</v>
       </c>
       <c r="AA34" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Universidad de Concepcion</t>
+          <t>Zaragoza</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Union La Calera</t>
+          <t>Malaga</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>2.3</v>
+        <v>4.3</v>
       </c>
       <c r="E35" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="F35" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -3804,11 +3826,11 @@
       </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Chile Primera División+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3818,7 +3840,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
@@ -3843,48 +3865,48 @@
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="n">
-        <v>44.7</v>
+        <v>46.2</v>
       </c>
       <c r="W35" t="n">
-        <v>18.4</v>
+        <v>23.1</v>
       </c>
       <c r="X35" t="n">
-        <v>36.8</v>
+        <v>30.8</v>
       </c>
       <c r="Y35" t="n">
-        <v>44.7</v>
+        <v>30.8</v>
       </c>
       <c r="Z35" t="n">
-        <v>10.5</v>
+        <v>15.4</v>
       </c>
       <c r="AA35" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Henan Jianye</t>
+          <t>Cordoba</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hangzhou Greentown</t>
+          <t>Huesca</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E36" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="F36" t="n">
-        <v>4.3</v>
+        <v>5.7</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -3893,11 +3915,11 @@
       </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>China Super League+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3932,48 +3954,48 @@
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="n">
-        <v>59.3</v>
+        <v>54.5</v>
       </c>
       <c r="W36" t="n">
-        <v>14.8</v>
+        <v>27.3</v>
       </c>
       <c r="X36" t="n">
-        <v>25.9</v>
+        <v>18.2</v>
       </c>
       <c r="Y36" t="n">
-        <v>37</v>
+        <v>27.3</v>
       </c>
       <c r="Z36" t="n">
-        <v>11.1</v>
+        <v>9.1</v>
       </c>
       <c r="AA36" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Chengdu Better City</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Shandong Luneng</t>
+          <t>Valladolid</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E37" t="n">
-        <v>3.8</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
-        <v>3.1</v>
+        <v>7.7</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -3982,11 +4004,11 @@
       </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>China Super League+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -4021,48 +4043,48 @@
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="n">
-        <v>45.5</v>
+        <v>53.8</v>
       </c>
       <c r="W37" t="n">
-        <v>27.3</v>
+        <v>23.1</v>
       </c>
       <c r="X37" t="n">
-        <v>27.3</v>
+        <v>23.1</v>
       </c>
       <c r="Y37" t="n">
-        <v>31.8</v>
+        <v>30.8</v>
       </c>
       <c r="Z37" t="n">
-        <v>4.5</v>
+        <v>7.7</v>
       </c>
       <c r="AA37" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Qingdao Youth Island</t>
+          <t>Castellón</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Shanghai Shenhua</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="E38" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F38" t="n">
-        <v>2.9</v>
+        <v>5.1</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -4071,11 +4093,11 @@
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>China Super League+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -4110,61 +4132,61 @@
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="n">
-        <v>38.2</v>
+        <v>44.4</v>
       </c>
       <c r="W38" t="n">
-        <v>26.5</v>
+        <v>27.8</v>
       </c>
       <c r="X38" t="n">
-        <v>35.3</v>
+        <v>27.8</v>
       </c>
       <c r="Y38" t="n">
-        <v>35.3</v>
+        <v>38.9</v>
       </c>
       <c r="Z38" t="n">
-        <v>8.800000000000001</v>
+        <v>16.7</v>
       </c>
       <c r="AA38" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sichuan Jiuniu</t>
+          <t>Deportivo La Coruna</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Qingdao Jonoon</t>
+          <t>Las Palmas</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1.9</v>
+        <v>3.4</v>
       </c>
       <c r="E39" t="n">
         <v>3.5</v>
       </c>
       <c r="F39" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>China Super League+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -4174,7 +4196,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -4199,48 +4221,48 @@
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="W39" t="n">
-        <v>18.8</v>
+        <v>18.5</v>
       </c>
       <c r="X39" t="n">
-        <v>31.2</v>
+        <v>44.4</v>
       </c>
       <c r="Y39" t="n">
-        <v>25</v>
+        <v>48.1</v>
       </c>
       <c r="Z39" t="n">
-        <v>3.1</v>
+        <v>18.5</v>
       </c>
       <c r="AA39" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vissel Kobe</t>
+          <t>Leganes</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Kashima</t>
+          <t>Mirandes</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="F40" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -4249,11 +4271,11 @@
       </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Japan J1 League+</t>
+          <t>Spain Segunda División+</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -4288,48 +4310,48 @@
       <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="n">
-        <v>58.8</v>
+        <v>46.7</v>
       </c>
       <c r="W40" t="n">
-        <v>14.7</v>
+        <v>23.3</v>
       </c>
       <c r="X40" t="n">
-        <v>26.5</v>
+        <v>30</v>
       </c>
       <c r="Y40" t="n">
-        <v>29.4</v>
+        <v>30</v>
       </c>
       <c r="Z40" t="n">
-        <v>2.9</v>
+        <v>6.7</v>
       </c>
       <c r="AA40" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ODD Ballklubb</t>
+          <t>Conquense</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>UD Ourense</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="E41" t="n">
-        <v>4.1</v>
+        <v>2.8</v>
       </c>
       <c r="F41" t="n">
-        <v>4.2</v>
+        <v>3.1</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -4338,11 +4360,11 @@
       </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Norway 1. Division+</t>
+          <t>Spain Segunda División RFEF - Play-offs+</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -4377,48 +4399,48 @@
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="n">
-        <v>58.3</v>
+        <v>58.8</v>
       </c>
       <c r="W41" t="n">
-        <v>16.7</v>
+        <v>23.5</v>
       </c>
       <c r="X41" t="n">
-        <v>25</v>
+        <v>17.6</v>
       </c>
       <c r="Y41" t="n">
-        <v>37.5</v>
+        <v>17.6</v>
       </c>
       <c r="Z41" t="n">
-        <v>12.5</v>
+        <v>5.9</v>
       </c>
       <c r="AA41" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CF Os Belenenses</t>
+          <t>Real Oviedo II</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Farense</t>
+          <t>CD Coria</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="E42" t="n">
         <v>3.2</v>
       </c>
       <c r="F42" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -4427,11 +4449,11 @@
       </c>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Portugal Segunda Liga+</t>
+          <t>Spain Segunda División RFEF - Play-offs+</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -4441,7 +4463,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M42" t="inlineStr"/>
@@ -4466,48 +4488,48 @@
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="n">
-        <v>43.9</v>
+        <v>53.8</v>
       </c>
       <c r="W42" t="n">
-        <v>22</v>
+        <v>23.1</v>
       </c>
       <c r="X42" t="n">
-        <v>34.1</v>
+        <v>23.1</v>
       </c>
       <c r="Y42" t="n">
-        <v>39</v>
+        <v>23.1</v>
       </c>
       <c r="Z42" t="n">
-        <v>14.6</v>
+        <v>3.8</v>
       </c>
       <c r="AA42" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Suwon City FC</t>
+          <t>Albion FC</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Seongnam FC</t>
+          <t>Atletico Torque</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="E43" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -4516,11 +4538,11 @@
       </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 2+</t>
+          <t>Uruguay Primera División - Apertura+</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -4530,7 +4552,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M43" t="inlineStr"/>
@@ -4555,467 +4577,22 @@
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="n">
-        <v>47.2</v>
+        <v>55.6</v>
       </c>
       <c r="W43" t="n">
-        <v>22.2</v>
+        <v>11.1</v>
       </c>
       <c r="X43" t="n">
-        <v>30.6</v>
+        <v>33.3</v>
       </c>
       <c r="Y43" t="n">
-        <v>38.9</v>
+        <v>40.7</v>
       </c>
       <c r="Z43" t="n">
-        <v>8.300000000000001</v>
+        <v>14.8</v>
       </c>
       <c r="AA43" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Granada CF</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Sporting Gijon</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="E44" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F44" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="n">
-        <v>34</v>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Spain Segunda División+</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr"/>
-      <c r="T44" t="inlineStr"/>
-      <c r="U44" t="inlineStr"/>
-      <c r="V44" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="W44" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="X44" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="Y44" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="Z44" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="AA44" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>14:15</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Real Sociedad II</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Cultural Leonesa</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="E45" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F45" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="n">
-        <v>41</v>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Spain Segunda División+</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
-      <c r="U45" t="inlineStr"/>
-      <c r="V45" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="W45" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="X45" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="Y45" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="Z45" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="AA45" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>SS Reyes</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>UD Logroñés</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E46" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="F46" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="n">
-        <v>23</v>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>Spain Segunda División RFEF - Play-offs+</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr"/>
-      <c r="T46" t="inlineStr"/>
-      <c r="U46" t="inlineStr"/>
-      <c r="V46" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="W46" t="n">
-        <v>13</v>
-      </c>
-      <c r="X46" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="Y46" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="Z46" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="AA46" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Meyrin</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Chênois</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="E47" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="F47" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="n">
-        <v>14</v>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>Switzerland 1. Liga Classic - Group 1+</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr"/>
-      <c r="U47" t="inlineStr"/>
-      <c r="V47" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="W47" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="X47" t="n">
-        <v>35.7</v>
-      </c>
-      <c r="Y47" t="n">
-        <v>35.7</v>
-      </c>
-      <c r="Z47" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="AA47" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Racing Montevideo</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Defensor Sporting</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="E48" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F48" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="n">
-        <v>28</v>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>Uruguay Primera División - Apertura+</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr"/>
-      <c r="U48" t="inlineStr"/>
-      <c r="V48" t="n">
-        <v>50</v>
-      </c>
-      <c r="W48" t="n">
-        <v>25</v>
-      </c>
-      <c r="X48" t="n">
-        <v>25</v>
-      </c>
-      <c r="Y48" t="n">
-        <v>25</v>
-      </c>
-      <c r="Z48" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="AA48" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-03 11:25
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,42 +556,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>02/06/2026 3:00</t>
+          <t>03/06/2026 9:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Boston River</t>
+          <t>Junior Barranquilla</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Liverpool (URU)</t>
+          <t>Atlético Nacional</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="E2" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="F2" t="n">
-        <v>2.2</v>
+        <v>2.7</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="I2" t="n">
         <v>11</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Uruguay Primera División - Apertura+</t>
+          <t>Colombia Primera A+</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -605,22 +605,22 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="N2" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -629,25 +629,25 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>57.7</v>
+        <v>32.3</v>
       </c>
       <c r="T2" t="n">
-        <v>49.1</v>
+        <v>44.4</v>
       </c>
       <c r="U2" t="n">
-        <v>35.3</v>
+        <v>14.3</v>
       </c>
       <c r="V2" t="n">
-        <v>36.4</v>
+        <v>45.5</v>
       </c>
       <c r="W2" t="n">
         <v>27.3</v>
       </c>
       <c r="X2" t="n">
-        <v>36.4</v>
+        <v>27.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>18.2</v>
+        <v>27.3</v>
       </c>
       <c r="Z2" t="n">
         <v>9.1</v>
@@ -659,38 +659,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>01/06/2026 9:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Palestino</t>
+          <t>Junior</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Audax Italiano</t>
+          <t>Atletico Nacional</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.9</v>
+        <v>2.8</v>
       </c>
       <c r="E3" t="n">
-        <v>3.5</v>
+        <v>2.8</v>
       </c>
       <c r="F3" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
+        <v>2.7</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Chile Primera División+</t>
+          <t>Colombia Primera A+</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -700,425 +702,47 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>57</v>
-      </c>
-      <c r="N3" t="n">
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="n">
+        <v>55</v>
+      </c>
+      <c r="W3" t="n">
+        <v>20</v>
+      </c>
+      <c r="X3" t="n">
         <v>25</v>
       </c>
-      <c r="O3" t="n">
-        <v>19</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="T3" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="U3" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="V3" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="W3" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0</v>
-      </c>
       <c r="Y3" t="n">
-        <v>33.3</v>
+        <v>40</v>
       </c>
       <c r="Z3" t="n">
-        <v>16.7</v>
+        <v>10</v>
       </c>
       <c r="AA3" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>02/06/2026 7:00</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Ponte Preta</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Botafogo SP</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Brazil Serie B+</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
-        <v>37</v>
-      </c>
-      <c r="N4" t="n">
-        <v>42</v>
-      </c>
-      <c r="O4" t="n">
-        <v>21</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S4" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="T4" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="U4" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="V4" t="n">
-        <v>50</v>
-      </c>
-      <c r="W4" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="X4" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Palestino</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>A. Italiano</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="E5" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="n">
-        <v>31</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Chile Primera División+</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="W5" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="X5" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Boston River</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Liverpool Montevideo</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="n">
-        <v>23</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Uruguay Primera División - Apertura+</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="W6" t="n">
-        <v>13</v>
-      </c>
-      <c r="X6" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Penarol</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Central Espanol</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="F7" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
-        <v>12</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Uruguay Primera División - Apertura+</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="W7" t="n">
-        <v>25</v>
-      </c>
-      <c r="X7" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-10 11:10
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,34 +556,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10/06/2026 7:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.4</v>
+        <v>1.7</v>
       </c>
       <c r="E2" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="F2" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
+        <v>4.7</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -597,26 +599,20 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>21</v>
-      </c>
-      <c r="N2" t="n">
-        <v>52</v>
-      </c>
-      <c r="O2" t="n">
-        <v>27</v>
-      </c>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -624,48 +620,52 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S2" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="T2" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="U2" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="W2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="X2" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>18.8</v>
+      </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Goias</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Castellón</t>
+          <t>Novorizontino</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="E3" t="n">
-        <v>3.7</v>
+        <v>2.9</v>
       </c>
       <c r="F3" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -674,11 +674,11 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Spain Segunda División+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -713,22 +713,111 @@
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>42.9</v>
+        <v>60.6</v>
       </c>
       <c r="W3" t="n">
-        <v>28.6</v>
+        <v>12.1</v>
       </c>
       <c r="X3" t="n">
-        <v>28.6</v>
+        <v>27.3</v>
       </c>
       <c r="Y3" t="n">
-        <v>38.1</v>
+        <v>21.2</v>
       </c>
       <c r="Z3" t="n">
-        <v>14.3</v>
+        <v>6.1</v>
       </c>
       <c r="AA3" t="n">
-        <v>21</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Malaga</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>31</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Spain Segunda División+</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="W4" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="X4" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-13 10:33
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,47 +556,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/06/2026 4:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>São Bernardo SP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bosnia-Herzegovina</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="E2" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="F2" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>무승부</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>World Cup+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -605,22 +605,22 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="N2" t="n">
+        <v>38</v>
+      </c>
+      <c r="O2" t="n">
         <v>35</v>
       </c>
-      <c r="O2" t="n">
-        <v>24</v>
-      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -629,93 +629,101 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>8</v>
+        <v>32.3</v>
       </c>
       <c r="T2" t="n">
-        <v>49.3</v>
+        <v>46.2</v>
       </c>
       <c r="U2" t="n">
-        <v>1.9</v>
+        <v>14.3</v>
       </c>
       <c r="V2" t="n">
-        <v>52.2</v>
+        <v>52.4</v>
       </c>
       <c r="W2" t="n">
-        <v>17.4</v>
+        <v>23.8</v>
       </c>
       <c r="X2" t="n">
-        <v>30.4</v>
+        <v>23.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>43.5</v>
+        <v>28.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>8.699999999999999</v>
+        <v>4.8</v>
       </c>
       <c r="AA2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Lyn Oslo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Bryne FK</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
       <c r="E3" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="F3" t="n">
-        <v>3.4</v>
+        <v>2.4</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>40</v>
+      </c>
       <c r="I3" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>Norway 1. Division+</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>39</v>
+      </c>
+      <c r="N3" t="n">
+        <v>21</v>
+      </c>
+      <c r="O3" t="n">
+        <v>40</v>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -723,115 +731,1961 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T3" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U3" t="n">
+        <v>35.3</v>
+      </c>
       <c r="V3" t="n">
-        <v>59.5</v>
+        <v>50</v>
       </c>
       <c r="W3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X3" t="n">
-        <v>21.4</v>
+        <v>30</v>
       </c>
       <c r="Y3" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Z3" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="AA3" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.7</v>
+        <v>5.2</v>
       </c>
       <c r="E4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>World Cup+</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>18</v>
+      </c>
+      <c r="N4" t="n">
+        <v>33</v>
+      </c>
+      <c r="O4" t="n">
+        <v>49</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>8</v>
+      </c>
+      <c r="T4" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="U4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>53</v>
+      </c>
+      <c r="N5" t="n">
+        <v>28</v>
+      </c>
+      <c r="O5" t="n">
+        <v>19</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T5" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U5" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V5" t="n">
+        <v>100</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N6" t="n">
+        <v>11</v>
+      </c>
+      <c r="O6" t="n">
+        <v>69</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T6" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U6" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Stromsgodset IF</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Raufoss IL</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>67</v>
+      </c>
+      <c r="N7" t="n">
+        <v>11</v>
+      </c>
+      <c r="O7" t="n">
+        <v>23</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T7" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="U7" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Moss FK</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="n">
         <v>3.1</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>45</v>
+      </c>
+      <c r="N8" t="n">
+        <v>33</v>
+      </c>
+      <c r="O8" t="n">
+        <v>22</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T8" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="U8" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V8" t="n">
+        <v>60</v>
+      </c>
+      <c r="W8" t="n">
+        <v>20</v>
+      </c>
+      <c r="X8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Egersunds IK</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>44</v>
+      </c>
+      <c r="N9" t="n">
+        <v>26</v>
+      </c>
+      <c r="O9" t="n">
+        <v>30</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>3:2</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="T9" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="U9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="V9" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="W9" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ranheim Fotball</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
         <v>3</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>48</v>
+      </c>
+      <c r="N10" t="n">
+        <v>24</v>
+      </c>
+      <c r="O10" t="n">
+        <v>28</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T10" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="U10" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V10" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="W10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Strommen IF</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>9</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>57</v>
+      </c>
+      <c r="N11" t="n">
+        <v>22</v>
+      </c>
+      <c r="O11" t="n">
+        <v>20</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T11" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U11" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V11" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="W11" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="X11" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IL Hodd</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>25</v>
+      </c>
+      <c r="N12" t="n">
+        <v>32</v>
+      </c>
+      <c r="O12" t="n">
+        <v>43</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T12" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U12" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V12" t="n">
+        <v>40</v>
+      </c>
+      <c r="W12" t="n">
+        <v>20</v>
+      </c>
+      <c r="X12" t="n">
+        <v>40</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>40</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G13" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="n">
-        <v>21</v>
-      </c>
-      <c r="J4" t="inlineStr">
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>40</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="n">
+        <v>55</v>
+      </c>
+      <c r="W13" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="X13" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Operario-PR</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>14</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="n">
+        <v>50</v>
+      </c>
+      <c r="W14" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="X14" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>19</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="W15" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="X15" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Novorizontino</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Nautico Recife</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>38</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="W16" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="X16" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Concepción</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Deportes Limache</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Chile Primera División+</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="W17" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="X17" t="n">
+        <v>40</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>U. Catolica</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Universidad de Concepcion</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>17</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Chile Primera División+</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="W18" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="X18" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Union La Calera</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Universidad de Chile</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>22</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Chile Primera División+</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="W19" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="X19" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Asane</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ODD Ballklubb</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>12</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Norway 1. Division+</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="n">
+        <v>50</v>
+      </c>
+      <c r="W20" t="n">
+        <v>25</v>
+      </c>
+      <c r="X20" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Malaga</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Almeria</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>30</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Spain Segunda División+</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="n">
+        <v>60</v>
+      </c>
+      <c r="W21" t="n">
+        <v>10</v>
+      </c>
+      <c r="X21" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>30</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="F22" t="n">
+        <v>51</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>11</v>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>World Cup+</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>❓</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="W4" t="n">
-        <v>19</v>
-      </c>
-      <c r="X4" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>21</v>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="W22" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="X22" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>11</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>World Cup+</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="W23" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="X23" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>36</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>World Cup+</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="W24" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="X24" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-09 12:28
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,45 +556,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>10/07/2026 3:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Vojvodina</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5.7</v>
+        <v>2.9</v>
       </c>
       <c r="E2" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="F2" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>37</v>
+      </c>
       <c r="I2" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -602,17 +604,23 @@
           <t>원정정배</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>28</v>
+      </c>
+      <c r="N2" t="n">
+        <v>35</v>
+      </c>
+      <c r="O2" t="n">
+        <v>37</v>
+      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -620,70 +628,78 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="S2" t="n">
+        <v>8</v>
+      </c>
+      <c r="T2" t="n">
+        <v>50</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1.9</v>
+      </c>
       <c r="V2" t="n">
-        <v>54.5</v>
+        <v>33.3</v>
       </c>
       <c r="W2" t="n">
-        <v>27.3</v>
+        <v>14.3</v>
       </c>
       <c r="X2" t="n">
-        <v>18.2</v>
+        <v>52.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>27.3</v>
+        <v>42.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>9.1</v>
+        <v>19</v>
       </c>
       <c r="AA2" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CSKA Sofia</t>
+          <t>Cheonan City</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Derry City</t>
+          <t>Gimhae City</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="E3" t="n">
-        <v>5.3</v>
+        <v>3.4</v>
       </c>
       <c r="F3" t="n">
-        <v>11</v>
+        <v>3.6</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>50</v>
+      </c>
       <c r="I3" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>World UEFA Europa League+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -691,17 +707,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>50</v>
+      </c>
+      <c r="N3" t="n">
+        <v>32</v>
+      </c>
+      <c r="O3" t="n">
+        <v>18</v>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -709,52 +731,58 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T3" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U3" t="n">
+        <v>35.3</v>
+      </c>
       <c r="V3" t="n">
-        <v>54.5</v>
+        <v>35.7</v>
       </c>
       <c r="W3" t="n">
-        <v>27.3</v>
+        <v>35.7</v>
       </c>
       <c r="X3" t="n">
-        <v>18.2</v>
+        <v>28.6</v>
       </c>
       <c r="Y3" t="n">
-        <v>27.3</v>
+        <v>28.6</v>
       </c>
       <c r="Z3" t="n">
-        <v>9.1</v>
+        <v>7.1</v>
       </c>
       <c r="AA3" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>10/07/2026 2:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dynamo Kyiv</t>
+          <t>Sheriff Tiraspol</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>NK Aluminij</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E4" t="n">
         <v>4.2</v>
       </c>
       <c r="F4" t="n">
-        <v>5.8</v>
+        <v>8.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -763,7 +791,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -790,7 +818,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -802,57 +830,55 @@
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>64.7</v>
+        <v>61.5</v>
       </c>
       <c r="W4" t="n">
-        <v>17.6</v>
+        <v>23.1</v>
       </c>
       <c r="X4" t="n">
-        <v>17.6</v>
+        <v>15.4</v>
       </c>
       <c r="Y4" t="n">
-        <v>41.2</v>
+        <v>30.8</v>
       </c>
       <c r="Z4" t="n">
-        <v>17.6</v>
+        <v>15.4</v>
       </c>
       <c r="AA4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>10/07/2026 1:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HNK Hajduk Split</t>
+          <t>Qarabag</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Žilina</t>
+          <t>Vestri</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>4.7</v>
+        <v>16</v>
       </c>
       <c r="F5" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+        <v>48</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -869,17 +895,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>55</v>
+      </c>
+      <c r="N5" t="n">
+        <v>19</v>
+      </c>
+      <c r="O5" t="n">
+        <v>26</v>
+      </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3:0</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -887,61 +919,65 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="S5" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T5" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U5" t="n">
+        <v>35.3</v>
+      </c>
       <c r="V5" t="n">
-        <v>53.8</v>
+        <v>100</v>
       </c>
       <c r="W5" t="n">
-        <v>30.8</v>
+        <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>15.4</v>
+        <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>23.1</v>
+        <v>100</v>
       </c>
       <c r="Z5" t="n">
-        <v>7.7</v>
+        <v>100</v>
       </c>
       <c r="AA5" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>10/07/2026 3:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Qarabag</t>
+          <t>CSKA-Sofia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vestri</t>
+          <t>Derry City</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E6" t="n">
-        <v>14.2</v>
+        <v>5.7</v>
       </c>
       <c r="F6" t="n">
-        <v>48</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+        <v>12.2</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -958,17 +994,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>34</v>
+      </c>
+      <c r="N6" t="n">
+        <v>43</v>
+      </c>
+      <c r="O6" t="n">
+        <v>23</v>
+      </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2:2</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -976,61 +1018,65 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T6" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="U6" t="n">
+        <v>56.7</v>
+      </c>
       <c r="V6" t="n">
-        <v>54.5</v>
+        <v>33.3</v>
       </c>
       <c r="W6" t="n">
-        <v>27.3</v>
+        <v>33.3</v>
       </c>
       <c r="X6" t="n">
-        <v>18.2</v>
+        <v>33.3</v>
       </c>
       <c r="Y6" t="n">
-        <v>27.3</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>9.1</v>
+        <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>10/07/2026 3:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sheriff Tiraspol</t>
+          <t>Hajduk Split</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Aluminij</t>
+          <t>MSK Zilina</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>1.4</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="F7" t="n">
         <v>7.7</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1047,17 +1093,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>36</v>
+      </c>
+      <c r="N7" t="n">
+        <v>34</v>
+      </c>
+      <c r="O7" t="n">
+        <v>30</v>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1065,65 +1117,69 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T7" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U7" t="n">
+        <v>35.3</v>
+      </c>
       <c r="V7" t="n">
-        <v>54.5</v>
+        <v>28.6</v>
       </c>
       <c r="W7" t="n">
-        <v>27.3</v>
+        <v>42.9</v>
       </c>
       <c r="X7" t="n">
-        <v>18.2</v>
+        <v>28.6</v>
       </c>
       <c r="Y7" t="n">
-        <v>27.3</v>
+        <v>0</v>
       </c>
       <c r="Z7" t="n">
-        <v>9.1</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>10/07/2026 5:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vojvodina</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ferencvarosi TC</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.9</v>
+        <v>1.6</v>
       </c>
       <c r="E8" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+        <v>6.7</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>World UEFA Europa League+</t>
+          <t>World Cup+</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1133,20 +1189,26 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>56</v>
+      </c>
+      <c r="N8" t="n">
+        <v>24</v>
+      </c>
+      <c r="O8" t="n">
+        <v>20</v>
+      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1154,115 +1216,675 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T8" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="U8" t="n">
+        <v>56.7</v>
+      </c>
       <c r="V8" t="n">
-        <v>43.9</v>
+        <v>100</v>
       </c>
       <c r="W8" t="n">
-        <v>14.6</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>41.5</v>
+        <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>41.5</v>
+        <v>33.3</v>
       </c>
       <c r="Z8" t="n">
-        <v>14.6</v>
+        <v>33.3</v>
       </c>
       <c r="AA8" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Suwon FC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Jeonnam Dragons</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>South Korea South-Korea K League 2+</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>46</v>
+      </c>
+      <c r="N9" t="n">
+        <v>43</v>
+      </c>
+      <c r="O9" t="n">
+        <v>11</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="T9" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="U9" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V9" t="n">
+        <v>50</v>
+      </c>
+      <c r="W9" t="n">
+        <v>50</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Shandong Luneng</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Yunnan Yukun</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>China Super League+</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>28</v>
+      </c>
+      <c r="N10" t="n">
+        <v>37</v>
+      </c>
+      <c r="O10" t="n">
+        <v>35</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="T10" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="U10" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="V10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="W10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="X10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dynamo Kyiv</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>15</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>World UEFA Europa League+</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="W11" t="n">
+        <v>20</v>
+      </c>
+      <c r="X11" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>27</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="W12" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="X12" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>41</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Brazil Serie B+</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="W13" t="n">
+        <v>22</v>
+      </c>
+      <c r="X13" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>39</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Deportivo Maldonado</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Albion FC</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>43</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Uruguay Primera División - Apertura+</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="W14" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="X14" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
         <v>1.6</v>
       </c>
-      <c r="E9" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F9" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="n">
-        <v>14</v>
-      </c>
-      <c r="J9" t="inlineStr">
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>17</v>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>World Cup+</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>❓</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="W9" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="X9" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>28.6</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>14</v>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="W15" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="X15" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-14 14:13
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,27 +556,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>15/07/2026 4:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FK Ural</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Torpedo Moscow</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="E2" t="n">
         <v>3.2</v>
       </c>
       <c r="F2" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -584,19 +584,19 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="I2" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Russia First League+</t>
+          <t>World Cup+</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -605,17 +605,17 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="N2" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="O2" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -632,168 +632,164 @@
         <v>57.7</v>
       </c>
       <c r="T2" t="n">
-        <v>48.8</v>
+        <v>47.4</v>
       </c>
       <c r="U2" t="n">
         <v>35.3</v>
       </c>
       <c r="V2" t="n">
-        <v>70</v>
+        <v>41.2</v>
       </c>
       <c r="W2" t="n">
-        <v>10</v>
+        <v>17.6</v>
       </c>
       <c r="X2" t="n">
-        <v>20</v>
+        <v>41.2</v>
       </c>
       <c r="Y2" t="n">
-        <v>40</v>
+        <v>23.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>20</v>
+        <v>5.9</v>
       </c>
       <c r="AA2" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14/07/2026 7:00</t>
+          <t>15/07/2026 0:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>América Mineiro</t>
+          <t>KuPS Kuopio</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Vardar Skopje</t>
         </is>
       </c>
       <c r="D3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>40</v>
+      </c>
+      <c r="N3" t="n">
+        <v>35</v>
+      </c>
+      <c r="O3" t="n">
+        <v>25</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>8</v>
+      </c>
+      <c r="T3" t="n">
+        <v>50</v>
+      </c>
+      <c r="U3" t="n">
         <v>1.9</v>
       </c>
-      <c r="E3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>38</v>
-      </c>
-      <c r="I3" t="n">
-        <v>20</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Brazil Serie B+</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>32</v>
-      </c>
-      <c r="N3" t="n">
-        <v>30</v>
-      </c>
-      <c r="O3" t="n">
-        <v>38</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="T3" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="U3" t="n">
-        <v>35.3</v>
-      </c>
       <c r="V3" t="n">
-        <v>45</v>
+        <v>83.3</v>
       </c>
       <c r="W3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>30</v>
+        <v>16.7</v>
       </c>
       <c r="Y3" t="n">
-        <v>25</v>
+        <v>66.7</v>
       </c>
       <c r="Z3" t="n">
-        <v>15</v>
+        <v>16.7</v>
       </c>
       <c r="AA3" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>15/07/2026 1:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FK Chelyabinsk</t>
+          <t>Saburtalo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SKA-Khabarovsk</t>
+          <t>Flora Tallinn</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="E4" t="n">
-        <v>3.4</v>
+        <v>4.4</v>
       </c>
       <c r="F4" t="n">
-        <v>4.4</v>
+        <v>5.1</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Russia First League+</t>
+          <t>World UEFA Champions League+</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -807,22 +803,22 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="N4" t="n">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="O4" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -831,58 +827,68 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>32.3</v>
+        <v>57.7</v>
       </c>
       <c r="T4" t="n">
-        <v>48.1</v>
+        <v>47.4</v>
       </c>
       <c r="U4" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
+        <v>35.3</v>
+      </c>
+      <c r="V4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14/07/2026 1:30</t>
+          <t>15/07/2026 1:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Arsenal Tula</t>
+          <t>Inter d'Escaldes</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tekstilshchik Iv.</t>
+          <t>Lincoln Red Imps</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="E5" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>5.7</v>
+        <v>4.3</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Russia First League+</t>
+          <t>World UEFA Champions League+</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -896,22 +902,22 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="N5" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="O5" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -920,68 +926,68 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>76.2</v>
       </c>
       <c r="T5" t="n">
-        <v>52.9</v>
+        <v>57.8</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>56.7</v>
       </c>
       <c r="V5" t="n">
-        <v>42.9</v>
+        <v>33.3</v>
       </c>
       <c r="W5" t="n">
-        <v>28.6</v>
+        <v>33.3</v>
       </c>
       <c r="X5" t="n">
-        <v>28.6</v>
+        <v>33.3</v>
       </c>
       <c r="Y5" t="n">
-        <v>14.3</v>
+        <v>33.3</v>
       </c>
       <c r="Z5" t="n">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14/07/2026 7:00</t>
+          <t>15/07/2026 2:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cerro Largo</t>
+          <t>Gyori ETO FC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Defensor Sporting</t>
+          <t>Vikingur Reykjavik</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.8</v>
+        <v>1.7</v>
       </c>
       <c r="E6" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="F6" t="n">
-        <v>2.5</v>
+        <v>4.2</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Uruguay Primera División - Apertura+</t>
+          <t>World UEFA Champions League+</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -991,26 +997,26 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="N6" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="O6" t="n">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1019,159 +1025,167 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>8</v>
+        <v>32.3</v>
       </c>
       <c r="T6" t="n">
-        <v>52.9</v>
+        <v>47.5</v>
       </c>
       <c r="U6" t="n">
-        <v>1.9</v>
+        <v>14.3</v>
       </c>
       <c r="V6" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="W6" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="X6" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>15/07/2026 2:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Riga FC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Ararat-Armenia</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="E7" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="F7" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>28</v>
+      </c>
+      <c r="N7" t="n">
+        <v>39</v>
+      </c>
+      <c r="O7" t="n">
+        <v>33</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
         <v>50</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Brazil Serie B+</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
       <c r="V7" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="W7" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="X7" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="Y7" t="n">
         <v>40</v>
       </c>
       <c r="Z7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="AA7" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>15/07/2026 2:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>Levski Sofia</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Borac</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="E8" t="n">
-        <v>3.1</v>
+        <v>4.5</v>
       </c>
       <c r="F8" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+        <v>10.5</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>World UEFA Champions League+</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1184,17 +1198,23 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>37</v>
+      </c>
+      <c r="N8" t="n">
+        <v>40</v>
+      </c>
+      <c r="O8" t="n">
+        <v>23</v>
+      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1202,65 +1222,69 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>50</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
       <c r="V8" t="n">
-        <v>51.4</v>
+        <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>25.7</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>22.9</v>
+        <v>100</v>
       </c>
       <c r="Y8" t="n">
-        <v>37.1</v>
+        <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>22.9</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15/07/2026 2:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ural</t>
+          <t>The New Saints</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Torpedo Moskva</t>
+          <t>Sabah</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.1</v>
+        <v>5.6</v>
       </c>
       <c r="E9" t="n">
-        <v>3.2</v>
+        <v>4.2</v>
       </c>
       <c r="F9" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+        <v>1.5</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
       <c r="I9" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Russia First League+</t>
+          <t>World UEFA Champions League+</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1270,20 +1294,26 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>29</v>
+      </c>
+      <c r="N9" t="n">
+        <v>24</v>
+      </c>
+      <c r="O9" t="n">
+        <v>47</v>
+      </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1291,115 +1321,740 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
+      <c r="S9" t="n">
+        <v>8</v>
+      </c>
+      <c r="T9" t="n">
+        <v>50</v>
+      </c>
+      <c r="U9" t="n">
+        <v>1.9</v>
+      </c>
       <c r="V9" t="n">
-        <v>55.6</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>22.2</v>
+        <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>22.2</v>
+        <v>100</v>
       </c>
       <c r="Y9" t="n">
-        <v>35.2</v>
+        <v>100</v>
       </c>
       <c r="Z9" t="n">
-        <v>11.1</v>
+        <v>50</v>
       </c>
       <c r="AA9" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>15/07/2026 4:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Shamrock Rovers</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Floriana FC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>42</v>
+      </c>
+      <c r="N10" t="n">
+        <v>21</v>
+      </c>
+      <c r="O10" t="n">
+        <v>37</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>8</v>
+      </c>
+      <c r="T10" t="n">
+        <v>50</v>
+      </c>
+      <c r="U10" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>15/07/2026 4:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Larne</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SP Tre Fiori</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="n">
+        <v>21</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>73</v>
+      </c>
+      <c r="N11" t="n">
+        <v>15</v>
+      </c>
+      <c r="O11" t="n">
+        <v>12</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>8</v>
+      </c>
+      <c r="T11" t="n">
+        <v>50</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Inter Club d'Escaldes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Lincoln Red Imps FC</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>14</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="n">
+        <v>50</v>
+      </c>
+      <c r="W12" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="X12" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Atert Bissen</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>KI Klaksvik</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>32</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="W13" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="X13" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="E10" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="F10" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Egnatia Rrogozhinë</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Petrocub</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="n">
-        <v>47</v>
-      </c>
-      <c r="J10" t="inlineStr">
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>13</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="W14" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="X14" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sutjeska</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Kairat Almaty</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="X15" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ML Vitebsk</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>World UEFA Champions League+</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>50</v>
+      </c>
+      <c r="W16" t="n">
+        <v>25</v>
+      </c>
+      <c r="X16" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>21</v>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>World Cup+</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>❓</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="W10" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="X10" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>47</v>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="W17" t="n">
+        <v>19</v>
+      </c>
+      <c r="X17" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-23 16:09
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA45"/>
+  <dimension ref="A1:AA33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,27 +556,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>24/07/2026 4:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FC Seoul</t>
+          <t>Hajduk Split</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pohang Steelers</t>
+          <t>Pafos</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="E2" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="F2" t="n">
-        <v>4.4</v>
+        <v>3.3</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -584,19 +584,19 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="I2" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 1+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -605,13 +605,13 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="N2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -632,54 +632,54 @@
         <v>57.7</v>
       </c>
       <c r="T2" t="n">
-        <v>49</v>
+        <v>50.3</v>
       </c>
       <c r="U2" t="n">
         <v>35.3</v>
       </c>
       <c r="V2" t="n">
-        <v>58.8</v>
+        <v>53.8</v>
       </c>
       <c r="W2" t="n">
-        <v>23.5</v>
+        <v>19.2</v>
       </c>
       <c r="X2" t="n">
-        <v>17.6</v>
+        <v>26.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>52.9</v>
+        <v>30.8</v>
       </c>
       <c r="Z2" t="n">
-        <v>23.5</v>
+        <v>7.7</v>
       </c>
       <c r="AA2" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>23/07/2026 9:30</t>
+          <t>24/07/2026 2:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Houston Dynamo</t>
+          <t>Hammarby IF</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DC United</t>
+          <t>Anderlecht</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="E3" t="n">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
       <c r="F3" t="n">
-        <v>4.4</v>
+        <v>3.1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -687,19 +687,19 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I3" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -708,17 +708,17 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="N3" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="O3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -732,72 +732,72 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>8</v>
+        <v>87.5</v>
       </c>
       <c r="T3" t="n">
-        <v>52.5</v>
+        <v>72.7</v>
       </c>
       <c r="U3" t="n">
-        <v>1.9</v>
+        <v>73.5</v>
       </c>
       <c r="V3" t="n">
-        <v>47.6</v>
+        <v>33.3</v>
       </c>
       <c r="W3" t="n">
-        <v>14.3</v>
+        <v>41.7</v>
       </c>
       <c r="X3" t="n">
-        <v>38.1</v>
+        <v>25</v>
       </c>
       <c r="Y3" t="n">
-        <v>57.1</v>
+        <v>16.7</v>
       </c>
       <c r="Z3" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="AA3" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>23/07/2026 2:30</t>
+          <t>24/07/2026 9:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Levski Sofia</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CS Univ Craiova</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="E4" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="F4" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>무승부</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="I4" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>World UEFA Champions League+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -811,22 +811,22 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="N4" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="O4" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>0:1</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -835,72 +835,72 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>76.2</v>
+        <v>8</v>
       </c>
       <c r="T4" t="n">
-        <v>57.3</v>
+        <v>52.9</v>
       </c>
       <c r="U4" t="n">
-        <v>56.7</v>
+        <v>1.9</v>
       </c>
       <c r="V4" t="n">
-        <v>47.8</v>
+        <v>30</v>
       </c>
       <c r="W4" t="n">
-        <v>26.1</v>
+        <v>40</v>
       </c>
       <c r="X4" t="n">
-        <v>26.1</v>
+        <v>30</v>
       </c>
       <c r="Y4" t="n">
-        <v>34.8</v>
+        <v>30</v>
       </c>
       <c r="Z4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="AA4" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>23/07/2026 8:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Columbus Crew</t>
+          <t>Gimhae City</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>New York City FC</t>
+          <t>Cheongju FC</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="F5" t="n">
-        <v>3.6</v>
+        <v>2.2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="I5" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -910,26 +910,26 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="N5" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="O5" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -941,74 +941,72 @@
         <v>57.7</v>
       </c>
       <c r="T5" t="n">
-        <v>49</v>
+        <v>50.3</v>
       </c>
       <c r="U5" t="n">
         <v>35.3</v>
       </c>
       <c r="V5" t="n">
-        <v>35</v>
+        <v>57.1</v>
       </c>
       <c r="W5" t="n">
-        <v>15</v>
+        <v>14.3</v>
       </c>
       <c r="X5" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="Y5" t="n">
         <v>50</v>
       </c>
-      <c r="Y5" t="n">
-        <v>25</v>
-      </c>
       <c r="Z5" t="n">
-        <v>20</v>
+        <v>7.1</v>
       </c>
       <c r="AA5" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>23/07/2026 9:30</t>
+          <t>24/07/2026 9:45</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Defensa y Justicia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>CA Aldosivi</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="E6" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="F6" t="n">
-        <v>3.3</v>
+        <v>4.6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>무승부</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>38</v>
-      </c>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>Argentina Liga Profesional +</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1016,18 +1014,12 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M6" t="n">
-        <v>29</v>
-      </c>
-      <c r="N6" t="n">
-        <v>38</v>
-      </c>
-      <c r="O6" t="n">
-        <v>33</v>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1040,97 +1032,87 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S6" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="T6" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="U6" t="n">
-        <v>14.3</v>
-      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>47.6</v>
+        <v>63.6</v>
       </c>
       <c r="W6" t="n">
-        <v>23.8</v>
+        <v>22.7</v>
       </c>
       <c r="X6" t="n">
-        <v>28.6</v>
+        <v>13.6</v>
       </c>
       <c r="Y6" t="n">
-        <v>42.9</v>
+        <v>40.9</v>
       </c>
       <c r="Z6" t="n">
-        <v>14.3</v>
+        <v>27.3</v>
       </c>
       <c r="AA6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23/07/2026 9:30</t>
+          <t>24/07/2026 1:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Austin FC</t>
+          <t>Qarabag</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Seattle Sounders</t>
+          <t>CSKA-Sofia</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3.2</v>
+        <v>1.4</v>
       </c>
       <c r="E7" t="n">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
       <c r="F7" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+        <v>6.8</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="N7" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="O7" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1144,77 +1126,73 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>8</v>
+        <v>32.3</v>
       </c>
       <c r="T7" t="n">
-        <v>52.5</v>
+        <v>47.8</v>
       </c>
       <c r="U7" t="n">
-        <v>1.9</v>
+        <v>14.3</v>
       </c>
       <c r="V7" t="n">
-        <v>30.8</v>
+        <v>100</v>
       </c>
       <c r="W7" t="n">
-        <v>15.4</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>53.8</v>
+        <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>53.8</v>
+        <v>0</v>
       </c>
       <c r="Z7" t="n">
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>23/07/2026 9:30</t>
+          <t>24/07/2026 2:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Hradec Kralove</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="E8" t="n">
-        <v>3.5</v>
+        <v>4.7</v>
       </c>
       <c r="F8" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>무승부</t>
-        </is>
-      </c>
+        <v>6.2</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1223,22 +1201,22 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="N8" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="O8" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1247,77 +1225,73 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>32.3</v>
       </c>
       <c r="T8" t="n">
-        <v>52.5</v>
+        <v>47.8</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="V8" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="W8" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="Y8" t="n">
         <v>50</v>
       </c>
       <c r="Z8" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="AA8" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>23/07/2026 9:30</t>
+          <t>24/07/2026 2:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sporting Cristal</t>
+          <t>Dynamo Kyiv</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RB Bragantino</t>
+          <t>PAOK</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3.3</v>
+        <v>2.9</v>
       </c>
       <c r="E9" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="F9" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
+        <v>2.4</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1326,22 +1300,22 @@
         </is>
       </c>
       <c r="M9" t="n">
+        <v>53</v>
+      </c>
+      <c r="N9" t="n">
+        <v>27</v>
+      </c>
+      <c r="O9" t="n">
         <v>20</v>
       </c>
-      <c r="N9" t="n">
-        <v>39</v>
-      </c>
-      <c r="O9" t="n">
-        <v>41</v>
-      </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>3:0</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1350,68 +1324,58 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T9" t="n">
-        <v>52.5</v>
+        <v>50.3</v>
       </c>
       <c r="U9" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="V9" t="n">
-        <v>40</v>
-      </c>
-      <c r="W9" t="n">
-        <v>20</v>
-      </c>
-      <c r="X9" t="n">
-        <v>40</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>40</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>30</v>
-      </c>
+        <v>35.3</v>
+      </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>24/07/2026 2:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gwangju FC</t>
+          <t>Sheriff Tiraspol</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sangju Sangmu</t>
+          <t>Maccabi Tel Aviv</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4.3</v>
+        <v>3.1</v>
       </c>
       <c r="E10" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="F10" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 1+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1425,22 +1389,22 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="N10" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="O10" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1449,68 +1413,68 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>32.3</v>
+        <v>87.5</v>
       </c>
       <c r="T10" t="n">
-        <v>46.4</v>
+        <v>72.7</v>
       </c>
       <c r="U10" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="V10" t="n">
         <v>14.3</v>
       </c>
-      <c r="V10" t="n">
-        <v>0</v>
-      </c>
       <c r="W10" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>66.7</v>
+        <v>85.7</v>
       </c>
       <c r="Y10" t="n">
-        <v>33.3</v>
+        <v>57.1</v>
       </c>
       <c r="Z10" t="n">
-        <v>33.3</v>
+        <v>28.6</v>
       </c>
       <c r="AA10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>24/07/2026 3:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bucheon FC 1995</t>
+          <t>Twente</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FC Anyang</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2.9</v>
+        <v>1.6</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>2.6</v>
+        <v>5.3</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>South Korea South-Korea K League 1+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1520,26 +1484,26 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="N11" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1548,68 +1512,68 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>32.3</v>
+        <v>8</v>
       </c>
       <c r="T11" t="n">
-        <v>46.4</v>
+        <v>52.9</v>
       </c>
       <c r="U11" t="n">
-        <v>14.3</v>
+        <v>1.9</v>
       </c>
       <c r="V11" t="n">
         <v>50</v>
       </c>
       <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
         <v>50</v>
       </c>
-      <c r="X11" t="n">
-        <v>0</v>
-      </c>
       <c r="Y11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Z11" t="n">
         <v>0</v>
       </c>
       <c r="AA11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>23/07/2026 2:00</t>
+          <t>24/07/2026 3:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lillestrom SK</t>
+          <t>St Gallen</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Viking FK</t>
+          <t>SL Benfica</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>7.2</v>
       </c>
       <c r="E12" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="F12" t="n">
-        <v>2.2</v>
+        <v>1.4</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1623,17 +1587,17 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="N12" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O12" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>0:2</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1647,68 +1611,58 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>57.7</v>
+        <v>32.3</v>
       </c>
       <c r="T12" t="n">
-        <v>49</v>
+        <v>47.8</v>
       </c>
       <c r="U12" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="V12" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="W12" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="X12" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>11.1</v>
-      </c>
+        <v>14.3</v>
+      </c>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>23/07/2026 2:00</t>
+          <t>24/07/2026 7:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bodo/Glimt</t>
+          <t>Sarmiento Junín</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HamKam</t>
+          <t>Argentinos Juniors</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1.1</v>
+        <v>4.5</v>
       </c>
       <c r="E13" t="n">
-        <v>10.2</v>
+        <v>2.9</v>
       </c>
       <c r="F13" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Norway Eliteserien+</t>
+          <t>Argentina Liga Profesional +</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1718,86 +1672,96 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M13" t="n">
+        <v>30</v>
+      </c>
+      <c r="N13" t="n">
+        <v>37</v>
+      </c>
+      <c r="O13" t="n">
+        <v>33</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" t="n">
         <v>50</v>
       </c>
-      <c r="N13" t="n">
-        <v>35</v>
-      </c>
-      <c r="O13" t="n">
-        <v>15</v>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>3:1</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S13" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="T13" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="U13" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
+      <c r="X13" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
       <c r="AA13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>23/07/2026 2:00</t>
+          <t>24/07/2026 7:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Omonia Nicosia</t>
+          <t>Belgrano Córdoba</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kairat Almaty</t>
+          <t>Rosario Central</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="E14" t="n">
-        <v>3.8</v>
+        <v>2.8</v>
       </c>
       <c r="F14" t="n">
-        <v>5</v>
+        <v>3.1</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>World UEFA Champions League+</t>
+          <t>Argentina Liga Profesional +</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1811,13 +1775,13 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="N14" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="O14" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
@@ -1838,65 +1802,65 @@
         <v>32.3</v>
       </c>
       <c r="T14" t="n">
-        <v>46.4</v>
+        <v>47.8</v>
       </c>
       <c r="U14" t="n">
         <v>14.3</v>
       </c>
       <c r="V14" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="W14" t="n">
-        <v>40</v>
+        <v>37.5</v>
       </c>
       <c r="X14" t="n">
-        <v>20</v>
+        <v>37.5</v>
       </c>
       <c r="Y14" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="Z14" t="n">
-        <v>20</v>
+        <v>12.5</v>
       </c>
       <c r="AA14" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>23/07/2026 4:00</t>
+          <t>24/07/2026 7:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Egnatia Rrogozhine</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Celje</t>
+          <t>Remo PA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="E15" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>6.6</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>World UEFA Champions League+</t>
+          <t>Brazil Serie A+</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1906,21 +1870,21 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="N15" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="O15" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1934,68 +1898,68 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>76.2</v>
+        <v>57.7</v>
       </c>
       <c r="T15" t="n">
-        <v>57.3</v>
+        <v>50.3</v>
       </c>
       <c r="U15" t="n">
-        <v>56.7</v>
+        <v>35.3</v>
       </c>
       <c r="V15" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="W15" t="n">
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Y15" t="n">
         <v>100</v>
       </c>
       <c r="Z15" t="n">
-        <v>33.3</v>
+        <v>100</v>
       </c>
       <c r="AA15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>23/07/2026 7:00</t>
+          <t>24/07/2026 7:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ind Medellin</t>
+          <t>Athletic Club MG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>São Bernardo SP</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
         <v>3.1</v>
       </c>
       <c r="F16" t="n">
-        <v>3.1</v>
+        <v>3.9</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2009,22 +1973,22 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="N16" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="O16" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2033,68 +1997,68 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>8</v>
+        <v>57.7</v>
       </c>
       <c r="T16" t="n">
-        <v>52.5</v>
+        <v>50.3</v>
       </c>
       <c r="U16" t="n">
-        <v>1.9</v>
+        <v>35.3</v>
       </c>
       <c r="V16" t="n">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="W16" t="n">
-        <v>25</v>
+        <v>37.5</v>
       </c>
       <c r="X16" t="n">
         <v>25</v>
       </c>
       <c r="Y16" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Z16" t="n">
-        <v>0</v>
+        <v>37.5</v>
       </c>
       <c r="AA16" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>23/07/2026 7:30</t>
+          <t>24/07/2026 9:30</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Boca Juniors</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>O Higgins</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4.5</v>
+        <v>1.3</v>
       </c>
       <c r="E17" t="n">
-        <v>3.4</v>
+        <v>5.1</v>
       </c>
       <c r="F17" t="n">
-        <v>1.8</v>
+        <v>11.2</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>World CONMEBOL Sudamericana+</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2104,26 +2068,26 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="N17" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="O17" t="n">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2135,65 +2099,55 @@
         <v>32.3</v>
       </c>
       <c r="T17" t="n">
-        <v>46.4</v>
+        <v>47.8</v>
       </c>
       <c r="U17" t="n">
         <v>14.3</v>
       </c>
-      <c r="V17" t="n">
-        <v>0</v>
-      </c>
-      <c r="W17" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="X17" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>33.3</v>
-      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>23/07/2026 8:30</t>
+          <t>24/07/2026 9:30</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>New England Revolution</t>
+          <t>Ind Santa Fe</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Toronto FC</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="E18" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="F18" t="n">
-        <v>4.5</v>
+        <v>10</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>World CONMEBOL Sudamericana+</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2207,17 +2161,17 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="N18" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="O18" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2231,68 +2185,58 @@
         </is>
       </c>
       <c r="S18" t="n">
-        <v>57.7</v>
+        <v>8</v>
       </c>
       <c r="T18" t="n">
-        <v>49</v>
+        <v>52.9</v>
       </c>
       <c r="U18" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="V18" t="n">
-        <v>60</v>
-      </c>
-      <c r="W18" t="n">
-        <v>0</v>
-      </c>
-      <c r="X18" t="n">
-        <v>40</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>60</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>0</v>
-      </c>
+        <v>1.9</v>
+      </c>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>23/07/2026 8:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FC Cincinnati</t>
+          <t>Seoul E-Land</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Vancouver Whitecaps</t>
+          <t>Cheonan City</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3.9</v>
+        <v>1.5</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="F19" t="n">
-        <v>1.8</v>
+        <v>5</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>South Korea South-Korea K League 2+</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2302,26 +2246,26 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="N19" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="O19" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2330,68 +2274,70 @@
         </is>
       </c>
       <c r="S19" t="n">
-        <v>87.5</v>
+        <v>57.7</v>
       </c>
       <c r="T19" t="n">
-        <v>68.40000000000001</v>
+        <v>50.3</v>
       </c>
       <c r="U19" t="n">
-        <v>73.5</v>
+        <v>35.3</v>
       </c>
       <c r="V19" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="W19" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="X19" t="n">
-        <v>40</v>
+        <v>16.7</v>
       </c>
       <c r="Y19" t="n">
-        <v>40</v>
+        <v>66.7</v>
       </c>
       <c r="Z19" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="AA19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>23/07/2026 8:30</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Philadelphia Union</t>
+          <t>Belgrano Cordoba</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>New York Red Bulls</t>
+          <t>Rosario Central</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.7</v>
+        <v>2.6</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="F20" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
+        <v>3.1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>Argentina Liga Profesional +</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2404,23 +2350,17 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M20" t="n">
-        <v>18</v>
-      </c>
-      <c r="N20" t="n">
-        <v>30</v>
-      </c>
-      <c r="O20" t="n">
-        <v>52</v>
-      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2428,69 +2368,63 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S20" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="T20" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="U20" t="n">
-        <v>14.3</v>
-      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>0</v>
+        <v>23.1</v>
       </c>
       <c r="W20" t="n">
-        <v>100</v>
+        <v>30.8</v>
       </c>
       <c r="X20" t="n">
-        <v>0</v>
+        <v>46.2</v>
       </c>
       <c r="Y20" t="n">
-        <v>50</v>
+        <v>38.5</v>
       </c>
       <c r="Z20" t="n">
-        <v>50</v>
+        <v>15.4</v>
       </c>
       <c r="AA20" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>23/07/2026 9:15</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Charlotte FC</t>
+          <t>Sarmiento Junin</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Atlanta United</t>
+          <t>Argentinos JRS</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1.9</v>
+        <v>4.5</v>
       </c>
       <c r="E21" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="F21" t="n">
-        <v>3.8</v>
+        <v>2</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>Argentina Liga Profesional +</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2500,26 +2434,20 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M21" t="n">
-        <v>61</v>
-      </c>
-      <c r="N21" t="n">
-        <v>22</v>
-      </c>
-      <c r="O21" t="n">
-        <v>17</v>
-      </c>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2527,20 +2455,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S21" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="T21" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="U21" t="n">
-        <v>14.3</v>
-      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="W21" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="X21" t="n">
         <v>50</v>
@@ -2552,40 +2474,42 @@
         <v>0</v>
       </c>
       <c r="AA21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>23/07/2026 9:30</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Chapecoense SC</t>
+          <t>Botafogo</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Vitoria</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>7</v>
+        <v>1.7</v>
       </c>
       <c r="E22" t="n">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="F22" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
+        <v>4.8</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -2599,26 +2523,20 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M22" t="n">
-        <v>14</v>
-      </c>
-      <c r="N22" t="n">
-        <v>24</v>
-      </c>
-      <c r="O22" t="n">
-        <v>61</v>
-      </c>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2626,69 +2544,65 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S22" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="T22" t="n">
-        <v>49</v>
-      </c>
-      <c r="U22" t="n">
-        <v>35.3</v>
-      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="W22" t="n">
-        <v>100</v>
+        <v>16</v>
       </c>
       <c r="X22" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="Y22" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="Z22" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="AA22" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>23/07/2026 9:30</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sporting Kansas City</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Minnesota United</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3.4</v>
+        <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>3.8</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
+        <v>4.1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>Brazil Serie B+</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2698,26 +2612,20 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M23" t="n">
-        <v>37</v>
-      </c>
-      <c r="N23" t="n">
-        <v>28</v>
-      </c>
-      <c r="O23" t="n">
-        <v>34</v>
-      </c>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2725,69 +2633,65 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S23" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="T23" t="n">
-        <v>49</v>
-      </c>
-      <c r="U23" t="n">
-        <v>35.3</v>
-      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>0</v>
+        <v>40.7</v>
       </c>
       <c r="W23" t="n">
-        <v>0</v>
+        <v>40.7</v>
       </c>
       <c r="X23" t="n">
-        <v>100</v>
+        <v>18.5</v>
       </c>
       <c r="Y23" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="Z23" t="n">
-        <v>0</v>
+        <v>18.5</v>
       </c>
       <c r="AA23" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>23/07/2026 9:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nashville SC</t>
+          <t>Bolívar</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Montreal Impact</t>
+          <t>Gremio</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E24" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
+        <v>4.8</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>USA Major League Soccer+</t>
+          <t>World CONMEBOL Sudamericana+</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2800,23 +2704,17 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M24" t="n">
-        <v>59</v>
-      </c>
-      <c r="N24" t="n">
-        <v>30</v>
-      </c>
-      <c r="O24" t="n">
-        <v>11</v>
-      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2824,55 +2722,49 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S24" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="T24" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="U24" t="n">
-        <v>56.7</v>
-      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="W24" t="n">
-        <v>50</v>
+        <v>6.7</v>
       </c>
       <c r="X24" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="Y24" t="n">
-        <v>0</v>
+        <v>53.3</v>
       </c>
       <c r="Z24" t="n">
-        <v>0</v>
+        <v>13.3</v>
       </c>
       <c r="AA24" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>Beşiktaş</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="F25" t="n">
         <v>3.4</v>
@@ -2884,11 +2776,11 @@
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2926,45 +2818,45 @@
         <v>50</v>
       </c>
       <c r="W25" t="n">
-        <v>26.1</v>
+        <v>17.5</v>
       </c>
       <c r="X25" t="n">
-        <v>23.9</v>
+        <v>32.5</v>
       </c>
       <c r="Y25" t="n">
-        <v>28.3</v>
+        <v>35</v>
       </c>
       <c r="Z25" t="n">
-        <v>10.9</v>
+        <v>15</v>
       </c>
       <c r="AA25" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Hammarby FF</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>Anderlecht</t>
         </is>
       </c>
       <c r="D26" t="n">
         <v>2.2</v>
       </c>
       <c r="E26" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F26" t="n">
         <v>3.1</v>
-      </c>
-      <c r="F26" t="n">
-        <v>3.3</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2973,11 +2865,11 @@
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3012,59 +2904,59 @@
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>47.8</v>
+        <v>38.6</v>
       </c>
       <c r="W26" t="n">
-        <v>26.1</v>
+        <v>31.8</v>
       </c>
       <c r="X26" t="n">
-        <v>26.1</v>
+        <v>29.5</v>
       </c>
       <c r="Y26" t="n">
-        <v>32.6</v>
+        <v>31.8</v>
       </c>
       <c r="Z26" t="n">
-        <v>10.9</v>
+        <v>11.4</v>
       </c>
       <c r="AA26" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Operario-PR</t>
+          <t>Tromso</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Hradec Králové</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>1.4</v>
       </c>
       <c r="E27" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="F27" t="n">
-        <v>8</v>
+        <v>6.2</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Brazil Serie B+</t>
+          <t>World UEFA Europa League+</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -3099,48 +2991,48 @@
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>50</v>
+        <v>57.1</v>
       </c>
       <c r="W27" t="n">
-        <v>33.3</v>
+        <v>14.3</v>
       </c>
       <c r="X27" t="n">
-        <v>16.7</v>
+        <v>28.6</v>
       </c>
       <c r="Y27" t="n">
-        <v>0</v>
+        <v>28.6</v>
       </c>
       <c r="Z27" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="AA27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Independiente Medellin</t>
+          <t>Gimnasia M.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Vasco DA Gama</t>
+          <t>Central Cordoba de Santiago</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="E28" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="F28" t="n">
-        <v>3.1</v>
+        <v>5</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -3149,11 +3041,11 @@
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana+</t>
+          <t>Argentina Liga Profesional +</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -3188,48 +3080,48 @@
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>45.1</v>
+        <v>46.7</v>
       </c>
       <c r="W28" t="n">
-        <v>27.5</v>
+        <v>13.3</v>
       </c>
       <c r="X28" t="n">
-        <v>27.5</v>
+        <v>40</v>
       </c>
       <c r="Y28" t="n">
-        <v>25.5</v>
+        <v>53.3</v>
       </c>
       <c r="Z28" t="n">
-        <v>7.8</v>
+        <v>20</v>
       </c>
       <c r="AA28" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Levski Sofia</t>
+          <t>Racing Club</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Gimnasia L.P.</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="E29" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="F29" t="n">
-        <v>3.5</v>
+        <v>4.7</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -3238,11 +3130,11 @@
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>World UEFA Champions League+</t>
+          <t>Argentina Liga Profesional +</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -3277,48 +3169,48 @@
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>46.7</v>
+        <v>65.2</v>
       </c>
       <c r="W29" t="n">
-        <v>22.2</v>
+        <v>13</v>
       </c>
       <c r="X29" t="n">
-        <v>31.1</v>
+        <v>21.7</v>
       </c>
       <c r="Y29" t="n">
-        <v>35.6</v>
+        <v>60.9</v>
       </c>
       <c r="Z29" t="n">
-        <v>8.9</v>
+        <v>39.1</v>
       </c>
       <c r="AA29" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Belgrano Cordoba</t>
+          <t>Velez Sarsfield</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Rosario Central</t>
+          <t>Instituto Cordoba</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="E30" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>3.3</v>
+        <v>3.9</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -3327,7 +3219,7 @@
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -3366,59 +3258,61 @@
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="n">
-        <v>20</v>
+        <v>22.7</v>
       </c>
       <c r="W30" t="n">
-        <v>50</v>
+        <v>45.5</v>
       </c>
       <c r="X30" t="n">
-        <v>30</v>
+        <v>31.8</v>
       </c>
       <c r="Y30" t="n">
-        <v>10</v>
+        <v>36.4</v>
       </c>
       <c r="Z30" t="n">
-        <v>10</v>
+        <v>13.6</v>
       </c>
       <c r="AA30" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarmiento Junin</t>
+          <t>Union La Calera</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Argentinos JRS</t>
+          <t>Everton de Vina</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>4.6</v>
+        <v>2.5</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
+        <v>2.8</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Argentina Liga Profesional +</t>
+          <t>Chile Primera División+</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3428,7 +3322,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
@@ -3453,59 +3347,59 @@
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>0</v>
+        <v>46.3</v>
       </c>
       <c r="W31" t="n">
-        <v>50</v>
+        <v>14.6</v>
       </c>
       <c r="X31" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="Y31" t="n">
-        <v>0</v>
+        <v>51.2</v>
       </c>
       <c r="Z31" t="n">
-        <v>0</v>
+        <v>12.2</v>
       </c>
       <c r="AA31" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Llaneros</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Remo</t>
+          <t>Deportivo Pereira</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="F32" t="n">
-        <v>6.6</v>
+        <v>5.8</v>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>Colombia Primera A+</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3540,48 +3434,48 @@
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
-        <v>71.40000000000001</v>
+        <v>0</v>
       </c>
       <c r="W32" t="n">
-        <v>14.3</v>
+        <v>66.7</v>
       </c>
       <c r="X32" t="n">
-        <v>14.3</v>
+        <v>33.3</v>
       </c>
       <c r="Y32" t="n">
-        <v>28.6</v>
+        <v>0</v>
       </c>
       <c r="Z32" t="n">
-        <v>28.6</v>
+        <v>0</v>
       </c>
       <c r="AA32" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Botafogo</t>
+          <t>CSKA Moscow</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Vitoria</t>
+          <t>Baltika</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="E33" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="F33" t="n">
-        <v>4.8</v>
+        <v>4.2</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -3590,11 +3484,11 @@
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Brazil Serie A+</t>
+          <t>Russia Premier League+</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3629,1086 +3523,22 @@
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="n">
-        <v>62.5</v>
+        <v>48.6</v>
       </c>
       <c r="W33" t="n">
-        <v>16.7</v>
+        <v>28.6</v>
       </c>
       <c r="X33" t="n">
-        <v>20.8</v>
+        <v>22.9</v>
       </c>
       <c r="Y33" t="n">
-        <v>50</v>
+        <v>37.1</v>
       </c>
       <c r="Z33" t="n">
-        <v>29.2</v>
+        <v>22.9</v>
       </c>
       <c r="AA33" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>22:30</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Athletic Club</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>São Bernardo</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F34" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="n">
-        <v>39</v>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Brazil Serie B+</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="W34" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="X34" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="Y34" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="AA34" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>23:30</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Cuiaba</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Atletico Goianiense</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>2</v>
-      </c>
-      <c r="E35" t="n">
-        <v>3</v>
-      </c>
-      <c r="F35" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="n">
-        <v>24</v>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Brazil Serie B+</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
-      <c r="U35" t="inlineStr"/>
-      <c r="V35" t="n">
-        <v>50</v>
-      </c>
-      <c r="W35" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="X35" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="Y35" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="AA35" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Bolívar</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Gremio</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="E36" t="n">
-        <v>4</v>
-      </c>
-      <c r="F36" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="n">
-        <v>14</v>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>World CONMEBOL Sudamericana+</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="W36" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="X36" t="n">
-        <v>35.7</v>
-      </c>
-      <c r="Y36" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="Z36" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="AA36" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Beşiktaş</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>FC Midtjylland</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>2</v>
-      </c>
-      <c r="E37" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F37" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="n">
-        <v>47</v>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="n">
-        <v>40.4</v>
-      </c>
-      <c r="W37" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="X37" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="Y37" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="Z37" t="n">
-        <v>17</v>
-      </c>
-      <c r="AA37" t="n">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Hammarby FF</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Anderlecht</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="E38" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="F38" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="n">
-        <v>36</v>
-      </c>
-      <c r="W38" t="n">
-        <v>28</v>
-      </c>
-      <c r="X38" t="n">
-        <v>36</v>
-      </c>
-      <c r="Y38" t="n">
-        <v>56</v>
-      </c>
-      <c r="Z38" t="n">
-        <v>24</v>
-      </c>
-      <c r="AA38" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>FC ST. Gallen</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Benfica</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="E39" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="F39" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>2</v>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="n">
-        <v>0</v>
-      </c>
-      <c r="W39" t="n">
-        <v>50</v>
-      </c>
-      <c r="X39" t="n">
-        <v>50</v>
-      </c>
-      <c r="Y39" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA39" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Tromso</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Hradec Králové</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E40" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="F40" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="n">
-        <v>12</v>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr"/>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="n">
-        <v>41.7</v>
-      </c>
-      <c r="W40" t="n">
-        <v>41.7</v>
-      </c>
-      <c r="X40" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="Y40" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="Z40" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="AA40" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Dynamo Kyiv</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>PAOK</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="E41" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F41" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="n">
-        <v>48</v>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
-      <c r="U41" t="inlineStr"/>
-      <c r="V41" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="W41" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="X41" t="n">
-        <v>50</v>
-      </c>
-      <c r="Y41" t="n">
-        <v>47.9</v>
-      </c>
-      <c r="Z41" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="AA41" t="n">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>HNK Hajduk Split</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Pafos</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E42" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="F42" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="n">
-        <v>51</v>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S42" t="inlineStr"/>
-      <c r="T42" t="inlineStr"/>
-      <c r="U42" t="inlineStr"/>
-      <c r="V42" t="n">
-        <v>51</v>
-      </c>
-      <c r="W42" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="X42" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="Y42" t="n">
-        <v>31.4</v>
-      </c>
-      <c r="Z42" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="AA42" t="n">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Qarabag</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>CSKA Sofia</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E43" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="F43" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>6</v>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S43" t="inlineStr"/>
-      <c r="T43" t="inlineStr"/>
-      <c r="U43" t="inlineStr"/>
-      <c r="V43" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="W43" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="X43" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="Y43" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="Z43" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="AA43" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Sheriff Tiraspol</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Maccabi Tel Aviv</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="E44" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="F44" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="n">
-        <v>28</v>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr"/>
-      <c r="T44" t="inlineStr"/>
-      <c r="U44" t="inlineStr"/>
-      <c r="V44" t="n">
-        <v>25</v>
-      </c>
-      <c r="W44" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="X44" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="Y44" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="Z44" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="AA44" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Twente</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Ferencvarosi TC</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="E45" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F45" t="n">
-        <v>5</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="n">
-        <v>15</v>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>World UEFA Europa League+</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
-      <c r="U45" t="inlineStr"/>
-      <c r="V45" t="n">
-        <v>60</v>
-      </c>
-      <c r="W45" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="X45" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="Y45" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Z45" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="AA45" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>